<commit_message>
Edited for thinner camshaft bearing
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1329D0C-381A-4A69-A225-2127C75776FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F291CAE-C194-4E3B-A39C-93DFF63A0A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="317">
   <si>
     <t>6-DoF Arm — Gravity Torque Budget v2 (elbow-mounted forearm roll)</t>
   </si>
@@ -859,18 +859,6 @@
     <t xml:space="preserve">Input/Output Flanged Bearings </t>
   </si>
   <si>
-    <t>M5x0.8 around 64mm in total length</t>
-  </si>
-  <si>
-    <t>ID 50mm x OD 65mm x 7mm</t>
-  </si>
-  <si>
-    <t>ID 5mm x  OD 10mm x 4mm</t>
-  </si>
-  <si>
-    <t>Ø5mm x 30mm</t>
-  </si>
-  <si>
     <t>Shoulder bolts M5</t>
   </si>
   <si>
@@ -880,12 +868,6 @@
     <t xml:space="preserve">M2.5 Heat Set Threaded Inserts </t>
   </si>
   <si>
-    <t>M5 x Ø10mm x 7mm</t>
-  </si>
-  <si>
-    <t>M2.5 x Ø3.5mm x 4mm</t>
-  </si>
-  <si>
     <t>M5 Screw</t>
   </si>
   <si>
@@ -976,10 +958,37 @@
     <t>3D Printed Parts</t>
   </si>
   <si>
-    <t xml:space="preserve"> ID 15mm x OD 28mm x 8mm</t>
-  </si>
-  <si>
     <t>Coupler</t>
+  </si>
+  <si>
+    <t>Hex Shaft</t>
+  </si>
+  <si>
+    <t>5mm x 51mm</t>
+  </si>
+  <si>
+    <t>Price/Pack</t>
+  </si>
+  <si>
+    <t>M5 x Ø10mm x 7mm (50 pcs)</t>
+  </si>
+  <si>
+    <t>ID 50mm x OD 65mm x 7mm (2 pcs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ID 15mm x OD 28mm x 7mm (8 pcs)</t>
+  </si>
+  <si>
+    <t>ID 5mm x  OD 10mm x 4mm (30 pcs)</t>
+  </si>
+  <si>
+    <t>Ø5mm x 30mm (50 pcs)</t>
+  </si>
+  <si>
+    <t>M2.5 x Ø3.5mm x 4mm (100 pcs)</t>
+  </si>
+  <si>
+    <t>M5x0.8 around 64mm in total length (4 pcs)</t>
   </si>
 </sst>
 </file>
@@ -1268,7 +1277,7 @@
     <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1367,7 +1376,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1415,6 +1423,12 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="4" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1424,10 +1438,17 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="4" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1747,17 +1768,17 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -1825,17 +1846,17 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46"/>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="46"/>
-      <c r="I11" s="46"/>
+      <c r="B11" s="68"/>
+      <c r="C11" s="68"/>
+      <c r="D11" s="68"/>
+      <c r="E11" s="68"/>
+      <c r="F11" s="68"/>
+      <c r="G11" s="68"/>
+      <c r="H11" s="68"/>
+      <c r="I11" s="68"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -1933,17 +1954,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="46" t="s">
+      <c r="A20" s="68" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="46"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46"/>
+      <c r="B20" s="68"/>
+      <c r="C20" s="68"/>
+      <c r="D20" s="68"/>
+      <c r="E20" s="68"/>
+      <c r="F20" s="68"/>
+      <c r="G20" s="68"/>
+      <c r="H20" s="68"/>
+      <c r="I20" s="68"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
@@ -1968,17 +1989,17 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="46" t="s">
+      <c r="A24" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="46"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="46"/>
+      <c r="B24" s="68"/>
+      <c r="C24" s="68"/>
+      <c r="D24" s="68"/>
+      <c r="E24" s="68"/>
+      <c r="F24" s="68"/>
+      <c r="G24" s="68"/>
+      <c r="H24" s="68"/>
+      <c r="I24" s="68"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
@@ -2118,17 +2139,17 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="46" t="s">
+      <c r="A36" s="68" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="46"/>
-      <c r="C36" s="46"/>
-      <c r="D36" s="46"/>
-      <c r="E36" s="46"/>
-      <c r="F36" s="46"/>
-      <c r="G36" s="46"/>
-      <c r="H36" s="46"/>
-      <c r="I36" s="46"/>
+      <c r="B36" s="68"/>
+      <c r="C36" s="68"/>
+      <c r="D36" s="68"/>
+      <c r="E36" s="68"/>
+      <c r="F36" s="68"/>
+      <c r="G36" s="68"/>
+      <c r="H36" s="68"/>
+      <c r="I36" s="68"/>
     </row>
     <row r="37" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
@@ -2339,17 +2360,17 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="46" t="s">
+      <c r="A47" s="68" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="46"/>
-      <c r="C47" s="46"/>
-      <c r="D47" s="46"/>
-      <c r="E47" s="46"/>
-      <c r="F47" s="46"/>
-      <c r="G47" s="46"/>
-      <c r="H47" s="46"/>
-      <c r="I47" s="46"/>
+      <c r="B47" s="68"/>
+      <c r="C47" s="68"/>
+      <c r="D47" s="68"/>
+      <c r="E47" s="68"/>
+      <c r="F47" s="68"/>
+      <c r="G47" s="68"/>
+      <c r="H47" s="68"/>
+      <c r="I47" s="68"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
@@ -2382,17 +2403,17 @@
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="46" t="s">
+      <c r="A52" s="68" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="46"/>
-      <c r="C52" s="46"/>
-      <c r="D52" s="46"/>
-      <c r="E52" s="46"/>
-      <c r="F52" s="46"/>
-      <c r="G52" s="46"/>
-      <c r="H52" s="46"/>
-      <c r="I52" s="46"/>
+      <c r="B52" s="68"/>
+      <c r="C52" s="68"/>
+      <c r="D52" s="68"/>
+      <c r="E52" s="68"/>
+      <c r="F52" s="68"/>
+      <c r="G52" s="68"/>
+      <c r="H52" s="68"/>
+      <c r="I52" s="68"/>
     </row>
     <row r="53" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
@@ -2943,7 +2964,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03C3DC63-880C-4C7A-BD99-15B2870A7881}">
-  <dimension ref="A1:N69"/>
+  <dimension ref="A1:N73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
@@ -3185,37 +3206,37 @@
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="62" t="s">
         <v>102</v>
       </c>
-      <c r="B13" s="63" t="s">
+      <c r="B13" s="62" t="s">
         <v>170</v>
       </c>
-      <c r="C13" s="63" t="s">
+      <c r="C13" s="62" t="s">
         <v>169</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="D13" s="62" t="s">
         <v>168</v>
       </c>
-      <c r="E13" s="63" t="s">
+      <c r="E13" s="62" t="s">
         <v>184</v>
       </c>
-      <c r="F13" s="63" t="s">
-        <v>301</v>
-      </c>
-      <c r="G13" s="63" t="s">
+      <c r="F13" s="62" t="s">
+        <v>295</v>
+      </c>
+      <c r="G13" s="62" t="s">
         <v>176</v>
       </c>
-      <c r="H13" s="63" t="s">
+      <c r="H13" s="62" t="s">
         <v>185</v>
       </c>
-      <c r="I13" s="63" t="s">
+      <c r="I13" s="62" t="s">
         <v>189</v>
       </c>
-      <c r="J13" s="63" t="s">
+      <c r="J13" s="62" t="s">
         <v>266</v>
       </c>
-      <c r="K13" s="63" t="s">
+      <c r="K13" s="62" t="s">
         <v>265</v>
       </c>
       <c r="N13" t="s">
@@ -3223,1223 +3244,1272 @@
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="60" t="s">
         <v>108</v>
       </c>
-      <c r="B14" s="61">
+      <c r="B14" s="60">
         <v>1</v>
       </c>
-      <c r="C14" s="62" t="s">
+      <c r="C14" s="61" t="s">
         <v>267</v>
       </c>
-      <c r="D14" s="61"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="61"/>
-      <c r="G14" s="61"/>
-      <c r="H14" s="61"/>
-      <c r="I14" s="61"/>
-      <c r="J14" s="60"/>
-      <c r="K14" s="50"/>
+      <c r="D14" s="60"/>
+      <c r="E14" s="59"/>
+      <c r="F14" s="60"/>
+      <c r="G14" s="60"/>
+      <c r="H14" s="60"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="59"/>
+      <c r="K14" s="49"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="55" t="s">
+      <c r="A15" s="54" t="s">
         <v>264</v>
       </c>
-      <c r="B15" s="55">
+      <c r="B15" s="54">
         <v>2</v>
       </c>
-      <c r="C15" s="56" t="s">
+      <c r="C15" s="55" t="s">
         <v>263</v>
       </c>
-      <c r="D15" s="55"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="55"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="59"/>
-      <c r="I15" s="55"/>
-      <c r="J15" s="54">
+      <c r="D15" s="54"/>
+      <c r="E15" s="53"/>
+      <c r="F15" s="54"/>
+      <c r="G15" s="54"/>
+      <c r="H15" s="58"/>
+      <c r="I15" s="54"/>
+      <c r="J15" s="53">
         <f>SUM(J16:J20)</f>
         <v>642</v>
       </c>
-      <c r="K15" s="50"/>
+      <c r="K15" s="49"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="52" t="s">
+      <c r="A16" s="51" t="s">
         <v>262</v>
       </c>
-      <c r="B16" s="52">
-        <v>3</v>
-      </c>
-      <c r="C16" s="53" t="s">
+      <c r="B16" s="51">
+        <v>3</v>
+      </c>
+      <c r="C16" s="52" t="s">
         <v>175</v>
       </c>
-      <c r="D16" s="52">
+      <c r="D16" s="51">
         <v>2</v>
       </c>
-      <c r="E16" s="51">
+      <c r="E16" s="50">
         <v>74</v>
       </c>
-      <c r="F16" s="52" t="s">
+      <c r="F16" s="51" t="s">
         <v>261</v>
       </c>
-      <c r="G16" s="57" t="s">
+      <c r="G16" s="56" t="s">
         <v>180</v>
       </c>
-      <c r="H16" s="52"/>
-      <c r="I16" s="52"/>
-      <c r="J16" s="51">
+      <c r="H16" s="51"/>
+      <c r="I16" s="51"/>
+      <c r="J16" s="50">
         <f>D16*E16</f>
         <v>148</v>
       </c>
-      <c r="K16" s="50"/>
+      <c r="K16" s="49"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="52" t="s">
+      <c r="A17" s="51" t="s">
         <v>260</v>
       </c>
-      <c r="B17" s="52">
-        <v>3</v>
-      </c>
-      <c r="C17" s="53" t="s">
+      <c r="B17" s="51">
+        <v>3</v>
+      </c>
+      <c r="C17" s="52" t="s">
         <v>174</v>
       </c>
-      <c r="D17" s="52">
+      <c r="D17" s="51">
         <v>2</v>
       </c>
-      <c r="E17" s="51">
+      <c r="E17" s="50">
         <v>94</v>
       </c>
-      <c r="F17" s="52" t="s">
+      <c r="F17" s="51" t="s">
         <v>259</v>
       </c>
-      <c r="G17" s="57" t="s">
+      <c r="G17" s="56" t="s">
         <v>180</v>
       </c>
-      <c r="H17" s="52"/>
-      <c r="I17" s="52"/>
-      <c r="J17" s="51">
+      <c r="H17" s="51"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="50">
         <f>D17*E17</f>
         <v>188</v>
       </c>
-      <c r="K17" s="50"/>
+      <c r="K17" s="49"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="52" t="s">
+      <c r="A18" s="51" t="s">
         <v>258</v>
       </c>
-      <c r="B18" s="52">
-        <v>3</v>
-      </c>
-      <c r="C18" s="53" t="s">
+      <c r="B18" s="51">
+        <v>3</v>
+      </c>
+      <c r="C18" s="52" t="s">
         <v>177</v>
       </c>
-      <c r="D18" s="52">
+      <c r="D18" s="51">
         <v>1</v>
       </c>
-      <c r="E18" s="51">
+      <c r="E18" s="50">
         <v>219</v>
       </c>
-      <c r="F18" s="52" t="s">
+      <c r="F18" s="51" t="s">
         <v>257</v>
       </c>
-      <c r="G18" s="57" t="s">
+      <c r="G18" s="56" t="s">
         <v>180</v>
       </c>
-      <c r="H18" s="58">
+      <c r="H18" s="57">
         <v>46213</v>
       </c>
-      <c r="I18" s="58"/>
-      <c r="J18" s="51">
+      <c r="I18" s="57"/>
+      <c r="J18" s="50">
         <f>D18*E18</f>
         <v>219</v>
       </c>
-      <c r="K18" s="50"/>
+      <c r="K18" s="49"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="52" t="s">
+      <c r="A19" s="51" t="s">
         <v>256</v>
       </c>
-      <c r="B19" s="52">
-        <v>3</v>
-      </c>
-      <c r="C19" s="53" t="s">
+      <c r="B19" s="51">
+        <v>3</v>
+      </c>
+      <c r="C19" s="52" t="s">
         <v>173</v>
       </c>
-      <c r="D19" s="52">
-        <v>3</v>
-      </c>
-      <c r="E19" s="51">
+      <c r="D19" s="51">
+        <v>3</v>
+      </c>
+      <c r="E19" s="50">
         <v>29</v>
       </c>
-      <c r="F19" s="52" t="s">
+      <c r="F19" s="51" t="s">
         <v>255</v>
       </c>
-      <c r="G19" s="57" t="s">
+      <c r="G19" s="56" t="s">
         <v>180</v>
       </c>
-      <c r="H19" s="58">
+      <c r="H19" s="57">
         <v>46213</v>
       </c>
-      <c r="I19" s="52" t="s">
+      <c r="I19" s="51" t="s">
         <v>254</v>
       </c>
-      <c r="J19" s="51">
+      <c r="J19" s="50">
         <f>D19*E19</f>
         <v>87</v>
       </c>
-      <c r="K19" s="50" t="s">
+      <c r="K19" s="49" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="52" t="s">
+      <c r="A20" s="51" t="s">
         <v>253</v>
       </c>
-      <c r="B20" s="52">
-        <v>3</v>
-      </c>
-      <c r="C20" s="53" t="s">
+      <c r="B20" s="51">
+        <v>3</v>
+      </c>
+      <c r="C20" s="52" t="s">
         <v>252</v>
       </c>
-      <c r="D20" s="52">
+      <c r="D20" s="51">
         <v>2</v>
       </c>
-      <c r="E20" s="51"/>
-      <c r="F20" s="52" t="s">
+      <c r="E20" s="50"/>
+      <c r="F20" s="51" t="s">
         <v>251</v>
       </c>
-      <c r="G20" s="52"/>
-      <c r="H20" s="58"/>
-      <c r="I20" s="58"/>
-      <c r="J20" s="51"/>
-      <c r="K20" s="50"/>
+      <c r="G20" s="51"/>
+      <c r="H20" s="57"/>
+      <c r="I20" s="57"/>
+      <c r="J20" s="50"/>
+      <c r="K20" s="49"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="55" t="s">
+      <c r="A21" s="54" t="s">
         <v>250</v>
       </c>
-      <c r="B21" s="55">
+      <c r="B21" s="54">
         <v>2</v>
       </c>
-      <c r="C21" s="56" t="s">
+      <c r="C21" s="55" t="s">
         <v>249</v>
       </c>
-      <c r="D21" s="55">
+      <c r="D21" s="54">
         <v>1</v>
       </c>
-      <c r="E21" s="54"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="55"/>
-      <c r="I21" s="55"/>
-      <c r="J21" s="54">
+      <c r="E21" s="53" t="s">
+        <v>309</v>
+      </c>
+      <c r="F21" s="54"/>
+      <c r="G21" s="54"/>
+      <c r="H21" s="54"/>
+      <c r="I21" s="54"/>
+      <c r="J21" s="53">
         <f>SUM(J22:J31)</f>
         <v>0</v>
       </c>
-      <c r="K21" s="50"/>
+      <c r="K21" s="49"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="52" t="s">
+      <c r="A22" s="51" t="s">
         <v>248</v>
       </c>
-      <c r="B22" s="52">
-        <v>3</v>
-      </c>
-      <c r="C22" s="53" t="s">
+      <c r="B22" s="51">
+        <v>3</v>
+      </c>
+      <c r="C22" s="52" t="s">
         <v>269</v>
       </c>
-      <c r="D22" s="52">
+      <c r="D22" s="51">
         <v>39</v>
       </c>
-      <c r="E22" s="51"/>
-      <c r="F22" s="52" t="s">
+      <c r="E22" s="50">
+        <v>7.21</v>
+      </c>
+      <c r="F22" s="51" t="s">
+        <v>314</v>
+      </c>
+      <c r="G22" s="63" t="s">
+        <v>180</v>
+      </c>
+      <c r="H22" s="51"/>
+      <c r="I22" s="51"/>
+      <c r="J22" s="50"/>
+      <c r="K22" s="49"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="51"/>
+      <c r="B23" s="51"/>
+      <c r="C23" s="52"/>
+      <c r="D23" s="51"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="51"/>
+      <c r="H23" s="57"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="50"/>
+      <c r="K23" s="49"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="51" t="s">
+        <v>247</v>
+      </c>
+      <c r="B24" s="51">
+        <v>3</v>
+      </c>
+      <c r="C24" s="52" t="s">
+        <v>270</v>
+      </c>
+      <c r="D24" s="51">
+        <v>78</v>
+      </c>
+      <c r="E24" s="50">
+        <v>12.99</v>
+      </c>
+      <c r="F24" s="51" t="s">
+        <v>313</v>
+      </c>
+      <c r="G24" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="H24" s="51"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="50"/>
+      <c r="K24" s="49"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="51" t="s">
+        <v>246</v>
+      </c>
+      <c r="B25" s="51">
+        <v>3</v>
+      </c>
+      <c r="C25" s="52" t="s">
+        <v>271</v>
+      </c>
+      <c r="D25" s="51">
+        <v>4</v>
+      </c>
+      <c r="E25" s="50">
+        <v>9.99</v>
+      </c>
+      <c r="F25" s="51" t="s">
+        <v>312</v>
+      </c>
+      <c r="G25" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="H25" s="51"/>
+      <c r="I25" s="51"/>
+      <c r="J25" s="50"/>
+      <c r="K25" s="49"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="51" t="s">
+        <v>245</v>
+      </c>
+      <c r="B26" s="51">
+        <v>3</v>
+      </c>
+      <c r="C26" s="52" t="s">
+        <v>272</v>
+      </c>
+      <c r="D26" s="51">
+        <v>2</v>
+      </c>
+      <c r="E26" s="50">
+        <v>9.7899999999999991</v>
+      </c>
+      <c r="F26" s="51" t="s">
+        <v>311</v>
+      </c>
+      <c r="G26" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="H26" s="51"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="50"/>
+      <c r="K26" s="49"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="51"/>
+      <c r="B27" s="51"/>
+      <c r="C27" s="52"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="50"/>
+      <c r="K27" s="49"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="51" t="s">
+        <v>244</v>
+      </c>
+      <c r="B28" s="51">
+        <v>3</v>
+      </c>
+      <c r="C28" s="52" t="s">
+        <v>274</v>
+      </c>
+      <c r="D28" s="51">
+        <v>15</v>
+      </c>
+      <c r="E28" s="50">
+        <v>6.99</v>
+      </c>
+      <c r="F28" s="51" t="s">
+        <v>310</v>
+      </c>
+      <c r="G28" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="H28" s="51"/>
+      <c r="I28" s="51"/>
+      <c r="J28" s="50"/>
+      <c r="K28" s="49"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="51" t="s">
+        <v>243</v>
+      </c>
+      <c r="B29" s="51">
+        <v>3</v>
+      </c>
+      <c r="C29" s="52" t="s">
+        <v>275</v>
+      </c>
+      <c r="D29" s="51">
+        <v>5</v>
+      </c>
+      <c r="E29" s="50">
+        <v>8.99</v>
+      </c>
+      <c r="F29" s="51" t="s">
+        <v>315</v>
+      </c>
+      <c r="G29" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="50"/>
+      <c r="K29" s="49"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="51" t="s">
+        <v>242</v>
+      </c>
+      <c r="B30" s="51"/>
+      <c r="C30" s="52"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="51"/>
+      <c r="H30" s="51"/>
+      <c r="I30" s="51"/>
+      <c r="J30" s="50"/>
+      <c r="K30" s="49"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="51" t="s">
+        <v>241</v>
+      </c>
+      <c r="B31" s="51">
+        <v>3</v>
+      </c>
+      <c r="C31" s="52" t="s">
+        <v>273</v>
+      </c>
+      <c r="D31" s="51">
+        <v>6</v>
+      </c>
+      <c r="E31" s="50">
+        <v>7.79</v>
+      </c>
+      <c r="F31" s="51" t="s">
+        <v>316</v>
+      </c>
+      <c r="G31" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="H31" s="51"/>
+      <c r="I31" s="51"/>
+      <c r="J31" s="50"/>
+      <c r="K31" s="49"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="51" t="s">
+        <v>240</v>
+      </c>
+      <c r="B32" s="51">
+        <v>3</v>
+      </c>
+      <c r="C32" s="52" t="s">
         <v>276</v>
       </c>
-      <c r="G22" s="67" t="s">
+      <c r="D32" s="51">
+        <v>3</v>
+      </c>
+      <c r="E32" s="50"/>
+      <c r="F32" s="51" t="s">
+        <v>281</v>
+      </c>
+      <c r="G32" s="51"/>
+      <c r="H32" s="51"/>
+      <c r="I32" s="51"/>
+      <c r="J32" s="50"/>
+      <c r="K32" s="49"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="51" t="s">
+        <v>239</v>
+      </c>
+      <c r="B33" s="51">
+        <v>3</v>
+      </c>
+      <c r="C33" s="52" t="s">
+        <v>280</v>
+      </c>
+      <c r="D33" s="51">
+        <v>7</v>
+      </c>
+      <c r="E33" s="50"/>
+      <c r="F33" s="51" t="s">
+        <v>282</v>
+      </c>
+      <c r="G33" s="51"/>
+      <c r="H33" s="51"/>
+      <c r="I33" s="51"/>
+      <c r="J33" s="50"/>
+      <c r="K33" s="49" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="51" t="s">
+        <v>277</v>
+      </c>
+      <c r="B34" s="51">
+        <v>3</v>
+      </c>
+      <c r="C34" s="52" t="s">
+        <v>307</v>
+      </c>
+      <c r="D34" s="51">
+        <v>1</v>
+      </c>
+      <c r="E34" s="50"/>
+      <c r="F34" s="51" t="s">
+        <v>308</v>
+      </c>
+      <c r="G34" s="51"/>
+      <c r="H34" s="51"/>
+      <c r="I34" s="51"/>
+      <c r="J34" s="50"/>
+      <c r="K34" s="49"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="51"/>
+      <c r="B35" s="51"/>
+      <c r="C35" s="52"/>
+      <c r="D35" s="51"/>
+      <c r="E35" s="50"/>
+      <c r="F35" s="69"/>
+      <c r="G35" s="51"/>
+      <c r="H35" s="51"/>
+      <c r="I35" s="51"/>
+      <c r="J35" s="50"/>
+      <c r="K35" s="49"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="51" t="s">
+        <v>277</v>
+      </c>
+      <c r="B36" s="51">
+        <v>3</v>
+      </c>
+      <c r="C36" s="52" t="s">
+        <v>294</v>
+      </c>
+      <c r="D36" s="51">
+        <v>1</v>
+      </c>
+      <c r="E36" s="50"/>
+      <c r="F36" s="65" t="s">
+        <v>305</v>
+      </c>
+      <c r="G36" s="51"/>
+      <c r="H36" s="51"/>
+      <c r="I36" s="51"/>
+      <c r="J36" s="50"/>
+      <c r="K36" s="49"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="51" t="s">
+        <v>278</v>
+      </c>
+      <c r="B37" s="51">
+        <v>3</v>
+      </c>
+      <c r="C37" s="52" t="s">
+        <v>293</v>
+      </c>
+      <c r="D37" s="51">
+        <v>1</v>
+      </c>
+      <c r="E37" s="50"/>
+      <c r="F37" s="66"/>
+      <c r="G37" s="51"/>
+      <c r="H37" s="51"/>
+      <c r="I37" s="51"/>
+      <c r="J37" s="50"/>
+      <c r="K37" s="49"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="51" t="s">
+        <v>279</v>
+      </c>
+      <c r="B38" s="51">
+        <v>3</v>
+      </c>
+      <c r="C38" s="52" t="s">
+        <v>291</v>
+      </c>
+      <c r="D38" s="51">
+        <v>78</v>
+      </c>
+      <c r="E38" s="50"/>
+      <c r="F38" s="66"/>
+      <c r="G38" s="51"/>
+      <c r="H38" s="51"/>
+      <c r="I38" s="51"/>
+      <c r="J38" s="50"/>
+      <c r="K38" s="49"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="51" t="s">
+        <v>283</v>
+      </c>
+      <c r="B39" s="51">
+        <v>3</v>
+      </c>
+      <c r="C39" s="52" t="s">
+        <v>292</v>
+      </c>
+      <c r="D39" s="51">
+        <v>39</v>
+      </c>
+      <c r="E39" s="50"/>
+      <c r="F39" s="66"/>
+      <c r="G39" s="51"/>
+      <c r="H39" s="51"/>
+      <c r="I39" s="51"/>
+      <c r="J39" s="50"/>
+      <c r="K39" s="49"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="51" t="s">
+        <v>284</v>
+      </c>
+      <c r="B40" s="51">
+        <v>3</v>
+      </c>
+      <c r="C40" s="52" t="s">
+        <v>296</v>
+      </c>
+      <c r="D40" s="51">
+        <v>2</v>
+      </c>
+      <c r="E40" s="50"/>
+      <c r="F40" s="66"/>
+      <c r="G40" s="51"/>
+      <c r="H40" s="51"/>
+      <c r="I40" s="51"/>
+      <c r="J40" s="50"/>
+      <c r="K40" s="49"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="51" t="s">
+        <v>285</v>
+      </c>
+      <c r="B41" s="51">
+        <v>3</v>
+      </c>
+      <c r="C41" s="52" t="s">
+        <v>297</v>
+      </c>
+      <c r="D41" s="51">
+        <v>2</v>
+      </c>
+      <c r="E41" s="50"/>
+      <c r="F41" s="66"/>
+      <c r="G41" s="51"/>
+      <c r="H41" s="51"/>
+      <c r="I41" s="51"/>
+      <c r="J41" s="50"/>
+      <c r="K41" s="49"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="51" t="s">
+        <v>286</v>
+      </c>
+      <c r="B42" s="51">
+        <v>3</v>
+      </c>
+      <c r="C42" s="52" t="s">
+        <v>299</v>
+      </c>
+      <c r="D42" s="51">
+        <v>1</v>
+      </c>
+      <c r="E42" s="50"/>
+      <c r="F42" s="66"/>
+      <c r="G42" s="51"/>
+      <c r="H42" s="51"/>
+      <c r="I42" s="51"/>
+      <c r="J42" s="50"/>
+      <c r="K42" s="49"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="51" t="s">
+        <v>287</v>
+      </c>
+      <c r="B43" s="51">
+        <v>3</v>
+      </c>
+      <c r="C43" s="52" t="s">
+        <v>300</v>
+      </c>
+      <c r="D43" s="51">
+        <v>1</v>
+      </c>
+      <c r="E43" s="50"/>
+      <c r="F43" s="66"/>
+      <c r="G43" s="51"/>
+      <c r="H43" s="51"/>
+      <c r="I43" s="51"/>
+      <c r="J43" s="50"/>
+      <c r="K43" s="49"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="51" t="s">
+        <v>288</v>
+      </c>
+      <c r="B44" s="51">
+        <v>3</v>
+      </c>
+      <c r="C44" s="52" t="s">
+        <v>301</v>
+      </c>
+      <c r="D44" s="51">
+        <v>1</v>
+      </c>
+      <c r="E44" s="50"/>
+      <c r="F44" s="66"/>
+      <c r="G44" s="51"/>
+      <c r="H44" s="51"/>
+      <c r="I44" s="51"/>
+      <c r="J44" s="50"/>
+      <c r="K44" s="49"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" s="51" t="s">
+        <v>289</v>
+      </c>
+      <c r="B45" s="51">
+        <v>3</v>
+      </c>
+      <c r="C45" s="52" t="s">
+        <v>303</v>
+      </c>
+      <c r="D45" s="51">
+        <v>1</v>
+      </c>
+      <c r="E45" s="50"/>
+      <c r="F45" s="66"/>
+      <c r="G45" s="51"/>
+      <c r="H45" s="51"/>
+      <c r="I45" s="51"/>
+      <c r="J45" s="50"/>
+      <c r="K45" s="49"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="51" t="s">
+        <v>290</v>
+      </c>
+      <c r="B46" s="51">
+        <v>3</v>
+      </c>
+      <c r="C46" s="52" t="s">
+        <v>304</v>
+      </c>
+      <c r="D46" s="51">
+        <v>1</v>
+      </c>
+      <c r="E46" s="50"/>
+      <c r="F46" s="66"/>
+      <c r="G46" s="51"/>
+      <c r="H46" s="51"/>
+      <c r="I46" s="51"/>
+      <c r="J46" s="50"/>
+      <c r="K46" s="49"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" s="51" t="s">
+        <v>298</v>
+      </c>
+      <c r="B47" s="51">
+        <v>3</v>
+      </c>
+      <c r="C47" s="52" t="s">
+        <v>304</v>
+      </c>
+      <c r="D47" s="51">
+        <v>1</v>
+      </c>
+      <c r="E47" s="50"/>
+      <c r="F47" s="66"/>
+      <c r="G47" s="51"/>
+      <c r="H47" s="51"/>
+      <c r="I47" s="51"/>
+      <c r="J47" s="50"/>
+      <c r="K47" s="49"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" s="51" t="s">
+        <v>302</v>
+      </c>
+      <c r="B48" s="51">
+        <v>3</v>
+      </c>
+      <c r="C48" s="52" t="s">
+        <v>306</v>
+      </c>
+      <c r="D48" s="51">
+        <v>1</v>
+      </c>
+      <c r="E48" s="50"/>
+      <c r="F48" s="67"/>
+      <c r="G48" s="51"/>
+      <c r="H48" s="51"/>
+      <c r="I48" s="51"/>
+      <c r="J48" s="50"/>
+      <c r="K48" s="49"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" s="70"/>
+      <c r="B49" s="70"/>
+      <c r="C49" s="71"/>
+      <c r="D49" s="70"/>
+      <c r="E49" s="72"/>
+      <c r="K49" s="49"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K50" s="49"/>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K51" s="49"/>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" s="54" t="s">
+        <v>238</v>
+      </c>
+      <c r="B52" s="54">
+        <v>2</v>
+      </c>
+      <c r="C52" s="55" t="s">
+        <v>237</v>
+      </c>
+      <c r="D52" s="54"/>
+      <c r="E52" s="53"/>
+      <c r="F52" s="54"/>
+      <c r="G52" s="54"/>
+      <c r="H52" s="54"/>
+      <c r="I52" s="54"/>
+      <c r="J52" s="53">
+        <f>SUM(J53:J55)</f>
+        <v>402</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="51" t="s">
+        <v>236</v>
+      </c>
+      <c r="B53" s="51">
+        <v>3</v>
+      </c>
+      <c r="C53" s="52" t="s">
+        <v>235</v>
+      </c>
+      <c r="D53" s="51">
+        <v>3</v>
+      </c>
+      <c r="E53" s="50">
+        <v>65</v>
+      </c>
+      <c r="F53" s="51" t="s">
+        <v>232</v>
+      </c>
+      <c r="G53" s="56" t="s">
         <v>180</v>
       </c>
-      <c r="H22" s="52"/>
-      <c r="I22" s="52"/>
-      <c r="J22" s="51"/>
-      <c r="K22" s="50"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
-      <c r="B23" s="52"/>
-      <c r="C23" s="53"/>
-      <c r="D23" s="52"/>
-      <c r="E23" s="51"/>
-      <c r="F23" s="52"/>
-      <c r="G23" s="52"/>
-      <c r="H23" s="58"/>
-      <c r="I23" s="52"/>
-      <c r="J23" s="51"/>
-      <c r="K23" s="50"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="52" t="s">
-        <v>247</v>
-      </c>
-      <c r="B24" s="52">
-        <v>3</v>
-      </c>
-      <c r="C24" s="53" t="s">
-        <v>270</v>
-      </c>
-      <c r="D24" s="52">
-        <v>78</v>
-      </c>
-      <c r="E24" s="51"/>
-      <c r="F24" s="52" t="s">
-        <v>275</v>
-      </c>
-      <c r="G24" s="68" t="s">
+      <c r="H53" s="57">
+        <v>46213</v>
+      </c>
+      <c r="I53" s="51"/>
+      <c r="J53" s="50">
+        <f>D53*E53</f>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="51" t="s">
+        <v>234</v>
+      </c>
+      <c r="B54" s="51">
+        <v>3</v>
+      </c>
+      <c r="C54" s="52" t="s">
+        <v>233</v>
+      </c>
+      <c r="D54" s="51">
+        <v>3</v>
+      </c>
+      <c r="E54" s="50">
+        <v>69</v>
+      </c>
+      <c r="F54" s="51" t="s">
+        <v>232</v>
+      </c>
+      <c r="G54" s="56" t="s">
         <v>180</v>
       </c>
-      <c r="H24" s="52"/>
-      <c r="I24" s="52"/>
-      <c r="J24" s="51"/>
-      <c r="K24" s="50"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="52" t="s">
-        <v>246</v>
-      </c>
-      <c r="B25" s="52">
-        <v>3</v>
-      </c>
-      <c r="C25" s="53" t="s">
-        <v>271</v>
-      </c>
-      <c r="D25" s="52">
-        <v>4</v>
-      </c>
-      <c r="E25" s="51"/>
-      <c r="F25" s="52" t="s">
-        <v>312</v>
-      </c>
-      <c r="G25" s="68" t="s">
-        <v>180</v>
-      </c>
-      <c r="H25" s="52"/>
-      <c r="I25" s="52"/>
-      <c r="J25" s="51"/>
-      <c r="K25" s="50"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="52" t="s">
-        <v>245</v>
-      </c>
-      <c r="B26" s="52">
-        <v>3</v>
-      </c>
-      <c r="C26" s="53" t="s">
-        <v>272</v>
-      </c>
-      <c r="D26" s="52">
+      <c r="H54" s="51"/>
+      <c r="I54" s="51"/>
+      <c r="J54" s="50">
+        <f>D54*E54</f>
+        <v>207</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="51" t="s">
+        <v>231</v>
+      </c>
+      <c r="B55" s="51">
+        <v>3</v>
+      </c>
+      <c r="C55" s="52" t="s">
+        <v>230</v>
+      </c>
+      <c r="D55" s="51">
+        <v>3</v>
+      </c>
+      <c r="E55" s="50"/>
+      <c r="F55" s="51" t="s">
+        <v>229</v>
+      </c>
+      <c r="G55" s="51"/>
+      <c r="H55" s="51"/>
+      <c r="I55" s="51"/>
+      <c r="J55" s="50"/>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="54" t="s">
+        <v>228</v>
+      </c>
+      <c r="B56" s="54">
         <v>2</v>
       </c>
-      <c r="E26" s="51"/>
-      <c r="F26" s="52" t="s">
-        <v>274</v>
-      </c>
-      <c r="G26" s="68" t="s">
-        <v>180</v>
-      </c>
-      <c r="H26" s="52"/>
-      <c r="I26" s="52"/>
-      <c r="J26" s="51"/>
-      <c r="K26" s="50"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="52"/>
-      <c r="B27" s="52"/>
-      <c r="C27" s="53"/>
-      <c r="D27" s="52"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="52"/>
-      <c r="G27" s="52"/>
-      <c r="H27" s="52"/>
-      <c r="I27" s="52"/>
-      <c r="J27" s="51"/>
-      <c r="K27" s="50"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="52" t="s">
-        <v>244</v>
-      </c>
-      <c r="B28" s="52">
-        <v>3</v>
-      </c>
-      <c r="C28" s="53" t="s">
-        <v>278</v>
-      </c>
-      <c r="D28" s="52">
-        <v>15</v>
-      </c>
-      <c r="E28" s="51"/>
-      <c r="F28" s="52" t="s">
-        <v>280</v>
-      </c>
-      <c r="G28" s="68" t="s">
-        <v>180</v>
-      </c>
-      <c r="H28" s="52"/>
-      <c r="I28" s="52"/>
-      <c r="J28" s="51"/>
-      <c r="K28" s="50"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="52" t="s">
-        <v>243</v>
-      </c>
-      <c r="B29" s="52">
-        <v>3</v>
-      </c>
-      <c r="C29" s="53" t="s">
-        <v>279</v>
-      </c>
-      <c r="D29" s="52">
-        <v>5</v>
-      </c>
-      <c r="E29" s="51"/>
-      <c r="F29" s="52" t="s">
-        <v>281</v>
-      </c>
-      <c r="G29" s="68" t="s">
-        <v>180</v>
-      </c>
-      <c r="H29" s="52"/>
-      <c r="I29" s="52"/>
-      <c r="J29" s="51"/>
-      <c r="K29" s="50"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="52" t="s">
-        <v>242</v>
-      </c>
-      <c r="B30" s="52"/>
-      <c r="C30" s="53"/>
-      <c r="D30" s="52"/>
-      <c r="E30" s="51"/>
-      <c r="F30" s="52"/>
-      <c r="G30" s="52"/>
-      <c r="H30" s="52"/>
-      <c r="I30" s="52"/>
-      <c r="J30" s="51"/>
-      <c r="K30" s="50"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="52" t="s">
-        <v>241</v>
-      </c>
-      <c r="B31" s="52">
-        <v>3</v>
-      </c>
-      <c r="C31" s="53" t="s">
-        <v>277</v>
-      </c>
-      <c r="D31" s="52">
-        <v>6</v>
-      </c>
-      <c r="E31" s="51"/>
-      <c r="F31" s="52" t="s">
-        <v>273</v>
-      </c>
-      <c r="G31" s="68" t="s">
-        <v>180</v>
-      </c>
-      <c r="H31" s="52"/>
-      <c r="I31" s="52"/>
-      <c r="J31" s="51"/>
-      <c r="K31" s="50"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="52" t="s">
-        <v>240</v>
-      </c>
-      <c r="B32" s="52">
-        <v>3</v>
-      </c>
-      <c r="C32" s="53" t="s">
-        <v>282</v>
-      </c>
-      <c r="D32" s="52">
-        <v>3</v>
-      </c>
-      <c r="E32" s="51"/>
-      <c r="F32" s="52" t="s">
-        <v>287</v>
-      </c>
-      <c r="G32" s="52"/>
-      <c r="H32" s="52"/>
-      <c r="I32" s="52"/>
-      <c r="J32" s="51"/>
-      <c r="K32" s="50"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="52" t="s">
-        <v>239</v>
-      </c>
-      <c r="B33" s="52">
-        <v>3</v>
-      </c>
-      <c r="C33" s="53" t="s">
-        <v>286</v>
-      </c>
-      <c r="D33" s="52">
-        <v>7</v>
-      </c>
-      <c r="E33" s="51"/>
-      <c r="F33" s="52" t="s">
-        <v>288</v>
-      </c>
-      <c r="G33" s="52"/>
-      <c r="H33" s="52"/>
-      <c r="I33" s="52"/>
-      <c r="J33" s="51"/>
-      <c r="K33" s="50" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" s="52"/>
-      <c r="B34" s="52"/>
-      <c r="C34" s="53"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="51"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="52"/>
-      <c r="H34" s="52"/>
-      <c r="I34" s="52"/>
-      <c r="J34" s="51"/>
-      <c r="K34" s="50"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="52" t="s">
-        <v>283</v>
-      </c>
-      <c r="B35" s="52">
-        <v>3</v>
-      </c>
-      <c r="C35" s="53" t="s">
-        <v>300</v>
-      </c>
-      <c r="D35" s="52">
+      <c r="C56" s="55" t="s">
+        <v>227</v>
+      </c>
+      <c r="D56" s="54"/>
+      <c r="E56" s="53"/>
+      <c r="F56" s="54"/>
+      <c r="G56" s="54"/>
+      <c r="H56" s="54"/>
+      <c r="I56" s="54"/>
+      <c r="J56" s="53">
+        <f>SUM(J57:J60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" s="51" t="s">
+        <v>226</v>
+      </c>
+      <c r="B57" s="51">
+        <v>3</v>
+      </c>
+      <c r="C57" s="52" t="s">
+        <v>225</v>
+      </c>
+      <c r="D57" s="51"/>
+      <c r="E57" s="50"/>
+      <c r="F57" s="51" t="s">
+        <v>224</v>
+      </c>
+      <c r="G57" s="51"/>
+      <c r="H57" s="51"/>
+      <c r="I57" s="51"/>
+      <c r="J57" s="50"/>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" s="51" t="s">
+        <v>223</v>
+      </c>
+      <c r="B58" s="51">
+        <v>3</v>
+      </c>
+      <c r="C58" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="D58" s="51"/>
+      <c r="E58" s="50"/>
+      <c r="F58" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="G58" s="51"/>
+      <c r="H58" s="51"/>
+      <c r="I58" s="51"/>
+      <c r="J58" s="50"/>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" s="51" t="s">
+        <v>220</v>
+      </c>
+      <c r="B59" s="51">
+        <v>3</v>
+      </c>
+      <c r="C59" s="52" t="s">
+        <v>219</v>
+      </c>
+      <c r="D59" s="51"/>
+      <c r="E59" s="50"/>
+      <c r="F59" s="51" t="s">
+        <v>191</v>
+      </c>
+      <c r="G59" s="51"/>
+      <c r="H59" s="51"/>
+      <c r="I59" s="51"/>
+      <c r="J59" s="50"/>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="B60" s="51">
+        <v>3</v>
+      </c>
+      <c r="C60" s="52" t="s">
+        <v>217</v>
+      </c>
+      <c r="D60" s="51"/>
+      <c r="E60" s="50"/>
+      <c r="F60" s="51" t="s">
+        <v>216</v>
+      </c>
+      <c r="G60" s="51"/>
+      <c r="H60" s="51"/>
+      <c r="I60" s="51"/>
+      <c r="J60" s="50"/>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" s="54" t="s">
+        <v>215</v>
+      </c>
+      <c r="B61" s="54">
+        <v>2</v>
+      </c>
+      <c r="C61" s="55" t="s">
+        <v>214</v>
+      </c>
+      <c r="D61" s="54"/>
+      <c r="E61" s="53"/>
+      <c r="F61" s="54"/>
+      <c r="G61" s="54"/>
+      <c r="H61" s="54"/>
+      <c r="I61" s="54"/>
+      <c r="J61" s="53">
+        <f>SUM(J62:J63)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" s="51" t="s">
+        <v>213</v>
+      </c>
+      <c r="B62" s="51">
+        <v>3</v>
+      </c>
+      <c r="C62" s="52" t="s">
+        <v>212</v>
+      </c>
+      <c r="D62" s="51"/>
+      <c r="E62" s="50"/>
+      <c r="F62" s="51" t="s">
+        <v>211</v>
+      </c>
+      <c r="G62" s="51"/>
+      <c r="H62" s="51"/>
+      <c r="I62" s="51"/>
+      <c r="J62" s="50"/>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" s="51" t="s">
+        <v>210</v>
+      </c>
+      <c r="B63" s="51">
+        <v>3</v>
+      </c>
+      <c r="C63" s="52" t="s">
+        <v>209</v>
+      </c>
+      <c r="D63" s="51"/>
+      <c r="E63" s="50"/>
+      <c r="F63" s="51" t="s">
+        <v>191</v>
+      </c>
+      <c r="G63" s="51"/>
+      <c r="H63" s="51"/>
+      <c r="I63" s="51"/>
+      <c r="J63" s="50"/>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A64" s="54" t="s">
+        <v>208</v>
+      </c>
+      <c r="B64" s="54">
+        <v>2</v>
+      </c>
+      <c r="C64" s="55" t="s">
+        <v>207</v>
+      </c>
+      <c r="D64" s="54"/>
+      <c r="E64" s="53"/>
+      <c r="F64" s="54"/>
+      <c r="G64" s="54"/>
+      <c r="H64" s="54"/>
+      <c r="I64" s="54"/>
+      <c r="J64" s="53">
+        <f>SUM(J65:J68)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" s="51" t="s">
+        <v>206</v>
+      </c>
+      <c r="B65" s="51">
+        <v>3</v>
+      </c>
+      <c r="C65" s="52" t="s">
+        <v>205</v>
+      </c>
+      <c r="D65" s="51"/>
+      <c r="E65" s="50"/>
+      <c r="F65" s="51" t="s">
+        <v>191</v>
+      </c>
+      <c r="G65" s="51"/>
+      <c r="H65" s="51"/>
+      <c r="I65" s="51"/>
+      <c r="J65" s="50"/>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" s="51" t="s">
+        <v>204</v>
+      </c>
+      <c r="B66" s="51">
+        <v>3</v>
+      </c>
+      <c r="C66" s="52" t="s">
+        <v>203</v>
+      </c>
+      <c r="D66" s="51">
         <v>1</v>
       </c>
-      <c r="E35" s="51"/>
-      <c r="F35" s="64" t="s">
-        <v>311</v>
-      </c>
-      <c r="G35" s="52"/>
-      <c r="H35" s="52"/>
-      <c r="I35" s="52"/>
-      <c r="J35" s="51"/>
-      <c r="K35" s="50"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="52" t="s">
-        <v>284</v>
-      </c>
-      <c r="B36" s="52">
-        <v>3</v>
-      </c>
-      <c r="C36" s="53" t="s">
-        <v>299</v>
-      </c>
-      <c r="D36" s="52">
-        <v>1</v>
-      </c>
-      <c r="E36" s="51"/>
-      <c r="F36" s="65"/>
-      <c r="G36" s="52"/>
-      <c r="H36" s="52"/>
-      <c r="I36" s="52"/>
-      <c r="J36" s="51"/>
-      <c r="K36" s="50"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" s="52" t="s">
-        <v>285</v>
-      </c>
-      <c r="B37" s="52">
-        <v>3</v>
-      </c>
-      <c r="C37" s="53" t="s">
-        <v>297</v>
-      </c>
-      <c r="D37" s="52">
-        <v>78</v>
-      </c>
-      <c r="E37" s="51"/>
-      <c r="F37" s="65"/>
-      <c r="G37" s="52"/>
-      <c r="H37" s="52"/>
-      <c r="I37" s="52"/>
-      <c r="J37" s="51"/>
-      <c r="K37" s="50"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" s="52" t="s">
-        <v>289</v>
-      </c>
-      <c r="B38" s="52">
-        <v>3</v>
-      </c>
-      <c r="C38" s="53" t="s">
-        <v>298</v>
-      </c>
-      <c r="D38" s="52">
-        <v>39</v>
-      </c>
-      <c r="E38" s="51"/>
-      <c r="F38" s="65"/>
-      <c r="G38" s="52"/>
-      <c r="H38" s="52"/>
-      <c r="I38" s="52"/>
-      <c r="J38" s="51"/>
-      <c r="K38" s="50"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" s="52" t="s">
-        <v>290</v>
-      </c>
-      <c r="B39" s="52">
-        <v>3</v>
-      </c>
-      <c r="C39" s="53" t="s">
-        <v>302</v>
-      </c>
-      <c r="D39" s="52">
+      <c r="E66" s="50"/>
+      <c r="F66" s="51" t="s">
+        <v>202</v>
+      </c>
+      <c r="G66" s="51"/>
+      <c r="H66" s="51"/>
+      <c r="I66" s="51"/>
+      <c r="J66" s="50"/>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" s="51" t="s">
+        <v>201</v>
+      </c>
+      <c r="B67" s="51">
+        <v>3</v>
+      </c>
+      <c r="C67" s="52" t="s">
+        <v>200</v>
+      </c>
+      <c r="D67" s="51"/>
+      <c r="E67" s="50"/>
+      <c r="F67" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="G67" s="51"/>
+      <c r="H67" s="51"/>
+      <c r="I67" s="51"/>
+      <c r="J67" s="50"/>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="B68" s="51">
+        <v>3</v>
+      </c>
+      <c r="C68" s="52" t="s">
+        <v>197</v>
+      </c>
+      <c r="D68" s="51"/>
+      <c r="E68" s="50"/>
+      <c r="F68" s="51" t="s">
+        <v>191</v>
+      </c>
+      <c r="G68" s="51"/>
+      <c r="H68" s="51"/>
+      <c r="I68" s="51"/>
+      <c r="J68" s="50"/>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" s="54" t="s">
+        <v>196</v>
+      </c>
+      <c r="B69" s="54">
         <v>2</v>
       </c>
-      <c r="E39" s="51"/>
-      <c r="F39" s="65"/>
-      <c r="G39" s="52"/>
-      <c r="H39" s="52"/>
-      <c r="I39" s="52"/>
-      <c r="J39" s="51"/>
-      <c r="K39" s="50"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" s="52" t="s">
-        <v>291</v>
-      </c>
-      <c r="B40" s="52">
-        <v>3</v>
-      </c>
-      <c r="C40" s="53" t="s">
-        <v>303</v>
-      </c>
-      <c r="D40" s="52">
+      <c r="C69" s="55" t="s">
+        <v>268</v>
+      </c>
+      <c r="D69" s="54">
         <v>2</v>
       </c>
-      <c r="E40" s="51"/>
-      <c r="F40" s="65"/>
-      <c r="G40" s="52"/>
-      <c r="H40" s="52"/>
-      <c r="I40" s="52"/>
-      <c r="J40" s="51"/>
-      <c r="K40" s="50"/>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" s="52" t="s">
-        <v>292</v>
-      </c>
-      <c r="B41" s="52">
-        <v>3</v>
-      </c>
-      <c r="C41" s="53" t="s">
-        <v>305</v>
-      </c>
-      <c r="D41" s="52">
-        <v>1</v>
-      </c>
-      <c r="E41" s="51"/>
-      <c r="F41" s="65"/>
-      <c r="G41" s="52"/>
-      <c r="H41" s="52"/>
-      <c r="I41" s="52"/>
-      <c r="J41" s="51"/>
-      <c r="K41" s="50"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" s="52" t="s">
-        <v>293</v>
-      </c>
-      <c r="B42" s="52">
-        <v>3</v>
-      </c>
-      <c r="C42" s="53" t="s">
-        <v>306</v>
-      </c>
-      <c r="D42" s="52">
-        <v>1</v>
-      </c>
-      <c r="E42" s="51"/>
-      <c r="F42" s="65"/>
-      <c r="G42" s="52"/>
-      <c r="H42" s="52"/>
-      <c r="I42" s="52"/>
-      <c r="J42" s="51"/>
-      <c r="K42" s="50"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" s="52" t="s">
-        <v>294</v>
-      </c>
-      <c r="B43" s="52">
-        <v>3</v>
-      </c>
-      <c r="C43" s="53" t="s">
-        <v>307</v>
-      </c>
-      <c r="D43" s="52">
-        <v>1</v>
-      </c>
-      <c r="E43" s="51"/>
-      <c r="F43" s="65"/>
-      <c r="G43" s="52"/>
-      <c r="H43" s="52"/>
-      <c r="I43" s="52"/>
-      <c r="J43" s="51"/>
-      <c r="K43" s="50"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" s="52" t="s">
-        <v>295</v>
-      </c>
-      <c r="B44" s="52">
-        <v>3</v>
-      </c>
-      <c r="C44" s="53" t="s">
-        <v>309</v>
-      </c>
-      <c r="D44" s="52">
-        <v>1</v>
-      </c>
-      <c r="E44" s="51"/>
-      <c r="F44" s="65"/>
-      <c r="G44" s="52"/>
-      <c r="H44" s="52"/>
-      <c r="I44" s="52"/>
-      <c r="J44" s="51"/>
-      <c r="K44" s="50"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" s="52" t="s">
-        <v>296</v>
-      </c>
-      <c r="B45" s="52">
-        <v>3</v>
-      </c>
-      <c r="C45" s="53" t="s">
-        <v>310</v>
-      </c>
-      <c r="D45" s="52">
-        <v>1</v>
-      </c>
-      <c r="E45" s="51"/>
-      <c r="F45" s="65"/>
-      <c r="G45" s="52"/>
-      <c r="H45" s="52"/>
-      <c r="I45" s="52"/>
-      <c r="J45" s="51"/>
-      <c r="K45" s="50"/>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" s="52" t="s">
-        <v>304</v>
-      </c>
-      <c r="B46" s="52">
-        <v>3</v>
-      </c>
-      <c r="C46" s="53" t="s">
-        <v>310</v>
-      </c>
-      <c r="D46" s="52">
-        <v>1</v>
-      </c>
-      <c r="E46" s="51"/>
-      <c r="F46" s="65"/>
-      <c r="G46" s="52"/>
-      <c r="H46" s="52"/>
-      <c r="I46" s="52"/>
-      <c r="J46" s="51"/>
-      <c r="K46" s="50"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" s="52" t="s">
-        <v>308</v>
-      </c>
-      <c r="B47" s="52">
-        <v>4</v>
-      </c>
-      <c r="C47" s="53" t="s">
-        <v>313</v>
-      </c>
-      <c r="D47" s="52">
-        <v>1</v>
-      </c>
-      <c r="E47" s="51"/>
-      <c r="F47" s="66"/>
-      <c r="G47" s="52"/>
-      <c r="H47" s="52"/>
-      <c r="I47" s="52"/>
-      <c r="J47" s="51"/>
-      <c r="K47" s="50"/>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A48" s="55" t="s">
-        <v>238</v>
-      </c>
-      <c r="B48" s="55">
-        <v>2</v>
-      </c>
-      <c r="C48" s="56" t="s">
-        <v>237</v>
-      </c>
-      <c r="D48" s="55"/>
-      <c r="E48" s="54"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="55"/>
-      <c r="J48" s="54">
-        <f>SUM(J49:J51)</f>
-        <v>402</v>
-      </c>
-      <c r="K48" s="50"/>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" s="52" t="s">
-        <v>236</v>
-      </c>
-      <c r="B49" s="52">
-        <v>3</v>
-      </c>
-      <c r="C49" s="53" t="s">
-        <v>235</v>
-      </c>
-      <c r="D49" s="52">
-        <v>3</v>
-      </c>
-      <c r="E49" s="51">
-        <v>65</v>
-      </c>
-      <c r="F49" s="52" t="s">
-        <v>232</v>
-      </c>
-      <c r="G49" s="57" t="s">
-        <v>180</v>
-      </c>
-      <c r="H49" s="58">
-        <v>46213</v>
-      </c>
-      <c r="I49" s="52"/>
-      <c r="J49" s="51">
-        <f>D49*E49</f>
+      <c r="E69" s="53"/>
+      <c r="F69" s="54"/>
+      <c r="G69" s="54"/>
+      <c r="H69" s="54"/>
+      <c r="I69" s="54"/>
+      <c r="J69" s="53">
+        <f>SUM(J70:J71)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" s="51" t="s">
         <v>195</v>
       </c>
-      <c r="K49" s="50"/>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A50" s="52" t="s">
-        <v>234</v>
-      </c>
-      <c r="B50" s="52">
-        <v>3</v>
-      </c>
-      <c r="C50" s="53" t="s">
-        <v>233</v>
-      </c>
-      <c r="D50" s="52">
-        <v>3</v>
-      </c>
-      <c r="E50" s="51">
-        <v>69</v>
-      </c>
-      <c r="F50" s="52" t="s">
-        <v>232</v>
-      </c>
-      <c r="G50" s="57" t="s">
-        <v>180</v>
-      </c>
-      <c r="H50" s="52"/>
-      <c r="I50" s="52"/>
-      <c r="J50" s="51">
-        <f>D50*E50</f>
-        <v>207</v>
-      </c>
-      <c r="K50" s="50"/>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A51" s="52" t="s">
-        <v>231</v>
-      </c>
-      <c r="B51" s="52">
-        <v>3</v>
-      </c>
-      <c r="C51" s="53" t="s">
-        <v>230</v>
-      </c>
-      <c r="D51" s="52">
-        <v>3</v>
-      </c>
-      <c r="E51" s="51"/>
-      <c r="F51" s="52" t="s">
-        <v>229</v>
-      </c>
-      <c r="G51" s="52"/>
-      <c r="H51" s="52"/>
-      <c r="I51" s="52"/>
-      <c r="J51" s="51"/>
-      <c r="K51" s="50"/>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A52" s="55" t="s">
-        <v>228</v>
-      </c>
-      <c r="B52" s="55">
-        <v>2</v>
-      </c>
-      <c r="C52" s="56" t="s">
-        <v>227</v>
-      </c>
-      <c r="D52" s="55"/>
-      <c r="E52" s="54"/>
-      <c r="F52" s="55"/>
-      <c r="G52" s="55"/>
-      <c r="H52" s="55"/>
-      <c r="I52" s="55"/>
-      <c r="J52" s="54">
-        <f>SUM(J53:J56)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A53" s="52" t="s">
-        <v>226</v>
-      </c>
-      <c r="B53" s="52">
-        <v>3</v>
-      </c>
-      <c r="C53" s="53" t="s">
-        <v>225</v>
-      </c>
-      <c r="D53" s="52"/>
-      <c r="E53" s="51"/>
-      <c r="F53" s="52" t="s">
-        <v>224</v>
-      </c>
-      <c r="G53" s="52"/>
-      <c r="H53" s="52"/>
-      <c r="I53" s="52"/>
-      <c r="J53" s="51"/>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A54" s="52" t="s">
-        <v>223</v>
-      </c>
-      <c r="B54" s="52">
-        <v>3</v>
-      </c>
-      <c r="C54" s="53" t="s">
-        <v>222</v>
-      </c>
-      <c r="D54" s="52"/>
-      <c r="E54" s="51"/>
-      <c r="F54" s="52" t="s">
-        <v>221</v>
-      </c>
-      <c r="G54" s="52"/>
-      <c r="H54" s="52"/>
-      <c r="I54" s="52"/>
-      <c r="J54" s="51"/>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A55" s="52" t="s">
-        <v>220</v>
-      </c>
-      <c r="B55" s="52">
-        <v>3</v>
-      </c>
-      <c r="C55" s="53" t="s">
-        <v>219</v>
-      </c>
-      <c r="D55" s="52"/>
-      <c r="E55" s="51"/>
-      <c r="F55" s="52" t="s">
+      <c r="B70" s="51">
+        <v>3</v>
+      </c>
+      <c r="C70" s="52" t="s">
+        <v>194</v>
+      </c>
+      <c r="D70" s="51"/>
+      <c r="E70" s="50"/>
+      <c r="F70" s="51" t="s">
         <v>191</v>
       </c>
-      <c r="G55" s="52"/>
-      <c r="H55" s="52"/>
-      <c r="I55" s="52"/>
-      <c r="J55" s="51"/>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A56" s="52" t="s">
-        <v>218</v>
-      </c>
-      <c r="B56" s="52">
-        <v>3</v>
-      </c>
-      <c r="C56" s="53" t="s">
-        <v>217</v>
-      </c>
-      <c r="D56" s="52"/>
-      <c r="E56" s="51"/>
-      <c r="F56" s="52" t="s">
-        <v>216</v>
-      </c>
-      <c r="G56" s="52"/>
-      <c r="H56" s="52"/>
-      <c r="I56" s="52"/>
-      <c r="J56" s="51"/>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A57" s="55" t="s">
-        <v>215</v>
-      </c>
-      <c r="B57" s="55">
-        <v>2</v>
-      </c>
-      <c r="C57" s="56" t="s">
-        <v>214</v>
-      </c>
-      <c r="D57" s="55"/>
-      <c r="E57" s="54"/>
-      <c r="F57" s="55"/>
-      <c r="G57" s="55"/>
-      <c r="H57" s="55"/>
-      <c r="I57" s="55"/>
-      <c r="J57" s="54">
-        <f>SUM(J58:J59)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A58" s="52" t="s">
-        <v>213</v>
-      </c>
-      <c r="B58" s="52">
-        <v>3</v>
-      </c>
-      <c r="C58" s="53" t="s">
-        <v>212</v>
-      </c>
-      <c r="D58" s="52"/>
-      <c r="E58" s="51"/>
-      <c r="F58" s="52" t="s">
-        <v>211</v>
-      </c>
-      <c r="G58" s="52"/>
-      <c r="H58" s="52"/>
-      <c r="I58" s="52"/>
-      <c r="J58" s="51"/>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A59" s="52" t="s">
-        <v>210</v>
-      </c>
-      <c r="B59" s="52">
-        <v>3</v>
-      </c>
-      <c r="C59" s="53" t="s">
-        <v>209</v>
-      </c>
-      <c r="D59" s="52"/>
-      <c r="E59" s="51"/>
-      <c r="F59" s="52" t="s">
+      <c r="G70" s="51"/>
+      <c r="H70" s="51"/>
+      <c r="I70" s="51"/>
+      <c r="J70" s="50"/>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" s="51" t="s">
+        <v>193</v>
+      </c>
+      <c r="B71" s="51">
+        <v>3</v>
+      </c>
+      <c r="C71" s="52" t="s">
+        <v>192</v>
+      </c>
+      <c r="D71" s="51"/>
+      <c r="E71" s="50"/>
+      <c r="F71" s="51" t="s">
         <v>191</v>
       </c>
-      <c r="G59" s="52"/>
-      <c r="H59" s="52"/>
-      <c r="I59" s="52"/>
-      <c r="J59" s="51"/>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A60" s="55" t="s">
-        <v>208</v>
-      </c>
-      <c r="B60" s="55">
-        <v>2</v>
-      </c>
-      <c r="C60" s="56" t="s">
-        <v>207</v>
-      </c>
-      <c r="D60" s="55"/>
-      <c r="E60" s="54"/>
-      <c r="F60" s="55"/>
-      <c r="G60" s="55"/>
-      <c r="H60" s="55"/>
-      <c r="I60" s="55"/>
-      <c r="J60" s="54">
-        <f>SUM(J61:J64)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A61" s="52" t="s">
-        <v>206</v>
-      </c>
-      <c r="B61" s="52">
-        <v>3</v>
-      </c>
-      <c r="C61" s="53" t="s">
-        <v>205</v>
-      </c>
-      <c r="D61" s="52"/>
-      <c r="E61" s="51"/>
-      <c r="F61" s="52" t="s">
-        <v>191</v>
-      </c>
-      <c r="G61" s="52"/>
-      <c r="H61" s="52"/>
-      <c r="I61" s="52"/>
-      <c r="J61" s="51"/>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A62" s="52" t="s">
-        <v>204</v>
-      </c>
-      <c r="B62" s="52">
-        <v>3</v>
-      </c>
-      <c r="C62" s="53" t="s">
-        <v>203</v>
-      </c>
-      <c r="D62" s="52">
-        <v>1</v>
-      </c>
-      <c r="E62" s="51"/>
-      <c r="F62" s="52" t="s">
-        <v>202</v>
-      </c>
-      <c r="G62" s="52"/>
-      <c r="H62" s="52"/>
-      <c r="I62" s="52"/>
-      <c r="J62" s="51"/>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A63" s="52" t="s">
-        <v>201</v>
-      </c>
-      <c r="B63" s="52">
-        <v>3</v>
-      </c>
-      <c r="C63" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="D63" s="52"/>
-      <c r="E63" s="51"/>
-      <c r="F63" s="52" t="s">
-        <v>199</v>
-      </c>
-      <c r="G63" s="52"/>
-      <c r="H63" s="52"/>
-      <c r="I63" s="52"/>
-      <c r="J63" s="51"/>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A64" s="52" t="s">
-        <v>198</v>
-      </c>
-      <c r="B64" s="52">
-        <v>3</v>
-      </c>
-      <c r="C64" s="53" t="s">
-        <v>197</v>
-      </c>
-      <c r="D64" s="52"/>
-      <c r="E64" s="51"/>
-      <c r="F64" s="52" t="s">
-        <v>191</v>
-      </c>
-      <c r="G64" s="52"/>
-      <c r="H64" s="52"/>
-      <c r="I64" s="52"/>
-      <c r="J64" s="51"/>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A65" s="55" t="s">
-        <v>196</v>
-      </c>
-      <c r="B65" s="55">
-        <v>2</v>
-      </c>
-      <c r="C65" s="56" t="s">
-        <v>268</v>
-      </c>
-      <c r="D65" s="55">
-        <v>2</v>
-      </c>
-      <c r="E65" s="54"/>
-      <c r="F65" s="55"/>
-      <c r="G65" s="55"/>
-      <c r="H65" s="55"/>
-      <c r="I65" s="55"/>
-      <c r="J65" s="54">
-        <f>SUM(J66:J67)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A66" s="52" t="s">
-        <v>195</v>
-      </c>
-      <c r="B66" s="52">
-        <v>3</v>
-      </c>
-      <c r="C66" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="D66" s="52"/>
-      <c r="E66" s="51"/>
-      <c r="F66" s="52" t="s">
-        <v>191</v>
-      </c>
-      <c r="G66" s="52"/>
-      <c r="H66" s="52"/>
-      <c r="I66" s="52"/>
-      <c r="J66" s="51"/>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A67" s="52" t="s">
-        <v>193</v>
-      </c>
-      <c r="B67" s="52">
-        <v>3</v>
-      </c>
-      <c r="C67" s="53" t="s">
-        <v>192</v>
-      </c>
-      <c r="D67" s="52"/>
-      <c r="E67" s="51"/>
-      <c r="F67" s="52" t="s">
-        <v>191</v>
-      </c>
-      <c r="G67" s="52"/>
-      <c r="H67" s="52"/>
-      <c r="I67" s="52"/>
-      <c r="J67" s="51"/>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F69" s="49" t="s">
+      <c r="G71" s="51"/>
+      <c r="H71" s="51"/>
+      <c r="I71" s="51"/>
+      <c r="J71" s="50"/>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F73" s="48" t="s">
         <v>190</v>
       </c>
-      <c r="G69" s="48"/>
-      <c r="H69" s="48"/>
-      <c r="I69" s="48"/>
-      <c r="J69" s="47">
-        <f>J15+J21+J48+J52+J57+J60+J65</f>
+      <c r="G73" s="47"/>
+      <c r="H73" s="47"/>
+      <c r="I73" s="47"/>
+      <c r="J73" s="46">
+        <f>J15+J21+J52+J56+J61+J64+J69</f>
         <v>1044</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="F35:F47"/>
+    <mergeCell ref="F36:F48"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <hyperlinks>
@@ -4449,8 +4519,8 @@
     <hyperlink ref="G8" r:id="rId4" xr:uid="{60429B27-A38D-454F-B173-6703031A5589}"/>
     <hyperlink ref="G6" r:id="rId5" xr:uid="{0A9A04AE-D73D-4785-8B94-5732DA2EFFEB}"/>
     <hyperlink ref="G4" r:id="rId6" xr:uid="{8965FEC0-8122-4167-90F4-C3780CE3A5C5}"/>
-    <hyperlink ref="G50" r:id="rId7" xr:uid="{8A31F0DB-620C-4B1D-BD14-CB8720C07EC8}"/>
-    <hyperlink ref="G49" r:id="rId8" xr:uid="{9E52DD90-A4C0-4AFB-B727-068C5A377BE2}"/>
+    <hyperlink ref="G54" r:id="rId7" xr:uid="{8A31F0DB-620C-4B1D-BD14-CB8720C07EC8}"/>
+    <hyperlink ref="G53" r:id="rId8" xr:uid="{9E52DD90-A4C0-4AFB-B727-068C5A377BE2}"/>
     <hyperlink ref="G19" r:id="rId9" xr:uid="{8091DB70-558E-4592-B9B4-38004DC7FBB7}"/>
     <hyperlink ref="G18" r:id="rId10" xr:uid="{F7F75BD6-DB10-4AC2-8841-880D0CC3617B}"/>
     <hyperlink ref="G17" r:id="rId11" xr:uid="{279313D3-1F5C-43AF-9B3D-757C7867AE3E}"/>

</xml_diff>

<commit_message>
Finished Bom. Ordering parts soon
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F291CAE-C194-4E3B-A39C-93DFF63A0A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A41B23B-C013-4DCA-B9FB-FCE87148EAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="323">
   <si>
     <t>6-DoF Arm — Gravity Torque Budget v2 (elbow-mounted forearm roll)</t>
   </si>
@@ -589,9 +589,6 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>s</t>
-  </si>
-  <si>
     <t>Price per Unit</t>
   </si>
   <si>
@@ -835,12 +832,6 @@
     <t>1.1</t>
   </si>
   <si>
-    <t>Order Notes</t>
-  </si>
-  <si>
-    <t>Ext. Cost</t>
-  </si>
-  <si>
     <t>6-DoF Robotic Arm</t>
   </si>
   <si>
@@ -883,12 +874,6 @@
     <t>M3 Screw</t>
   </si>
   <si>
-    <t>M5x0.8 x 13mm length (Cap Head)</t>
-  </si>
-  <si>
-    <t>M3 x ___mm length (Cap Head)</t>
-  </si>
-  <si>
     <t>1.2.14</t>
   </si>
   <si>
@@ -964,9 +949,6 @@
     <t>Hex Shaft</t>
   </si>
   <si>
-    <t>5mm x 51mm</t>
-  </si>
-  <si>
     <t>Price/Pack</t>
   </si>
   <si>
@@ -989,6 +971,42 @@
   </si>
   <si>
     <t>M5x0.8 around 64mm in total length (4 pcs)</t>
+  </si>
+  <si>
+    <t>M2.5 Screw</t>
+  </si>
+  <si>
+    <t>1.2.24</t>
+  </si>
+  <si>
+    <t>1.2.25</t>
+  </si>
+  <si>
+    <t>5mm x 51mm (4 pcs 400mm in length each)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3 x 4mm length </t>
+  </si>
+  <si>
+    <t>M5x0.8 x 13mm length</t>
+  </si>
+  <si>
+    <t>Already Have</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2.5 x 4mm length </t>
+  </si>
+  <si>
+    <t>Shipping</t>
+  </si>
+  <si>
+    <t>Total Cost</t>
+  </si>
+  <si>
+    <t>M2.5 Set Screw</t>
+  </si>
+  <si>
+    <t>M2.5 x 4mm length (50 pieces)</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +1019,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1100,6 +1118,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="12">
@@ -1277,7 +1308,7 @@
     <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1430,6 +1461,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1439,17 +1473,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1768,17 +1812,17 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="69"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -1846,17 +1890,17 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="68" t="s">
+      <c r="A11" s="69" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="68"/>
-      <c r="C11" s="68"/>
-      <c r="D11" s="68"/>
-      <c r="E11" s="68"/>
-      <c r="F11" s="68"/>
-      <c r="G11" s="68"/>
-      <c r="H11" s="68"/>
-      <c r="I11" s="68"/>
+      <c r="B11" s="69"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="69"/>
+      <c r="I11" s="69"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -1954,17 +1998,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="68" t="s">
+      <c r="A20" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="68"/>
-      <c r="C20" s="68"/>
-      <c r="D20" s="68"/>
-      <c r="E20" s="68"/>
-      <c r="F20" s="68"/>
-      <c r="G20" s="68"/>
-      <c r="H20" s="68"/>
-      <c r="I20" s="68"/>
+      <c r="B20" s="69"/>
+      <c r="C20" s="69"/>
+      <c r="D20" s="69"/>
+      <c r="E20" s="69"/>
+      <c r="F20" s="69"/>
+      <c r="G20" s="69"/>
+      <c r="H20" s="69"/>
+      <c r="I20" s="69"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
@@ -1989,17 +2033,17 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="68" t="s">
+      <c r="A24" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="68"/>
-      <c r="C24" s="68"/>
-      <c r="D24" s="68"/>
-      <c r="E24" s="68"/>
-      <c r="F24" s="68"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="68"/>
-      <c r="I24" s="68"/>
+      <c r="B24" s="69"/>
+      <c r="C24" s="69"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="69"/>
+      <c r="F24" s="69"/>
+      <c r="G24" s="69"/>
+      <c r="H24" s="69"/>
+      <c r="I24" s="69"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
@@ -2139,17 +2183,17 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="68" t="s">
+      <c r="A36" s="69" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="68"/>
-      <c r="C36" s="68"/>
-      <c r="D36" s="68"/>
-      <c r="E36" s="68"/>
-      <c r="F36" s="68"/>
-      <c r="G36" s="68"/>
-      <c r="H36" s="68"/>
-      <c r="I36" s="68"/>
+      <c r="B36" s="69"/>
+      <c r="C36" s="69"/>
+      <c r="D36" s="69"/>
+      <c r="E36" s="69"/>
+      <c r="F36" s="69"/>
+      <c r="G36" s="69"/>
+      <c r="H36" s="69"/>
+      <c r="I36" s="69"/>
     </row>
     <row r="37" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
@@ -2360,17 +2404,17 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="68" t="s">
+      <c r="A47" s="69" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="68"/>
-      <c r="C47" s="68"/>
-      <c r="D47" s="68"/>
-      <c r="E47" s="68"/>
-      <c r="F47" s="68"/>
-      <c r="G47" s="68"/>
-      <c r="H47" s="68"/>
-      <c r="I47" s="68"/>
+      <c r="B47" s="69"/>
+      <c r="C47" s="69"/>
+      <c r="D47" s="69"/>
+      <c r="E47" s="69"/>
+      <c r="F47" s="69"/>
+      <c r="G47" s="69"/>
+      <c r="H47" s="69"/>
+      <c r="I47" s="69"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
@@ -2403,17 +2447,17 @@
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="68" t="s">
+      <c r="A52" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="68"/>
-      <c r="C52" s="68"/>
-      <c r="D52" s="68"/>
-      <c r="E52" s="68"/>
-      <c r="F52" s="68"/>
-      <c r="G52" s="68"/>
-      <c r="H52" s="68"/>
-      <c r="I52" s="68"/>
+      <c r="B52" s="69"/>
+      <c r="C52" s="69"/>
+      <c r="D52" s="69"/>
+      <c r="E52" s="69"/>
+      <c r="F52" s="69"/>
+      <c r="G52" s="69"/>
+      <c r="H52" s="69"/>
+      <c r="I52" s="69"/>
     </row>
     <row r="53" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
@@ -2964,7 +3008,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03C3DC63-880C-4C7A-BD99-15B2870A7881}">
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:Q73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
@@ -2974,14 +3018,14 @@
     <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="66.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="31" t="s">
         <v>102</v>
       </c>
@@ -2995,7 +3039,7 @@
         <v>168</v>
       </c>
       <c r="E1" s="31" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F1" s="31" t="s">
         <v>171</v>
@@ -3004,13 +3048,13 @@
         <v>176</v>
       </c>
       <c r="H1" s="35" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I1" s="35" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="36">
         <v>1</v>
       </c>
@@ -3035,7 +3079,7 @@
       <c r="H2" s="45"/>
       <c r="I2" s="45"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="39">
         <v>2</v>
       </c>
@@ -3061,13 +3105,13 @@
         <v>46213</v>
       </c>
       <c r="I3" s="42" t="s">
+        <v>185</v>
+      </c>
+      <c r="K3" t="s">
         <v>186</v>
       </c>
-      <c r="K3" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="36">
         <v>3</v>
       </c>
@@ -3092,7 +3136,7 @@
       <c r="H4" s="36"/>
       <c r="I4" s="36"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="39">
         <v>4</v>
       </c>
@@ -3117,7 +3161,7 @@
       <c r="H5" s="34"/>
       <c r="I5" s="42"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="36">
         <v>5</v>
       </c>
@@ -3144,7 +3188,7 @@
       </c>
       <c r="I6" s="44"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="39"/>
       <c r="B7" s="39"/>
       <c r="C7" s="39"/>
@@ -3155,7 +3199,7 @@
       <c r="H7" s="34"/>
       <c r="I7" s="42"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="36">
         <v>6</v>
       </c>
@@ -3182,10 +3226,10 @@
       </c>
       <c r="I8" s="44"/>
       <c r="K8" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="34"/>
       <c r="B9" s="42"/>
       <c r="C9" s="42"/>
@@ -3196,7 +3240,7 @@
       <c r="H9" s="42"/>
       <c r="I9" s="42"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F10" s="32" t="s">
         <v>181</v>
       </c>
@@ -3205,7 +3249,7 @@
         <v>1044</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="62" t="s">
         <v>102</v>
       </c>
@@ -3219,31 +3263,28 @@
         <v>168</v>
       </c>
       <c r="E13" s="62" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F13" s="62" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="G13" s="62" t="s">
         <v>176</v>
       </c>
       <c r="H13" s="62" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I13" s="62" t="s">
-        <v>189</v>
-      </c>
-      <c r="J13" s="62" t="s">
-        <v>266</v>
-      </c>
-      <c r="K13" s="62" t="s">
-        <v>265</v>
-      </c>
-      <c r="N13" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+      <c r="J13" s="76" t="s">
+        <v>319</v>
+      </c>
+      <c r="K13" s="76" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="60" t="s">
         <v>108</v>
       </c>
@@ -3251,7 +3292,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="61" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D14" s="60"/>
       <c r="E14" s="59"/>
@@ -3260,17 +3301,17 @@
       <c r="H14" s="60"/>
       <c r="I14" s="60"/>
       <c r="J14" s="59"/>
-      <c r="K14" s="49"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K14" s="59"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="54" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B15" s="54">
         <v>2</v>
       </c>
       <c r="C15" s="55" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D15" s="54"/>
       <c r="E15" s="53"/>
@@ -3278,15 +3319,15 @@
       <c r="G15" s="54"/>
       <c r="H15" s="58"/>
       <c r="I15" s="54"/>
-      <c r="J15" s="53">
-        <f>SUM(J16:J20)</f>
+      <c r="J15" s="53"/>
+      <c r="K15" s="53">
+        <f>SUM(K16:K20)</f>
         <v>642</v>
       </c>
-      <c r="K15" s="49"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="51" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B16" s="51">
         <v>3</v>
@@ -3301,22 +3342,22 @@
         <v>74</v>
       </c>
       <c r="F16" s="51" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G16" s="56" t="s">
         <v>180</v>
       </c>
       <c r="H16" s="51"/>
       <c r="I16" s="51"/>
-      <c r="J16" s="50">
+      <c r="J16" s="50"/>
+      <c r="K16" s="50">
         <f>D16*E16</f>
         <v>148</v>
       </c>
-      <c r="K16" s="49"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="51" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B17" s="51">
         <v>3</v>
@@ -3331,22 +3372,22 @@
         <v>94</v>
       </c>
       <c r="F17" s="51" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G17" s="56" t="s">
         <v>180</v>
       </c>
       <c r="H17" s="51"/>
       <c r="I17" s="51"/>
-      <c r="J17" s="50">
+      <c r="J17" s="50"/>
+      <c r="K17" s="50">
         <f>D17*E17</f>
         <v>188</v>
       </c>
-      <c r="K17" s="49"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="51" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B18" s="51">
         <v>3</v>
@@ -3361,7 +3402,7 @@
         <v>219</v>
       </c>
       <c r="F18" s="51" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G18" s="56" t="s">
         <v>180</v>
@@ -3370,15 +3411,15 @@
         <v>46213</v>
       </c>
       <c r="I18" s="57"/>
-      <c r="J18" s="50">
+      <c r="J18" s="50"/>
+      <c r="K18" s="50">
         <f>D18*E18</f>
         <v>219</v>
       </c>
-      <c r="K18" s="49"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="51" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B19" s="51">
         <v>3</v>
@@ -3393,7 +3434,7 @@
         <v>29</v>
       </c>
       <c r="F19" s="51" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G19" s="56" t="s">
         <v>180</v>
@@ -3402,74 +3443,74 @@
         <v>46213</v>
       </c>
       <c r="I19" s="51" t="s">
-        <v>254</v>
-      </c>
-      <c r="J19" s="50">
+        <v>253</v>
+      </c>
+      <c r="J19" s="50" t="s">
+        <v>186</v>
+      </c>
+      <c r="K19" s="50">
         <f>D19*E19</f>
         <v>87</v>
       </c>
-      <c r="K19" s="49" t="s">
-        <v>187</v>
-      </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="51" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B20" s="51">
         <v>3</v>
       </c>
       <c r="C20" s="52" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D20" s="51">
         <v>2</v>
       </c>
       <c r="E20" s="50"/>
       <c r="F20" s="51" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G20" s="51"/>
       <c r="H20" s="57"/>
       <c r="I20" s="57"/>
       <c r="J20" s="50"/>
-      <c r="K20" s="49"/>
+      <c r="K20" s="50"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="54" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B21" s="54">
         <v>2</v>
       </c>
       <c r="C21" s="55" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D21" s="54">
         <v>1</v>
       </c>
       <c r="E21" s="53" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="F21" s="54"/>
       <c r="G21" s="54"/>
       <c r="H21" s="54"/>
       <c r="I21" s="54"/>
-      <c r="J21" s="53">
-        <f>SUM(J22:J31)</f>
+      <c r="J21" s="53"/>
+      <c r="K21" s="53">
+        <f>SUM(K22:K31)</f>
         <v>0</v>
       </c>
-      <c r="K21" s="49"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="51" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B22" s="51">
         <v>3</v>
       </c>
       <c r="C22" s="52" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D22" s="51">
         <v>39</v>
@@ -3478,7 +3519,7 @@
         <v>7.21</v>
       </c>
       <c r="F22" s="51" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="G22" s="63" t="s">
         <v>180</v>
@@ -3486,7 +3527,7 @@
       <c r="H22" s="51"/>
       <c r="I22" s="51"/>
       <c r="J22" s="50"/>
-      <c r="K22" s="49"/>
+      <c r="K22" s="50"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="51"/>
@@ -3499,17 +3540,17 @@
       <c r="H23" s="57"/>
       <c r="I23" s="51"/>
       <c r="J23" s="50"/>
-      <c r="K23" s="49"/>
+      <c r="K23" s="50"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="51" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B24" s="51">
         <v>3</v>
       </c>
       <c r="C24" s="52" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D24" s="51">
         <v>78</v>
@@ -3518,7 +3559,7 @@
         <v>12.99</v>
       </c>
       <c r="F24" s="51" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="G24" s="64" t="s">
         <v>180</v>
@@ -3526,17 +3567,17 @@
       <c r="H24" s="51"/>
       <c r="I24" s="51"/>
       <c r="J24" s="50"/>
-      <c r="K24" s="49"/>
+      <c r="K24" s="50"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="51" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B25" s="51">
         <v>3</v>
       </c>
       <c r="C25" s="52" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D25" s="51">
         <v>4</v>
@@ -3545,7 +3586,7 @@
         <v>9.99</v>
       </c>
       <c r="F25" s="51" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="G25" s="64" t="s">
         <v>180</v>
@@ -3553,17 +3594,17 @@
       <c r="H25" s="51"/>
       <c r="I25" s="51"/>
       <c r="J25" s="50"/>
-      <c r="K25" s="49"/>
+      <c r="K25" s="50"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="51" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B26" s="51">
         <v>3</v>
       </c>
       <c r="C26" s="52" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D26" s="51">
         <v>2</v>
@@ -3572,7 +3613,7 @@
         <v>9.7899999999999991</v>
       </c>
       <c r="F26" s="51" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="G26" s="64" t="s">
         <v>180</v>
@@ -3580,7 +3621,7 @@
       <c r="H26" s="51"/>
       <c r="I26" s="51"/>
       <c r="J26" s="50"/>
-      <c r="K26" s="49"/>
+      <c r="K26" s="50"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="51"/>
@@ -3593,17 +3634,17 @@
       <c r="H27" s="51"/>
       <c r="I27" s="51"/>
       <c r="J27" s="50"/>
-      <c r="K27" s="49"/>
+      <c r="K27" s="50"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="51" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B28" s="51">
         <v>3</v>
       </c>
       <c r="C28" s="52" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D28" s="51">
         <v>15</v>
@@ -3612,7 +3653,7 @@
         <v>6.99</v>
       </c>
       <c r="F28" s="51" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="G28" s="64" t="s">
         <v>180</v>
@@ -3620,17 +3661,17 @@
       <c r="H28" s="51"/>
       <c r="I28" s="51"/>
       <c r="J28" s="50"/>
-      <c r="K28" s="49"/>
+      <c r="K28" s="50"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="51" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B29" s="51">
         <v>3</v>
       </c>
       <c r="C29" s="52" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D29" s="51">
         <v>5</v>
@@ -3639,7 +3680,7 @@
         <v>8.99</v>
       </c>
       <c r="F29" s="51" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="G29" s="64" t="s">
         <v>180</v>
@@ -3647,11 +3688,11 @@
       <c r="H29" s="51"/>
       <c r="I29" s="51"/>
       <c r="J29" s="50"/>
-      <c r="K29" s="49"/>
+      <c r="K29" s="50"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="51" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B30" s="51"/>
       <c r="C30" s="52"/>
@@ -3662,17 +3703,17 @@
       <c r="H30" s="51"/>
       <c r="I30" s="51"/>
       <c r="J30" s="50"/>
-      <c r="K30" s="49"/>
+      <c r="K30" s="50"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="51" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B31" s="51">
         <v>3</v>
       </c>
       <c r="C31" s="52" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D31" s="51">
         <v>6</v>
@@ -3681,7 +3722,7 @@
         <v>7.79</v>
       </c>
       <c r="F31" s="51" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="G31" s="64" t="s">
         <v>180</v>
@@ -3689,355 +3730,374 @@
       <c r="H31" s="51"/>
       <c r="I31" s="51"/>
       <c r="J31" s="50"/>
-      <c r="K31" s="49"/>
+      <c r="K31" s="50"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="51" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B32" s="51">
         <v>3</v>
       </c>
       <c r="C32" s="52" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D32" s="51">
-        <v>3</v>
-      </c>
-      <c r="E32" s="50"/>
-      <c r="F32" s="51" t="s">
-        <v>281</v>
-      </c>
-      <c r="G32" s="51"/>
-      <c r="H32" s="51"/>
-      <c r="I32" s="51"/>
+        <v>9</v>
+      </c>
+      <c r="E32" s="73">
+        <v>22.99</v>
+      </c>
+      <c r="F32" s="70" t="s">
+        <v>316</v>
+      </c>
+      <c r="G32" s="71" t="s">
+        <v>180</v>
+      </c>
+      <c r="H32" s="66"/>
+      <c r="I32" s="66"/>
       <c r="J32" s="50"/>
-      <c r="K32" s="49"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K32" s="50"/>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="51" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B33" s="51">
         <v>3</v>
       </c>
       <c r="C33" s="52" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D33" s="51">
         <v>7</v>
       </c>
-      <c r="E33" s="50"/>
-      <c r="F33" s="51" t="s">
-        <v>282</v>
-      </c>
-      <c r="G33" s="51"/>
-      <c r="H33" s="51"/>
-      <c r="I33" s="51"/>
+      <c r="E33" s="74"/>
+      <c r="F33" s="70" t="s">
+        <v>315</v>
+      </c>
+      <c r="G33" s="72"/>
+      <c r="H33" s="68"/>
+      <c r="I33" s="68"/>
       <c r="J33" s="50"/>
-      <c r="K33" s="49" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K33" s="50"/>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="51" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="B34" s="51">
         <v>3</v>
       </c>
       <c r="C34" s="52" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="D34" s="51">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E34" s="50"/>
-      <c r="F34" s="51" t="s">
-        <v>308</v>
+      <c r="F34" s="70" t="s">
+        <v>318</v>
       </c>
       <c r="G34" s="51"/>
-      <c r="H34" s="51"/>
+      <c r="H34" s="70" t="s">
+        <v>317</v>
+      </c>
       <c r="I34" s="51"/>
       <c r="J34" s="50"/>
-      <c r="K34" s="49"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="51"/>
-      <c r="B35" s="51"/>
-      <c r="C35" s="52"/>
-      <c r="D35" s="51"/>
-      <c r="E35" s="50"/>
-      <c r="F35" s="69"/>
-      <c r="G35" s="51"/>
-      <c r="H35" s="51"/>
+      <c r="K34" s="50"/>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A35" s="51" t="s">
+        <v>275</v>
+      </c>
+      <c r="B35" s="51">
+        <v>3</v>
+      </c>
+      <c r="C35" s="77" t="s">
+        <v>321</v>
+      </c>
+      <c r="D35" s="51">
+        <v>1</v>
+      </c>
+      <c r="E35" s="50">
+        <v>7.29</v>
+      </c>
+      <c r="F35" s="70" t="s">
+        <v>322</v>
+      </c>
+      <c r="G35" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="H35" s="70"/>
       <c r="I35" s="51"/>
       <c r="J35" s="50"/>
-      <c r="K35" s="49"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K35" s="50"/>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="51" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B36" s="51">
         <v>3</v>
       </c>
       <c r="C36" s="52" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="D36" s="51">
         <v>1</v>
       </c>
-      <c r="E36" s="50"/>
-      <c r="F36" s="65" t="s">
-        <v>305</v>
-      </c>
-      <c r="G36" s="51"/>
-      <c r="H36" s="51"/>
+      <c r="E36" s="50">
+        <v>21.45</v>
+      </c>
+      <c r="F36" s="70" t="s">
+        <v>314</v>
+      </c>
+      <c r="G36" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="H36" s="70" t="s">
+        <v>317</v>
+      </c>
       <c r="I36" s="51"/>
       <c r="J36" s="50"/>
-      <c r="K36" s="49"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" s="51" t="s">
-        <v>278</v>
-      </c>
-      <c r="B37" s="51">
-        <v>3</v>
-      </c>
-      <c r="C37" s="52" t="s">
-        <v>293</v>
-      </c>
-      <c r="D37" s="51">
-        <v>1</v>
-      </c>
+      <c r="K36" s="50"/>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A37" s="51"/>
+      <c r="B37" s="51"/>
+      <c r="C37" s="52"/>
+      <c r="D37" s="51"/>
       <c r="E37" s="50"/>
-      <c r="F37" s="66"/>
+      <c r="F37" s="65"/>
       <c r="G37" s="51"/>
       <c r="H37" s="51"/>
       <c r="I37" s="51"/>
       <c r="J37" s="50"/>
-      <c r="K37" s="49"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K37" s="50"/>
+      <c r="Q37" s="75"/>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="51" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="B38" s="51">
         <v>3</v>
       </c>
       <c r="C38" s="52" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D38" s="51">
-        <v>78</v>
+        <v>1</v>
       </c>
       <c r="E38" s="50"/>
-      <c r="F38" s="66"/>
+      <c r="F38" s="66" t="s">
+        <v>300</v>
+      </c>
       <c r="G38" s="51"/>
       <c r="H38" s="51"/>
       <c r="I38" s="51"/>
       <c r="J38" s="50"/>
-      <c r="K38" s="49"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K38" s="50"/>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="51" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="B39" s="51">
         <v>3</v>
       </c>
       <c r="C39" s="52" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="D39" s="51">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="E39" s="50"/>
-      <c r="F39" s="66"/>
+      <c r="F39" s="67"/>
       <c r="G39" s="51"/>
       <c r="H39" s="51"/>
       <c r="I39" s="51"/>
       <c r="J39" s="50"/>
-      <c r="K39" s="49"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K39" s="50"/>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="51" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="B40" s="51">
         <v>3</v>
       </c>
       <c r="C40" s="52" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="D40" s="51">
-        <v>2</v>
+        <v>78</v>
       </c>
       <c r="E40" s="50"/>
-      <c r="F40" s="66"/>
+      <c r="F40" s="67"/>
       <c r="G40" s="51"/>
       <c r="H40" s="51"/>
       <c r="I40" s="51"/>
       <c r="J40" s="50"/>
-      <c r="K40" s="49"/>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K40" s="50"/>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="51" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="B41" s="51">
         <v>3</v>
       </c>
       <c r="C41" s="52" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="D41" s="51">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="E41" s="50"/>
-      <c r="F41" s="66"/>
+      <c r="F41" s="67"/>
       <c r="G41" s="51"/>
       <c r="H41" s="51"/>
       <c r="I41" s="51"/>
       <c r="J41" s="50"/>
-      <c r="K41" s="49"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K41" s="50"/>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="51" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="B42" s="51">
         <v>3</v>
       </c>
       <c r="C42" s="52" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="D42" s="51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42" s="50"/>
-      <c r="F42" s="66"/>
+      <c r="F42" s="67"/>
       <c r="G42" s="51"/>
       <c r="H42" s="51"/>
       <c r="I42" s="51"/>
       <c r="J42" s="50"/>
-      <c r="K42" s="49"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K42" s="50"/>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="51" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="B43" s="51">
         <v>3</v>
       </c>
       <c r="C43" s="52" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="D43" s="51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E43" s="50"/>
-      <c r="F43" s="66"/>
+      <c r="F43" s="67"/>
       <c r="G43" s="51"/>
       <c r="H43" s="51"/>
       <c r="I43" s="51"/>
       <c r="J43" s="50"/>
-      <c r="K43" s="49"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K43" s="50"/>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="51" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B44" s="51">
         <v>3</v>
       </c>
       <c r="C44" s="52" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="D44" s="51">
         <v>1</v>
       </c>
       <c r="E44" s="50"/>
-      <c r="F44" s="66"/>
+      <c r="F44" s="67"/>
       <c r="G44" s="51"/>
       <c r="H44" s="51"/>
       <c r="I44" s="51"/>
       <c r="J44" s="50"/>
-      <c r="K44" s="49"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K44" s="50"/>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="51" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="B45" s="51">
         <v>3</v>
       </c>
       <c r="C45" s="52" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="D45" s="51">
         <v>1</v>
       </c>
       <c r="E45" s="50"/>
-      <c r="F45" s="66"/>
+      <c r="F45" s="67"/>
       <c r="G45" s="51"/>
       <c r="H45" s="51"/>
       <c r="I45" s="51"/>
       <c r="J45" s="50"/>
-      <c r="K45" s="49"/>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K45" s="50"/>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="51" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="B46" s="51">
         <v>3</v>
       </c>
       <c r="C46" s="52" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="D46" s="51">
         <v>1</v>
       </c>
       <c r="E46" s="50"/>
-      <c r="F46" s="66"/>
+      <c r="F46" s="67"/>
       <c r="G46" s="51"/>
       <c r="H46" s="51"/>
       <c r="I46" s="51"/>
       <c r="J46" s="50"/>
-      <c r="K46" s="49"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K46" s="50"/>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="51" t="s">
+        <v>293</v>
+      </c>
+      <c r="B47" s="51">
+        <v>3</v>
+      </c>
+      <c r="C47" s="52" t="s">
         <v>298</v>
-      </c>
-      <c r="B47" s="51">
-        <v>3</v>
-      </c>
-      <c r="C47" s="52" t="s">
-        <v>304</v>
       </c>
       <c r="D47" s="51">
         <v>1</v>
       </c>
       <c r="E47" s="50"/>
-      <c r="F47" s="66"/>
+      <c r="F47" s="67"/>
       <c r="G47" s="51"/>
       <c r="H47" s="51"/>
       <c r="I47" s="51"/>
       <c r="J47" s="50"/>
-      <c r="K47" s="49"/>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K47" s="50"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="51" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="B48" s="51">
         <v>3</v>
       </c>
       <c r="C48" s="52" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="D48" s="51">
         <v>1</v>
@@ -4048,31 +4108,63 @@
       <c r="H48" s="51"/>
       <c r="I48" s="51"/>
       <c r="J48" s="50"/>
-      <c r="K48" s="49"/>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" s="70"/>
-      <c r="B49" s="70"/>
-      <c r="C49" s="71"/>
-      <c r="D49" s="70"/>
-      <c r="E49" s="72"/>
-      <c r="K49" s="49"/>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="K50" s="49"/>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K48" s="50"/>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A49" s="51" t="s">
+        <v>312</v>
+      </c>
+      <c r="B49" s="51">
+        <v>3</v>
+      </c>
+      <c r="C49" s="52" t="s">
+        <v>299</v>
+      </c>
+      <c r="D49" s="51">
+        <v>1</v>
+      </c>
+      <c r="E49" s="50"/>
+      <c r="F49" s="67"/>
+      <c r="G49" s="51"/>
+      <c r="H49" s="51"/>
+      <c r="I49" s="51"/>
+      <c r="J49" s="50"/>
+      <c r="K49" s="50"/>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A50" s="51" t="s">
+        <v>313</v>
+      </c>
+      <c r="B50" s="51">
+        <v>3</v>
+      </c>
+      <c r="C50" s="52" t="s">
+        <v>301</v>
+      </c>
+      <c r="D50" s="51">
+        <v>1</v>
+      </c>
+      <c r="E50" s="50"/>
+      <c r="F50" s="68"/>
+      <c r="G50" s="51"/>
+      <c r="H50" s="51"/>
+      <c r="I50" s="51"/>
+      <c r="J50" s="50"/>
+      <c r="K50" s="50"/>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="K51" s="49"/>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="Q51" s="49"/>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="54" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B52" s="54">
         <v>2</v>
       </c>
       <c r="C52" s="55" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D52" s="54"/>
       <c r="E52" s="53"/>
@@ -4085,15 +4177,15 @@
         <v>402</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="51" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B53" s="51">
         <v>3</v>
       </c>
       <c r="C53" s="52" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D53" s="51">
         <v>3</v>
@@ -4102,7 +4194,7 @@
         <v>65</v>
       </c>
       <c r="F53" s="51" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G53" s="56" t="s">
         <v>180</v>
@@ -4110,21 +4202,23 @@
       <c r="H53" s="57">
         <v>46213</v>
       </c>
-      <c r="I53" s="51"/>
+      <c r="I53" s="51" t="s">
+        <v>187</v>
+      </c>
       <c r="J53" s="50">
         <f>D53*E53</f>
         <v>195</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="51" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B54" s="51">
         <v>3</v>
       </c>
       <c r="C54" s="52" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D54" s="51">
         <v>3</v>
@@ -4133,7 +4227,7 @@
         <v>69</v>
       </c>
       <c r="F54" s="51" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G54" s="56" t="s">
         <v>180</v>
@@ -4145,37 +4239,37 @@
         <v>207</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="51" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B55" s="51">
         <v>3</v>
       </c>
       <c r="C55" s="52" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D55" s="51">
         <v>3</v>
       </c>
       <c r="E55" s="50"/>
       <c r="F55" s="51" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G55" s="51"/>
       <c r="H55" s="51"/>
       <c r="I55" s="51"/>
       <c r="J55" s="50"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="54" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B56" s="54">
         <v>2</v>
       </c>
       <c r="C56" s="55" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D56" s="54"/>
       <c r="E56" s="53"/>
@@ -4188,95 +4282,95 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="51" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B57" s="51">
         <v>3</v>
       </c>
       <c r="C57" s="52" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D57" s="51"/>
       <c r="E57" s="50"/>
       <c r="F57" s="51" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G57" s="51"/>
       <c r="H57" s="51"/>
       <c r="I57" s="51"/>
       <c r="J57" s="50"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="51" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B58" s="51">
         <v>3</v>
       </c>
       <c r="C58" s="52" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D58" s="51"/>
       <c r="E58" s="50"/>
       <c r="F58" s="51" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G58" s="51"/>
       <c r="H58" s="51"/>
       <c r="I58" s="51"/>
       <c r="J58" s="50"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="51" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B59" s="51">
         <v>3</v>
       </c>
       <c r="C59" s="52" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D59" s="51"/>
       <c r="E59" s="50"/>
       <c r="F59" s="51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G59" s="51"/>
       <c r="H59" s="51"/>
       <c r="I59" s="51"/>
       <c r="J59" s="50"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="51" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B60" s="51">
         <v>3</v>
       </c>
       <c r="C60" s="52" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D60" s="51"/>
       <c r="E60" s="50"/>
       <c r="F60" s="51" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G60" s="51"/>
       <c r="H60" s="51"/>
       <c r="I60" s="51"/>
       <c r="J60" s="50"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="54" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B61" s="54">
         <v>2</v>
       </c>
       <c r="C61" s="55" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D61" s="54"/>
       <c r="E61" s="53"/>
@@ -4289,55 +4383,55 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="51" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B62" s="51">
         <v>3</v>
       </c>
       <c r="C62" s="52" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D62" s="51"/>
       <c r="E62" s="50"/>
       <c r="F62" s="51" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G62" s="51"/>
       <c r="H62" s="51"/>
       <c r="I62" s="51"/>
       <c r="J62" s="50"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="51" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B63" s="51">
         <v>3</v>
       </c>
       <c r="C63" s="52" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D63" s="51"/>
       <c r="E63" s="50"/>
       <c r="F63" s="51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G63" s="51"/>
       <c r="H63" s="51"/>
       <c r="I63" s="51"/>
       <c r="J63" s="50"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="54" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B64" s="54">
         <v>2</v>
       </c>
       <c r="C64" s="55" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D64" s="54"/>
       <c r="E64" s="53"/>
@@ -4352,18 +4446,18 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="51" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B65" s="51">
         <v>3</v>
       </c>
       <c r="C65" s="52" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D65" s="51"/>
       <c r="E65" s="50"/>
       <c r="F65" s="51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G65" s="51"/>
       <c r="H65" s="51"/>
@@ -4372,20 +4466,20 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="51" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B66" s="51">
         <v>3</v>
       </c>
       <c r="C66" s="52" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D66" s="51">
         <v>1</v>
       </c>
       <c r="E66" s="50"/>
       <c r="F66" s="51" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G66" s="51"/>
       <c r="H66" s="51"/>
@@ -4394,18 +4488,18 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="51" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B67" s="51">
         <v>3</v>
       </c>
       <c r="C67" s="52" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D67" s="51"/>
       <c r="E67" s="50"/>
       <c r="F67" s="51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G67" s="51"/>
       <c r="H67" s="51"/>
@@ -4414,18 +4508,18 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B68" s="51">
         <v>3</v>
       </c>
       <c r="C68" s="52" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D68" s="51"/>
       <c r="E68" s="50"/>
       <c r="F68" s="51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G68" s="51"/>
       <c r="H68" s="51"/>
@@ -4434,13 +4528,13 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="54" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B69" s="54">
         <v>2</v>
       </c>
       <c r="C69" s="55" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D69" s="54">
         <v>2</v>
@@ -4457,18 +4551,18 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="51" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B70" s="51">
         <v>3</v>
       </c>
       <c r="C70" s="52" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D70" s="51"/>
       <c r="E70" s="50"/>
       <c r="F70" s="51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G70" s="51"/>
       <c r="H70" s="51"/>
@@ -4477,18 +4571,18 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="51" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B71" s="51">
         <v>3</v>
       </c>
       <c r="C71" s="52" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D71" s="51"/>
       <c r="E71" s="50"/>
       <c r="F71" s="51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G71" s="51"/>
       <c r="H71" s="51"/>
@@ -4497,19 +4591,23 @@
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F73" s="48" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G73" s="47"/>
       <c r="H73" s="47"/>
       <c r="I73" s="47"/>
       <c r="J73" s="46">
-        <f>J15+J21+J52+J56+J61+J64+J69</f>
+        <f>K15+K21+J52+J56+J61+J64+J69</f>
         <v>1044</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="F36:F48"/>
+  <mergeCells count="5">
+    <mergeCell ref="I32:I33"/>
+    <mergeCell ref="F38:F50"/>
+    <mergeCell ref="G32:G33"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="H32:H33"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <hyperlinks>
@@ -4532,6 +4630,9 @@
     <hyperlink ref="G28" r:id="rId17" xr:uid="{490592CB-759D-43DE-B1A2-208282D5996C}"/>
     <hyperlink ref="G29" r:id="rId18" xr:uid="{5DF8CFDD-7940-473E-A87F-DADA18BF04F0}"/>
     <hyperlink ref="G31" r:id="rId19" xr:uid="{1412C55E-6A1A-4053-A18E-D6A0EE5D9AF0}"/>
+    <hyperlink ref="G36" r:id="rId20" xr:uid="{DEBF1BA2-46DF-49AD-9E35-D39C010E82A9}"/>
+    <hyperlink ref="G32:G33" r:id="rId21" display="Here" xr:uid="{1C078BBA-02DB-42FD-A3D4-817F8269DFFD}"/>
+    <hyperlink ref="G35" r:id="rId22" xr:uid="{71953ECA-F332-45BA-A578-4C4B7FEF587E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Start of 15:1 cycloidal gearbox
something is wrong with my assembly of the 15:1 cycloidal gearbox. The outer roller pins don't seem to match up with the cycloidal disks causing interferences.
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A41B23B-C013-4DCA-B9FB-FCE87148EAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C720699E-F331-41C9-9D49-56EFBDC42975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="323">
   <si>
     <t>6-DoF Arm — Gravity Torque Budget v2 (elbow-mounted forearm roll)</t>
   </si>
@@ -1463,29 +1463,7 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1495,6 +1473,28 @@
     <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1812,17 +1812,17 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="69" t="s">
+      <c r="A4" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
-      <c r="D4" s="69"/>
-      <c r="E4" s="69"/>
-      <c r="F4" s="69"/>
-      <c r="G4" s="69"/>
-      <c r="H4" s="69"/>
-      <c r="I4" s="69"/>
+      <c r="B4" s="77"/>
+      <c r="C4" s="77"/>
+      <c r="D4" s="77"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
+      <c r="I4" s="77"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -1890,17 +1890,17 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="69" t="s">
+      <c r="A11" s="77" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="69"/>
-      <c r="C11" s="69"/>
-      <c r="D11" s="69"/>
-      <c r="E11" s="69"/>
-      <c r="F11" s="69"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="69"/>
-      <c r="I11" s="69"/>
+      <c r="B11" s="77"/>
+      <c r="C11" s="77"/>
+      <c r="D11" s="77"/>
+      <c r="E11" s="77"/>
+      <c r="F11" s="77"/>
+      <c r="G11" s="77"/>
+      <c r="H11" s="77"/>
+      <c r="I11" s="77"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -1998,17 +1998,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="69" t="s">
+      <c r="A20" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="69"/>
-      <c r="C20" s="69"/>
-      <c r="D20" s="69"/>
-      <c r="E20" s="69"/>
-      <c r="F20" s="69"/>
-      <c r="G20" s="69"/>
-      <c r="H20" s="69"/>
-      <c r="I20" s="69"/>
+      <c r="B20" s="77"/>
+      <c r="C20" s="77"/>
+      <c r="D20" s="77"/>
+      <c r="E20" s="77"/>
+      <c r="F20" s="77"/>
+      <c r="G20" s="77"/>
+      <c r="H20" s="77"/>
+      <c r="I20" s="77"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
@@ -2033,17 +2033,17 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="69" t="s">
+      <c r="A24" s="77" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="69"/>
-      <c r="C24" s="69"/>
-      <c r="D24" s="69"/>
-      <c r="E24" s="69"/>
-      <c r="F24" s="69"/>
-      <c r="G24" s="69"/>
-      <c r="H24" s="69"/>
-      <c r="I24" s="69"/>
+      <c r="B24" s="77"/>
+      <c r="C24" s="77"/>
+      <c r="D24" s="77"/>
+      <c r="E24" s="77"/>
+      <c r="F24" s="77"/>
+      <c r="G24" s="77"/>
+      <c r="H24" s="77"/>
+      <c r="I24" s="77"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
@@ -2183,17 +2183,17 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="69" t="s">
+      <c r="A36" s="77" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="69"/>
-      <c r="C36" s="69"/>
-      <c r="D36" s="69"/>
-      <c r="E36" s="69"/>
-      <c r="F36" s="69"/>
-      <c r="G36" s="69"/>
-      <c r="H36" s="69"/>
-      <c r="I36" s="69"/>
+      <c r="B36" s="77"/>
+      <c r="C36" s="77"/>
+      <c r="D36" s="77"/>
+      <c r="E36" s="77"/>
+      <c r="F36" s="77"/>
+      <c r="G36" s="77"/>
+      <c r="H36" s="77"/>
+      <c r="I36" s="77"/>
     </row>
     <row r="37" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
@@ -2404,17 +2404,17 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="69" t="s">
+      <c r="A47" s="77" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="69"/>
-      <c r="C47" s="69"/>
-      <c r="D47" s="69"/>
-      <c r="E47" s="69"/>
-      <c r="F47" s="69"/>
-      <c r="G47" s="69"/>
-      <c r="H47" s="69"/>
-      <c r="I47" s="69"/>
+      <c r="B47" s="77"/>
+      <c r="C47" s="77"/>
+      <c r="D47" s="77"/>
+      <c r="E47" s="77"/>
+      <c r="F47" s="77"/>
+      <c r="G47" s="77"/>
+      <c r="H47" s="77"/>
+      <c r="I47" s="77"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
@@ -2447,17 +2447,17 @@
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="69" t="s">
+      <c r="A52" s="77" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="69"/>
-      <c r="C52" s="69"/>
-      <c r="D52" s="69"/>
-      <c r="E52" s="69"/>
-      <c r="F52" s="69"/>
-      <c r="G52" s="69"/>
-      <c r="H52" s="69"/>
-      <c r="I52" s="69"/>
+      <c r="B52" s="77"/>
+      <c r="C52" s="77"/>
+      <c r="D52" s="77"/>
+      <c r="E52" s="77"/>
+      <c r="F52" s="77"/>
+      <c r="G52" s="77"/>
+      <c r="H52" s="77"/>
+      <c r="I52" s="77"/>
     </row>
     <row r="53" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
@@ -3008,7 +3008,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03C3DC63-880C-4C7A-BD99-15B2870A7881}">
-  <dimension ref="A1:Q73"/>
+  <dimension ref="A1:Q99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
@@ -3020,7 +3020,7 @@
     <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -3277,10 +3277,10 @@
       <c r="I13" s="62" t="s">
         <v>188</v>
       </c>
-      <c r="J13" s="76" t="s">
+      <c r="J13" s="68" t="s">
         <v>319</v>
       </c>
-      <c r="K13" s="76" t="s">
+      <c r="K13" s="68" t="s">
         <v>320</v>
       </c>
     </row>
@@ -3745,17 +3745,17 @@
       <c r="D32" s="51">
         <v>9</v>
       </c>
-      <c r="E32" s="73">
+      <c r="E32" s="75">
         <v>22.99</v>
       </c>
-      <c r="F32" s="70" t="s">
+      <c r="F32" s="66" t="s">
         <v>316</v>
       </c>
-      <c r="G32" s="71" t="s">
+      <c r="G32" s="73" t="s">
         <v>180</v>
       </c>
-      <c r="H32" s="66"/>
-      <c r="I32" s="66"/>
+      <c r="H32" s="70"/>
+      <c r="I32" s="70"/>
       <c r="J32" s="50"/>
       <c r="K32" s="50"/>
     </row>
@@ -3772,13 +3772,13 @@
       <c r="D33" s="51">
         <v>7</v>
       </c>
-      <c r="E33" s="74"/>
-      <c r="F33" s="70" t="s">
+      <c r="E33" s="76"/>
+      <c r="F33" s="66" t="s">
         <v>315</v>
       </c>
-      <c r="G33" s="72"/>
-      <c r="H33" s="68"/>
-      <c r="I33" s="68"/>
+      <c r="G33" s="74"/>
+      <c r="H33" s="71"/>
+      <c r="I33" s="71"/>
       <c r="J33" s="50"/>
       <c r="K33" s="50"/>
     </row>
@@ -3796,11 +3796,11 @@
         <v>4</v>
       </c>
       <c r="E34" s="50"/>
-      <c r="F34" s="70" t="s">
+      <c r="F34" s="66" t="s">
         <v>318</v>
       </c>
       <c r="G34" s="51"/>
-      <c r="H34" s="70" t="s">
+      <c r="H34" s="66" t="s">
         <v>317</v>
       </c>
       <c r="I34" s="51"/>
@@ -3814,7 +3814,7 @@
       <c r="B35" s="51">
         <v>3</v>
       </c>
-      <c r="C35" s="77" t="s">
+      <c r="C35" s="69" t="s">
         <v>321</v>
       </c>
       <c r="D35" s="51">
@@ -3823,13 +3823,13 @@
       <c r="E35" s="50">
         <v>7.29</v>
       </c>
-      <c r="F35" s="70" t="s">
+      <c r="F35" s="66" t="s">
         <v>322</v>
       </c>
       <c r="G35" s="64" t="s">
         <v>180</v>
       </c>
-      <c r="H35" s="70"/>
+      <c r="H35" s="66"/>
       <c r="I35" s="51"/>
       <c r="J35" s="50"/>
       <c r="K35" s="50"/>
@@ -3850,13 +3850,13 @@
       <c r="E36" s="50">
         <v>21.45</v>
       </c>
-      <c r="F36" s="70" t="s">
+      <c r="F36" s="66" t="s">
         <v>314</v>
       </c>
       <c r="G36" s="64" t="s">
         <v>180</v>
       </c>
-      <c r="H36" s="70" t="s">
+      <c r="H36" s="66" t="s">
         <v>317</v>
       </c>
       <c r="I36" s="51"/>
@@ -3875,7 +3875,7 @@
       <c r="I37" s="51"/>
       <c r="J37" s="50"/>
       <c r="K37" s="50"/>
-      <c r="Q37" s="75"/>
+      <c r="Q37" s="67"/>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="51" t="s">
@@ -3891,7 +3891,7 @@
         <v>1</v>
       </c>
       <c r="E38" s="50"/>
-      <c r="F38" s="66" t="s">
+      <c r="F38" s="70" t="s">
         <v>300</v>
       </c>
       <c r="G38" s="51"/>
@@ -3914,7 +3914,7 @@
         <v>1</v>
       </c>
       <c r="E39" s="50"/>
-      <c r="F39" s="67"/>
+      <c r="F39" s="72"/>
       <c r="G39" s="51"/>
       <c r="H39" s="51"/>
       <c r="I39" s="51"/>
@@ -3935,7 +3935,7 @@
         <v>78</v>
       </c>
       <c r="E40" s="50"/>
-      <c r="F40" s="67"/>
+      <c r="F40" s="72"/>
       <c r="G40" s="51"/>
       <c r="H40" s="51"/>
       <c r="I40" s="51"/>
@@ -3956,7 +3956,7 @@
         <v>39</v>
       </c>
       <c r="E41" s="50"/>
-      <c r="F41" s="67"/>
+      <c r="F41" s="72"/>
       <c r="G41" s="51"/>
       <c r="H41" s="51"/>
       <c r="I41" s="51"/>
@@ -3977,7 +3977,7 @@
         <v>2</v>
       </c>
       <c r="E42" s="50"/>
-      <c r="F42" s="67"/>
+      <c r="F42" s="72"/>
       <c r="G42" s="51"/>
       <c r="H42" s="51"/>
       <c r="I42" s="51"/>
@@ -3998,7 +3998,7 @@
         <v>2</v>
       </c>
       <c r="E43" s="50"/>
-      <c r="F43" s="67"/>
+      <c r="F43" s="72"/>
       <c r="G43" s="51"/>
       <c r="H43" s="51"/>
       <c r="I43" s="51"/>
@@ -4019,7 +4019,7 @@
         <v>1</v>
       </c>
       <c r="E44" s="50"/>
-      <c r="F44" s="67"/>
+      <c r="F44" s="72"/>
       <c r="G44" s="51"/>
       <c r="H44" s="51"/>
       <c r="I44" s="51"/>
@@ -4040,7 +4040,7 @@
         <v>1</v>
       </c>
       <c r="E45" s="50"/>
-      <c r="F45" s="67"/>
+      <c r="F45" s="72"/>
       <c r="G45" s="51"/>
       <c r="H45" s="51"/>
       <c r="I45" s="51"/>
@@ -4061,7 +4061,7 @@
         <v>1</v>
       </c>
       <c r="E46" s="50"/>
-      <c r="F46" s="67"/>
+      <c r="F46" s="72"/>
       <c r="G46" s="51"/>
       <c r="H46" s="51"/>
       <c r="I46" s="51"/>
@@ -4082,7 +4082,7 @@
         <v>1</v>
       </c>
       <c r="E47" s="50"/>
-      <c r="F47" s="67"/>
+      <c r="F47" s="72"/>
       <c r="G47" s="51"/>
       <c r="H47" s="51"/>
       <c r="I47" s="51"/>
@@ -4103,7 +4103,7 @@
         <v>1</v>
       </c>
       <c r="E48" s="50"/>
-      <c r="F48" s="67"/>
+      <c r="F48" s="72"/>
       <c r="G48" s="51"/>
       <c r="H48" s="51"/>
       <c r="I48" s="51"/>
@@ -4124,7 +4124,7 @@
         <v>1</v>
       </c>
       <c r="E49" s="50"/>
-      <c r="F49" s="67"/>
+      <c r="F49" s="72"/>
       <c r="G49" s="51"/>
       <c r="H49" s="51"/>
       <c r="I49" s="51"/>
@@ -4145,7 +4145,7 @@
         <v>1</v>
       </c>
       <c r="E50" s="50"/>
-      <c r="F50" s="68"/>
+      <c r="F50" s="71"/>
       <c r="G50" s="51"/>
       <c r="H50" s="51"/>
       <c r="I50" s="51"/>
@@ -4156,105 +4156,43 @@
       <c r="K51" s="49"/>
       <c r="Q51" s="49"/>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A52" s="54" t="s">
-        <v>237</v>
-      </c>
-      <c r="B52" s="54">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A54" s="54" t="s">
+        <v>195</v>
+      </c>
+      <c r="B54" s="54">
         <v>2</v>
       </c>
-      <c r="C52" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D52" s="54"/>
-      <c r="E52" s="53"/>
-      <c r="F52" s="54"/>
-      <c r="G52" s="54"/>
-      <c r="H52" s="54"/>
-      <c r="I52" s="54"/>
-      <c r="J52" s="53">
-        <f>SUM(J53:J55)</f>
-        <v>402</v>
-      </c>
-    </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A53" s="51" t="s">
-        <v>235</v>
-      </c>
-      <c r="B53" s="51">
-        <v>3</v>
-      </c>
-      <c r="C53" s="52" t="s">
-        <v>234</v>
-      </c>
-      <c r="D53" s="51">
-        <v>3</v>
-      </c>
-      <c r="E53" s="50">
-        <v>65</v>
-      </c>
-      <c r="F53" s="51" t="s">
-        <v>231</v>
-      </c>
-      <c r="G53" s="56" t="s">
-        <v>180</v>
-      </c>
-      <c r="H53" s="57">
-        <v>46213</v>
-      </c>
-      <c r="I53" s="51" t="s">
-        <v>187</v>
-      </c>
-      <c r="J53" s="50">
-        <f>D53*E53</f>
-        <v>195</v>
-      </c>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A54" s="51" t="s">
-        <v>233</v>
-      </c>
-      <c r="B54" s="51">
-        <v>3</v>
-      </c>
-      <c r="C54" s="52" t="s">
-        <v>232</v>
-      </c>
-      <c r="D54" s="51">
-        <v>3</v>
-      </c>
-      <c r="E54" s="50">
-        <v>69</v>
-      </c>
-      <c r="F54" s="51" t="s">
-        <v>231</v>
-      </c>
-      <c r="G54" s="56" t="s">
-        <v>180</v>
-      </c>
-      <c r="H54" s="51"/>
-      <c r="I54" s="51"/>
-      <c r="J54" s="50">
-        <f>D54*E54</f>
-        <v>207</v>
+      <c r="C54" s="55" t="s">
+        <v>265</v>
+      </c>
+      <c r="D54" s="54">
+        <v>2</v>
+      </c>
+      <c r="E54" s="53"/>
+      <c r="F54" s="54"/>
+      <c r="G54" s="54"/>
+      <c r="H54" s="54"/>
+      <c r="I54" s="54"/>
+      <c r="J54" s="53">
+        <f>SUM(J55:J56)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="51" t="s">
-        <v>230</v>
+        <v>194</v>
       </c>
       <c r="B55" s="51">
         <v>3</v>
       </c>
       <c r="C55" s="52" t="s">
-        <v>229</v>
-      </c>
-      <c r="D55" s="51">
-        <v>3</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="D55" s="51"/>
       <c r="E55" s="50"/>
       <c r="F55" s="51" t="s">
-        <v>228</v>
+        <v>190</v>
       </c>
       <c r="G55" s="51"/>
       <c r="H55" s="51"/>
@@ -4262,342 +4200,467 @@
       <c r="J55" s="50"/>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A56" s="54" t="s">
+      <c r="A56" s="51" t="s">
+        <v>192</v>
+      </c>
+      <c r="B56" s="51">
+        <v>3</v>
+      </c>
+      <c r="C56" s="52" t="s">
+        <v>191</v>
+      </c>
+      <c r="D56" s="51"/>
+      <c r="E56" s="50"/>
+      <c r="F56" s="51" t="s">
+        <v>190</v>
+      </c>
+      <c r="G56" s="51"/>
+      <c r="H56" s="51"/>
+      <c r="I56" s="51"/>
+      <c r="J56" s="50"/>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A78" s="54" t="s">
+        <v>237</v>
+      </c>
+      <c r="B78" s="54">
+        <v>2</v>
+      </c>
+      <c r="C78" s="55" t="s">
+        <v>236</v>
+      </c>
+      <c r="D78" s="54"/>
+      <c r="E78" s="53"/>
+      <c r="F78" s="54"/>
+      <c r="G78" s="54"/>
+      <c r="H78" s="54"/>
+      <c r="I78" s="54"/>
+      <c r="J78" s="53">
+        <f>SUM(J79:J81)</f>
+        <v>402</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A79" s="51" t="s">
+        <v>235</v>
+      </c>
+      <c r="B79" s="51">
+        <v>3</v>
+      </c>
+      <c r="C79" s="52" t="s">
+        <v>234</v>
+      </c>
+      <c r="D79" s="51">
+        <v>3</v>
+      </c>
+      <c r="E79" s="50">
+        <v>65</v>
+      </c>
+      <c r="F79" s="51" t="s">
+        <v>231</v>
+      </c>
+      <c r="G79" s="56" t="s">
+        <v>180</v>
+      </c>
+      <c r="H79" s="57">
+        <v>46213</v>
+      </c>
+      <c r="I79" s="51" t="s">
+        <v>187</v>
+      </c>
+      <c r="J79" s="50">
+        <f>D79*E79</f>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A80" s="51" t="s">
+        <v>233</v>
+      </c>
+      <c r="B80" s="51">
+        <v>3</v>
+      </c>
+      <c r="C80" s="52" t="s">
+        <v>232</v>
+      </c>
+      <c r="D80" s="51">
+        <v>3</v>
+      </c>
+      <c r="E80" s="50">
+        <v>69</v>
+      </c>
+      <c r="F80" s="51" t="s">
+        <v>231</v>
+      </c>
+      <c r="G80" s="56" t="s">
+        <v>180</v>
+      </c>
+      <c r="H80" s="51"/>
+      <c r="I80" s="51"/>
+      <c r="J80" s="50">
+        <f>D80*E80</f>
+        <v>207</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A81" s="51" t="s">
+        <v>230</v>
+      </c>
+      <c r="B81" s="51">
+        <v>3</v>
+      </c>
+      <c r="C81" s="52" t="s">
+        <v>229</v>
+      </c>
+      <c r="D81" s="51">
+        <v>3</v>
+      </c>
+      <c r="E81" s="50"/>
+      <c r="F81" s="51" t="s">
+        <v>228</v>
+      </c>
+      <c r="G81" s="51"/>
+      <c r="H81" s="51"/>
+      <c r="I81" s="51"/>
+      <c r="J81" s="50"/>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A82" s="54" t="s">
         <v>227</v>
       </c>
-      <c r="B56" s="54">
+      <c r="B82" s="54">
         <v>2</v>
       </c>
-      <c r="C56" s="55" t="s">
+      <c r="C82" s="55" t="s">
         <v>226</v>
       </c>
-      <c r="D56" s="54"/>
-      <c r="E56" s="53"/>
-      <c r="F56" s="54"/>
-      <c r="G56" s="54"/>
-      <c r="H56" s="54"/>
-      <c r="I56" s="54"/>
-      <c r="J56" s="53">
-        <f>SUM(J57:J60)</f>
+      <c r="D82" s="54"/>
+      <c r="E82" s="53"/>
+      <c r="F82" s="54"/>
+      <c r="G82" s="54"/>
+      <c r="H82" s="54"/>
+      <c r="I82" s="54"/>
+      <c r="J82" s="53">
+        <f>SUM(J83:J86)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A57" s="51" t="s">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A83" s="51" t="s">
         <v>225</v>
       </c>
-      <c r="B57" s="51">
-        <v>3</v>
-      </c>
-      <c r="C57" s="52" t="s">
+      <c r="B83" s="51">
+        <v>3</v>
+      </c>
+      <c r="C83" s="52" t="s">
         <v>224</v>
       </c>
-      <c r="D57" s="51"/>
-      <c r="E57" s="50"/>
-      <c r="F57" s="51" t="s">
+      <c r="D83" s="51"/>
+      <c r="E83" s="50"/>
+      <c r="F83" s="51" t="s">
         <v>223</v>
       </c>
-      <c r="G57" s="51"/>
-      <c r="H57" s="51"/>
-      <c r="I57" s="51"/>
-      <c r="J57" s="50"/>
-    </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A58" s="51" t="s">
+      <c r="G83" s="51"/>
+      <c r="H83" s="51"/>
+      <c r="I83" s="51"/>
+      <c r="J83" s="50"/>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" s="51" t="s">
         <v>222</v>
       </c>
-      <c r="B58" s="51">
-        <v>3</v>
-      </c>
-      <c r="C58" s="52" t="s">
+      <c r="B84" s="51">
+        <v>3</v>
+      </c>
+      <c r="C84" s="52" t="s">
         <v>221</v>
       </c>
-      <c r="D58" s="51"/>
-      <c r="E58" s="50"/>
-      <c r="F58" s="51" t="s">
+      <c r="D84" s="51"/>
+      <c r="E84" s="50"/>
+      <c r="F84" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="G58" s="51"/>
-      <c r="H58" s="51"/>
-      <c r="I58" s="51"/>
-      <c r="J58" s="50"/>
-    </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A59" s="51" t="s">
+      <c r="G84" s="51"/>
+      <c r="H84" s="51"/>
+      <c r="I84" s="51"/>
+      <c r="J84" s="50"/>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" s="51" t="s">
         <v>219</v>
       </c>
-      <c r="B59" s="51">
-        <v>3</v>
-      </c>
-      <c r="C59" s="52" t="s">
+      <c r="B85" s="51">
+        <v>3</v>
+      </c>
+      <c r="C85" s="52" t="s">
         <v>218</v>
       </c>
-      <c r="D59" s="51"/>
-      <c r="E59" s="50"/>
-      <c r="F59" s="51" t="s">
+      <c r="D85" s="51"/>
+      <c r="E85" s="50"/>
+      <c r="F85" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="G59" s="51"/>
-      <c r="H59" s="51"/>
-      <c r="I59" s="51"/>
-      <c r="J59" s="50"/>
-    </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A60" s="51" t="s">
+      <c r="G85" s="51"/>
+      <c r="H85" s="51"/>
+      <c r="I85" s="51"/>
+      <c r="J85" s="50"/>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A86" s="51" t="s">
         <v>217</v>
       </c>
-      <c r="B60" s="51">
-        <v>3</v>
-      </c>
-      <c r="C60" s="52" t="s">
+      <c r="B86" s="51">
+        <v>3</v>
+      </c>
+      <c r="C86" s="52" t="s">
         <v>216</v>
       </c>
-      <c r="D60" s="51"/>
-      <c r="E60" s="50"/>
-      <c r="F60" s="51" t="s">
+      <c r="D86" s="51"/>
+      <c r="E86" s="50"/>
+      <c r="F86" s="51" t="s">
         <v>215</v>
       </c>
-      <c r="G60" s="51"/>
-      <c r="H60" s="51"/>
-      <c r="I60" s="51"/>
-      <c r="J60" s="50"/>
-    </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A61" s="54" t="s">
+      <c r="G86" s="51"/>
+      <c r="H86" s="51"/>
+      <c r="I86" s="51"/>
+      <c r="J86" s="50"/>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" s="54" t="s">
         <v>214</v>
       </c>
-      <c r="B61" s="54">
+      <c r="B87" s="54">
         <v>2</v>
       </c>
-      <c r="C61" s="55" t="s">
+      <c r="C87" s="55" t="s">
         <v>213</v>
       </c>
-      <c r="D61" s="54"/>
-      <c r="E61" s="53"/>
-      <c r="F61" s="54"/>
-      <c r="G61" s="54"/>
-      <c r="H61" s="54"/>
-      <c r="I61" s="54"/>
-      <c r="J61" s="53">
-        <f>SUM(J62:J63)</f>
+      <c r="D87" s="54"/>
+      <c r="E87" s="53"/>
+      <c r="F87" s="54"/>
+      <c r="G87" s="54"/>
+      <c r="H87" s="54"/>
+      <c r="I87" s="54"/>
+      <c r="J87" s="53">
+        <f>SUM(J88:J89)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A62" s="51" t="s">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" s="51" t="s">
         <v>212</v>
       </c>
-      <c r="B62" s="51">
-        <v>3</v>
-      </c>
-      <c r="C62" s="52" t="s">
+      <c r="B88" s="51">
+        <v>3</v>
+      </c>
+      <c r="C88" s="52" t="s">
         <v>211</v>
       </c>
-      <c r="D62" s="51"/>
-      <c r="E62" s="50"/>
-      <c r="F62" s="51" t="s">
+      <c r="D88" s="51"/>
+      <c r="E88" s="50"/>
+      <c r="F88" s="51" t="s">
         <v>210</v>
       </c>
-      <c r="G62" s="51"/>
-      <c r="H62" s="51"/>
-      <c r="I62" s="51"/>
-      <c r="J62" s="50"/>
-    </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A63" s="51" t="s">
+      <c r="G88" s="51"/>
+      <c r="H88" s="51"/>
+      <c r="I88" s="51"/>
+      <c r="J88" s="50"/>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" s="51" t="s">
         <v>209</v>
       </c>
-      <c r="B63" s="51">
-        <v>3</v>
-      </c>
-      <c r="C63" s="52" t="s">
+      <c r="B89" s="51">
+        <v>3</v>
+      </c>
+      <c r="C89" s="52" t="s">
         <v>208</v>
       </c>
-      <c r="D63" s="51"/>
-      <c r="E63" s="50"/>
-      <c r="F63" s="51" t="s">
+      <c r="D89" s="51"/>
+      <c r="E89" s="50"/>
+      <c r="F89" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="G63" s="51"/>
-      <c r="H63" s="51"/>
-      <c r="I63" s="51"/>
-      <c r="J63" s="50"/>
-    </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A64" s="54" t="s">
+      <c r="G89" s="51"/>
+      <c r="H89" s="51"/>
+      <c r="I89" s="51"/>
+      <c r="J89" s="50"/>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A90" s="54" t="s">
         <v>207</v>
       </c>
-      <c r="B64" s="54">
+      <c r="B90" s="54">
         <v>2</v>
       </c>
-      <c r="C64" s="55" t="s">
+      <c r="C90" s="55" t="s">
         <v>206</v>
       </c>
-      <c r="D64" s="54"/>
-      <c r="E64" s="53"/>
-      <c r="F64" s="54"/>
-      <c r="G64" s="54"/>
-      <c r="H64" s="54"/>
-      <c r="I64" s="54"/>
-      <c r="J64" s="53">
-        <f>SUM(J65:J68)</f>
+      <c r="D90" s="54"/>
+      <c r="E90" s="53"/>
+      <c r="F90" s="54"/>
+      <c r="G90" s="54"/>
+      <c r="H90" s="54"/>
+      <c r="I90" s="54"/>
+      <c r="J90" s="53">
+        <f>SUM(J91:J94)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A65" s="51" t="s">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A91" s="51" t="s">
         <v>205</v>
       </c>
-      <c r="B65" s="51">
-        <v>3</v>
-      </c>
-      <c r="C65" s="52" t="s">
+      <c r="B91" s="51">
+        <v>3</v>
+      </c>
+      <c r="C91" s="52" t="s">
         <v>204</v>
       </c>
-      <c r="D65" s="51"/>
-      <c r="E65" s="50"/>
-      <c r="F65" s="51" t="s">
+      <c r="D91" s="51"/>
+      <c r="E91" s="50"/>
+      <c r="F91" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="G65" s="51"/>
-      <c r="H65" s="51"/>
-      <c r="I65" s="51"/>
-      <c r="J65" s="50"/>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A66" s="51" t="s">
+      <c r="G91" s="51"/>
+      <c r="H91" s="51"/>
+      <c r="I91" s="51"/>
+      <c r="J91" s="50"/>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A92" s="51" t="s">
         <v>203</v>
       </c>
-      <c r="B66" s="51">
-        <v>3</v>
-      </c>
-      <c r="C66" s="52" t="s">
+      <c r="B92" s="51">
+        <v>3</v>
+      </c>
+      <c r="C92" s="52" t="s">
         <v>202</v>
       </c>
-      <c r="D66" s="51">
+      <c r="D92" s="51">
         <v>1</v>
       </c>
-      <c r="E66" s="50"/>
-      <c r="F66" s="51" t="s">
+      <c r="E92" s="50"/>
+      <c r="F92" s="51" t="s">
         <v>201</v>
       </c>
-      <c r="G66" s="51"/>
-      <c r="H66" s="51"/>
-      <c r="I66" s="51"/>
-      <c r="J66" s="50"/>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A67" s="51" t="s">
+      <c r="G92" s="51"/>
+      <c r="H92" s="51"/>
+      <c r="I92" s="51"/>
+      <c r="J92" s="50"/>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A93" s="51" t="s">
         <v>200</v>
       </c>
-      <c r="B67" s="51">
-        <v>3</v>
-      </c>
-      <c r="C67" s="52" t="s">
+      <c r="B93" s="51">
+        <v>3</v>
+      </c>
+      <c r="C93" s="52" t="s">
         <v>199</v>
       </c>
-      <c r="D67" s="51"/>
-      <c r="E67" s="50"/>
-      <c r="F67" s="51" t="s">
+      <c r="D93" s="51"/>
+      <c r="E93" s="50"/>
+      <c r="F93" s="51" t="s">
         <v>198</v>
       </c>
-      <c r="G67" s="51"/>
-      <c r="H67" s="51"/>
-      <c r="I67" s="51"/>
-      <c r="J67" s="50"/>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A68" s="51" t="s">
+      <c r="G93" s="51"/>
+      <c r="H93" s="51"/>
+      <c r="I93" s="51"/>
+      <c r="J93" s="50"/>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A94" s="51" t="s">
         <v>197</v>
       </c>
-      <c r="B68" s="51">
-        <v>3</v>
-      </c>
-      <c r="C68" s="52" t="s">
+      <c r="B94" s="51">
+        <v>3</v>
+      </c>
+      <c r="C94" s="52" t="s">
         <v>196</v>
       </c>
-      <c r="D68" s="51"/>
-      <c r="E68" s="50"/>
-      <c r="F68" s="51" t="s">
+      <c r="D94" s="51"/>
+      <c r="E94" s="50"/>
+      <c r="F94" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="G68" s="51"/>
-      <c r="H68" s="51"/>
-      <c r="I68" s="51"/>
-      <c r="J68" s="50"/>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A69" s="54" t="s">
+      <c r="G94" s="51"/>
+      <c r="H94" s="51"/>
+      <c r="I94" s="51"/>
+      <c r="J94" s="50"/>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A95" s="54" t="s">
         <v>195</v>
       </c>
-      <c r="B69" s="54">
+      <c r="B95" s="54">
         <v>2</v>
       </c>
-      <c r="C69" s="55" t="s">
+      <c r="C95" s="55" t="s">
         <v>265</v>
       </c>
-      <c r="D69" s="54">
+      <c r="D95" s="54">
         <v>2</v>
       </c>
-      <c r="E69" s="53"/>
-      <c r="F69" s="54"/>
-      <c r="G69" s="54"/>
-      <c r="H69" s="54"/>
-      <c r="I69" s="54"/>
-      <c r="J69" s="53">
-        <f>SUM(J70:J71)</f>
+      <c r="E95" s="53"/>
+      <c r="F95" s="54"/>
+      <c r="G95" s="54"/>
+      <c r="H95" s="54"/>
+      <c r="I95" s="54"/>
+      <c r="J95" s="53">
+        <f>SUM(J96:J97)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A70" s="51" t="s">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A96" s="51" t="s">
         <v>194</v>
       </c>
-      <c r="B70" s="51">
-        <v>3</v>
-      </c>
-      <c r="C70" s="52" t="s">
+      <c r="B96" s="51">
+        <v>3</v>
+      </c>
+      <c r="C96" s="52" t="s">
         <v>193</v>
       </c>
-      <c r="D70" s="51"/>
-      <c r="E70" s="50"/>
-      <c r="F70" s="51" t="s">
+      <c r="D96" s="51"/>
+      <c r="E96" s="50"/>
+      <c r="F96" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="G70" s="51"/>
-      <c r="H70" s="51"/>
-      <c r="I70" s="51"/>
-      <c r="J70" s="50"/>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A71" s="51" t="s">
+      <c r="G96" s="51"/>
+      <c r="H96" s="51"/>
+      <c r="I96" s="51"/>
+      <c r="J96" s="50"/>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A97" s="51" t="s">
         <v>192</v>
       </c>
-      <c r="B71" s="51">
-        <v>3</v>
-      </c>
-      <c r="C71" s="52" t="s">
+      <c r="B97" s="51">
+        <v>3</v>
+      </c>
+      <c r="C97" s="52" t="s">
         <v>191</v>
       </c>
-      <c r="D71" s="51"/>
-      <c r="E71" s="50"/>
-      <c r="F71" s="51" t="s">
+      <c r="D97" s="51"/>
+      <c r="E97" s="50"/>
+      <c r="F97" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="G71" s="51"/>
-      <c r="H71" s="51"/>
-      <c r="I71" s="51"/>
-      <c r="J71" s="50"/>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F73" s="48" t="s">
+      <c r="G97" s="51"/>
+      <c r="H97" s="51"/>
+      <c r="I97" s="51"/>
+      <c r="J97" s="50"/>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F99" s="48" t="s">
         <v>189</v>
       </c>
-      <c r="G73" s="47"/>
-      <c r="H73" s="47"/>
-      <c r="I73" s="47"/>
-      <c r="J73" s="46">
-        <f>K15+K21+J52+J56+J61+J64+J69</f>
+      <c r="G99" s="47"/>
+      <c r="H99" s="47"/>
+      <c r="I99" s="47"/>
+      <c r="J99" s="46">
+        <f>K15+K21+J78+J82+J87+J90+J95</f>
         <v>1044</v>
       </c>
     </row>
@@ -4617,8 +4680,8 @@
     <hyperlink ref="G8" r:id="rId4" xr:uid="{60429B27-A38D-454F-B173-6703031A5589}"/>
     <hyperlink ref="G6" r:id="rId5" xr:uid="{0A9A04AE-D73D-4785-8B94-5732DA2EFFEB}"/>
     <hyperlink ref="G4" r:id="rId6" xr:uid="{8965FEC0-8122-4167-90F4-C3780CE3A5C5}"/>
-    <hyperlink ref="G54" r:id="rId7" xr:uid="{8A31F0DB-620C-4B1D-BD14-CB8720C07EC8}"/>
-    <hyperlink ref="G53" r:id="rId8" xr:uid="{9E52DD90-A4C0-4AFB-B727-068C5A377BE2}"/>
+    <hyperlink ref="G80" r:id="rId7" xr:uid="{8A31F0DB-620C-4B1D-BD14-CB8720C07EC8}"/>
+    <hyperlink ref="G79" r:id="rId8" xr:uid="{9E52DD90-A4C0-4AFB-B727-068C5A377BE2}"/>
     <hyperlink ref="G19" r:id="rId9" xr:uid="{8091DB70-558E-4592-B9B4-38004DC7FBB7}"/>
     <hyperlink ref="G18" r:id="rId10" xr:uid="{F7F75BD6-DB10-4AC2-8841-880D0CC3617B}"/>
     <hyperlink ref="G17" r:id="rId11" xr:uid="{279313D3-1F5C-43AF-9B3D-757C7867AE3E}"/>

</xml_diff>

<commit_message>
15:1 Cycloidal Gearbox Gears
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C720699E-F331-41C9-9D49-56EFBDC42975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA663457-41B3-4D8E-AB62-70FE1944A91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="326">
   <si>
     <t>6-DoF Arm — Gravity Torque Budget v2 (elbow-mounted forearm roll)</t>
   </si>
@@ -997,9 +997,6 @@
     <t xml:space="preserve">M2.5 x 4mm length </t>
   </si>
   <si>
-    <t>Shipping</t>
-  </si>
-  <si>
     <t>Total Cost</t>
   </si>
   <si>
@@ -1007,6 +1004,18 @@
   </si>
   <si>
     <t>M2.5 x 4mm length (50 pieces)</t>
+  </si>
+  <si>
+    <t>.5 spacer</t>
+  </si>
+  <si>
+    <t>1.2.26</t>
+  </si>
+  <si>
+    <t>Shipping/Tax</t>
+  </si>
+  <si>
+    <t># of Packs Ordered</t>
   </si>
 </sst>
 </file>
@@ -1308,7 +1317,7 @@
     <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1495,6 +1504,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -3019,7 +3037,7 @@
     <col min="6" max="6" width="66.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
@@ -3275,13 +3293,13 @@
         <v>184</v>
       </c>
       <c r="I13" s="62" t="s">
-        <v>188</v>
+        <v>325</v>
       </c>
       <c r="J13" s="68" t="s">
+        <v>324</v>
+      </c>
+      <c r="K13" s="68" t="s">
         <v>319</v>
-      </c>
-      <c r="K13" s="68" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -3498,8 +3516,8 @@
       <c r="I21" s="54"/>
       <c r="J21" s="53"/>
       <c r="K21" s="53">
-        <f>SUM(K22:K31)</f>
-        <v>0</v>
+        <f>SUM(K22:K51)+SUM(J22:J51)</f>
+        <v>135.47999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -3524,10 +3542,19 @@
       <c r="G22" s="63" t="s">
         <v>180</v>
       </c>
-      <c r="H22" s="51"/>
-      <c r="I22" s="51"/>
-      <c r="J22" s="50"/>
-      <c r="K22" s="50"/>
+      <c r="H22" s="57">
+        <v>46230</v>
+      </c>
+      <c r="I22" s="51">
+        <v>1</v>
+      </c>
+      <c r="J22" s="75">
+        <v>7.68</v>
+      </c>
+      <c r="K22" s="50">
+        <f>I22*E22</f>
+        <v>7.21</v>
+      </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="51"/>
@@ -3539,7 +3566,7 @@
       <c r="G23" s="51"/>
       <c r="H23" s="57"/>
       <c r="I23" s="51"/>
-      <c r="J23" s="50"/>
+      <c r="J23" s="78"/>
       <c r="K23" s="50"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -3564,10 +3591,17 @@
       <c r="G24" s="64" t="s">
         <v>180</v>
       </c>
-      <c r="H24" s="51"/>
-      <c r="I24" s="51"/>
-      <c r="J24" s="50"/>
-      <c r="K24" s="50"/>
+      <c r="H24" s="57">
+        <v>46230</v>
+      </c>
+      <c r="I24" s="51">
+        <v>3</v>
+      </c>
+      <c r="J24" s="78"/>
+      <c r="K24" s="50">
+        <f t="shared" ref="K23:K36" si="0">I24*E24</f>
+        <v>38.97</v>
+      </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="51" t="s">
@@ -3591,10 +3625,17 @@
       <c r="G25" s="64" t="s">
         <v>180</v>
       </c>
-      <c r="H25" s="51"/>
-      <c r="I25" s="51"/>
-      <c r="J25" s="50"/>
-      <c r="K25" s="50"/>
+      <c r="H25" s="57">
+        <v>46230</v>
+      </c>
+      <c r="I25" s="51">
+        <v>1</v>
+      </c>
+      <c r="J25" s="78"/>
+      <c r="K25" s="50">
+        <f t="shared" si="0"/>
+        <v>9.99</v>
+      </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="51" t="s">
@@ -3618,10 +3659,17 @@
       <c r="G26" s="64" t="s">
         <v>180</v>
       </c>
-      <c r="H26" s="51"/>
-      <c r="I26" s="51"/>
-      <c r="J26" s="50"/>
-      <c r="K26" s="50"/>
+      <c r="H26" s="57">
+        <v>46230</v>
+      </c>
+      <c r="I26" s="51">
+        <v>1</v>
+      </c>
+      <c r="J26" s="78"/>
+      <c r="K26" s="50">
+        <f t="shared" si="0"/>
+        <v>9.7899999999999991</v>
+      </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="51"/>
@@ -3633,7 +3681,7 @@
       <c r="G27" s="51"/>
       <c r="H27" s="51"/>
       <c r="I27" s="51"/>
-      <c r="J27" s="50"/>
+      <c r="J27" s="78"/>
       <c r="K27" s="50"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -3658,10 +3706,17 @@
       <c r="G28" s="64" t="s">
         <v>180</v>
       </c>
-      <c r="H28" s="51"/>
-      <c r="I28" s="51"/>
-      <c r="J28" s="50"/>
-      <c r="K28" s="50"/>
+      <c r="H28" s="57">
+        <v>46230</v>
+      </c>
+      <c r="I28" s="51">
+        <v>1</v>
+      </c>
+      <c r="J28" s="78"/>
+      <c r="K28" s="50">
+        <f t="shared" si="0"/>
+        <v>6.99</v>
+      </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="51" t="s">
@@ -3685,10 +3740,17 @@
       <c r="G29" s="64" t="s">
         <v>180</v>
       </c>
-      <c r="H29" s="51"/>
-      <c r="I29" s="51"/>
-      <c r="J29" s="50"/>
-      <c r="K29" s="50"/>
+      <c r="H29" s="57">
+        <v>46230</v>
+      </c>
+      <c r="I29" s="51">
+        <v>1</v>
+      </c>
+      <c r="J29" s="78"/>
+      <c r="K29" s="50">
+        <f t="shared" si="0"/>
+        <v>8.99</v>
+      </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="51" t="s">
@@ -3702,7 +3764,7 @@
       <c r="G30" s="51"/>
       <c r="H30" s="51"/>
       <c r="I30" s="51"/>
-      <c r="J30" s="50"/>
+      <c r="J30" s="78"/>
       <c r="K30" s="50"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -3727,10 +3789,17 @@
       <c r="G31" s="64" t="s">
         <v>180</v>
       </c>
-      <c r="H31" s="51"/>
-      <c r="I31" s="51"/>
-      <c r="J31" s="50"/>
-      <c r="K31" s="50"/>
+      <c r="H31" s="57">
+        <v>46230</v>
+      </c>
+      <c r="I31" s="51">
+        <v>2</v>
+      </c>
+      <c r="J31" s="78"/>
+      <c r="K31" s="50">
+        <f t="shared" si="0"/>
+        <v>15.58</v>
+      </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="51" t="s">
@@ -3754,10 +3823,17 @@
       <c r="G32" s="73" t="s">
         <v>180</v>
       </c>
-      <c r="H32" s="70"/>
-      <c r="I32" s="70"/>
-      <c r="J32" s="50"/>
-      <c r="K32" s="50"/>
+      <c r="H32" s="79">
+        <v>46230</v>
+      </c>
+      <c r="I32" s="70">
+        <v>1</v>
+      </c>
+      <c r="J32" s="78"/>
+      <c r="K32" s="75">
+        <f t="shared" si="0"/>
+        <v>22.99</v>
+      </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="51" t="s">
@@ -3777,10 +3853,10 @@
         <v>315</v>
       </c>
       <c r="G33" s="74"/>
-      <c r="H33" s="71"/>
+      <c r="H33" s="80"/>
       <c r="I33" s="71"/>
-      <c r="J33" s="50"/>
-      <c r="K33" s="50"/>
+      <c r="J33" s="78"/>
+      <c r="K33" s="76"/>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="51" t="s">
@@ -3804,7 +3880,7 @@
         <v>317</v>
       </c>
       <c r="I34" s="51"/>
-      <c r="J34" s="50"/>
+      <c r="J34" s="78"/>
       <c r="K34" s="50"/>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
@@ -3815,7 +3891,7 @@
         <v>3</v>
       </c>
       <c r="C35" s="69" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D35" s="51">
         <v>1</v>
@@ -3824,15 +3900,22 @@
         <v>7.29</v>
       </c>
       <c r="F35" s="66" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G35" s="64" t="s">
         <v>180</v>
       </c>
-      <c r="H35" s="66"/>
-      <c r="I35" s="51"/>
-      <c r="J35" s="50"/>
-      <c r="K35" s="50"/>
+      <c r="H35" s="57">
+        <v>46230</v>
+      </c>
+      <c r="I35" s="51">
+        <v>1</v>
+      </c>
+      <c r="J35" s="78"/>
+      <c r="K35" s="50">
+        <f t="shared" si="0"/>
+        <v>7.29</v>
+      </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="51" t="s">
@@ -3860,7 +3943,7 @@
         <v>317</v>
       </c>
       <c r="I36" s="51"/>
-      <c r="J36" s="50"/>
+      <c r="J36" s="76"/>
       <c r="K36" s="50"/>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
@@ -3971,10 +4054,10 @@
         <v>3</v>
       </c>
       <c r="C42" s="52" t="s">
-        <v>291</v>
+        <v>322</v>
       </c>
       <c r="D42" s="51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E42" s="50"/>
       <c r="F42" s="72"/>
@@ -3992,7 +4075,7 @@
         <v>3</v>
       </c>
       <c r="C43" s="52" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D43" s="51">
         <v>2</v>
@@ -4013,10 +4096,10 @@
         <v>3</v>
       </c>
       <c r="C44" s="52" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D44" s="51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E44" s="50"/>
       <c r="F44" s="72"/>
@@ -4034,7 +4117,7 @@
         <v>3</v>
       </c>
       <c r="C45" s="52" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D45" s="51">
         <v>1</v>
@@ -4055,7 +4138,7 @@
         <v>3</v>
       </c>
       <c r="C46" s="52" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D46" s="51">
         <v>1</v>
@@ -4076,7 +4159,7 @@
         <v>3</v>
       </c>
       <c r="C47" s="52" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D47" s="51">
         <v>1</v>
@@ -4097,7 +4180,7 @@
         <v>3</v>
       </c>
       <c r="C48" s="52" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D48" s="51">
         <v>1</v>
@@ -4139,13 +4222,13 @@
         <v>3</v>
       </c>
       <c r="C50" s="52" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D50" s="51">
         <v>1</v>
       </c>
       <c r="E50" s="50"/>
-      <c r="F50" s="71"/>
+      <c r="F50" s="72"/>
       <c r="G50" s="51"/>
       <c r="H50" s="51"/>
       <c r="I50" s="51"/>
@@ -4153,7 +4236,25 @@
       <c r="K50" s="50"/>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K51" s="49"/>
+      <c r="A51" s="51" t="s">
+        <v>323</v>
+      </c>
+      <c r="B51" s="51">
+        <v>3</v>
+      </c>
+      <c r="C51" s="52" t="s">
+        <v>301</v>
+      </c>
+      <c r="D51" s="51">
+        <v>1</v>
+      </c>
+      <c r="E51" s="50"/>
+      <c r="F51" s="71"/>
+      <c r="G51" s="51"/>
+      <c r="H51" s="51"/>
+      <c r="I51" s="51"/>
+      <c r="J51" s="50"/>
+      <c r="K51" s="50"/>
       <c r="Q51" s="49"/>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
@@ -4174,8 +4275,9 @@
       <c r="G54" s="54"/>
       <c r="H54" s="54"/>
       <c r="I54" s="54"/>
-      <c r="J54" s="53">
-        <f>SUM(J55:J56)</f>
+      <c r="J54" s="53"/>
+      <c r="K54" s="53">
+        <f>SUM(K55:K56)</f>
         <v>0</v>
       </c>
     </row>
@@ -4198,6 +4300,7 @@
       <c r="H55" s="51"/>
       <c r="I55" s="51"/>
       <c r="J55" s="50"/>
+      <c r="K55" s="50"/>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="51" t="s">
@@ -4218,6 +4321,7 @@
       <c r="H56" s="51"/>
       <c r="I56" s="51"/>
       <c r="J56" s="50"/>
+      <c r="K56" s="50"/>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="54" t="s">
@@ -4661,16 +4765,18 @@
       <c r="I99" s="47"/>
       <c r="J99" s="46">
         <f>K15+K21+J78+J82+J87+J90+J95</f>
-        <v>1044</v>
+        <v>1179.48</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
+    <mergeCell ref="J22:J36"/>
+    <mergeCell ref="K32:K33"/>
     <mergeCell ref="I32:I33"/>
-    <mergeCell ref="F38:F50"/>
     <mergeCell ref="G32:G33"/>
     <mergeCell ref="E32:E33"/>
     <mergeCell ref="H32:H33"/>
+    <mergeCell ref="F38:F51"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Finished with 15:1 gearbox
Next step is to start printing the parts of the gearbox.
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA663457-41B3-4D8E-AB62-70FE1944A91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BA4751-F5D9-45A3-9659-608289DA6FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3778,7 +3778,7 @@
         <v>270</v>
       </c>
       <c r="D31" s="51">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E31" s="50">
         <v>7.79</v>

</xml_diff>

<commit_message>
Ordered parts for 15:1
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5291A94D-636D-4B0F-8115-4E7C3D7B2448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADBA8DFD-6C6E-4C1A-AA6F-0940B37E4555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="319">
   <si>
     <t>6-DoF Arm — Gravity Torque Budget v2 (elbow-mounted forearm roll)</t>
   </si>
@@ -821,9 +821,6 @@
   </si>
   <si>
     <t>M5x0.8 x 10mm length</t>
-  </si>
-  <si>
-    <t>NEED TO PURCHASE</t>
   </si>
   <si>
     <t>30-Ouput Flange</t>
@@ -912,10 +909,6 @@
 Purchase 1 pack for two 15:1 gearboxes</t>
   </si>
   <si>
-    <t xml:space="preserve"> ID 10mm x OD 15mm x 4mm (8 pcs)
-Purchase 2 packs for two 15:1 gearboxes</t>
-  </si>
-  <si>
     <t>ID 5mm x  OD 10mm x 4mm (30 pcs)
 Purchase 3 packs for two 15:1 gearboxes</t>
   </si>
@@ -924,9 +917,6 @@
 Need to 2x prints for two 15:1 gearboxes</t>
   </si>
   <si>
-    <t>SHIPPING COST WHEN ORDERED</t>
-  </si>
-  <si>
     <t>1.3.4</t>
   </si>
   <si>
@@ -1008,6 +998,10 @@
   <si>
     <t>1/3
 2/3</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ID 10mm x OD 15mm x 4mm (10 pcs)
+Purchase 1 pack for two 15:1 gearboxes</t>
   </si>
 </sst>
 </file>
@@ -1469,117 +1463,117 @@
     <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="44" fontId="10" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="14" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="10" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1875,9 +1869,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I67"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.85546875" customWidth="1"/>
+    <col min="1" max="1" width="45.88671875" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
@@ -1887,30 +1881,30 @@
     <col min="9" max="9" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="60" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="60"/>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="87"/>
+      <c r="F4" s="87"/>
+      <c r="G4" s="87"/>
+      <c r="H4" s="87"/>
+      <c r="I4" s="87"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1921,7 +1915,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
@@ -1932,7 +1926,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -1946,7 +1940,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
@@ -1960,7 +1954,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -1975,20 +1969,20 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="60" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="87" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="87"/>
+      <c r="C11" s="87"/>
+      <c r="D11" s="87"/>
+      <c r="E11" s="87"/>
+      <c r="F11" s="87"/>
+      <c r="G11" s="87"/>
+      <c r="H11" s="87"/>
+      <c r="I11" s="87"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
@@ -2002,7 +1996,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>16</v>
       </c>
@@ -2016,7 +2010,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -2030,7 +2024,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>20</v>
       </c>
@@ -2044,7 +2038,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>22</v>
       </c>
@@ -2058,7 +2052,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -2069,7 +2063,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>25</v>
       </c>
@@ -2083,20 +2077,20 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="60" t="s">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="60"/>
-      <c r="C20" s="60"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="60"/>
-      <c r="H20" s="60"/>
-      <c r="I20" s="60"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="87"/>
+      <c r="C20" s="87"/>
+      <c r="D20" s="87"/>
+      <c r="E20" s="87"/>
+      <c r="F20" s="87"/>
+      <c r="G20" s="87"/>
+      <c r="H20" s="87"/>
+      <c r="I20" s="87"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>28</v>
       </c>
@@ -2107,7 +2101,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>30</v>
       </c>
@@ -2118,20 +2112,20 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="60" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" s="87" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="60"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
-      <c r="H24" s="60"/>
-      <c r="I24" s="60"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="87"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="87"/>
+      <c r="E24" s="87"/>
+      <c r="F24" s="87"/>
+      <c r="G24" s="87"/>
+      <c r="H24" s="87"/>
+      <c r="I24" s="87"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>33</v>
       </c>
@@ -2145,7 +2139,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>36</v>
       </c>
@@ -2159,7 +2153,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>38</v>
       </c>
@@ -2173,7 +2167,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>41</v>
       </c>
@@ -2187,7 +2181,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>44</v>
       </c>
@@ -2201,7 +2195,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>47</v>
       </c>
@@ -2215,7 +2209,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>49</v>
       </c>
@@ -2229,7 +2223,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>51</v>
       </c>
@@ -2243,7 +2237,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>53</v>
       </c>
@@ -2257,7 +2251,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>55</v>
       </c>
@@ -2268,20 +2262,20 @@
         <v>42</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="60" t="s">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" s="87" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="60"/>
-      <c r="C36" s="60"/>
-      <c r="D36" s="60"/>
-      <c r="E36" s="60"/>
-      <c r="F36" s="60"/>
-      <c r="G36" s="60"/>
-      <c r="H36" s="60"/>
-      <c r="I36" s="60"/>
-    </row>
-    <row r="37" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B36" s="87"/>
+      <c r="C36" s="87"/>
+      <c r="D36" s="87"/>
+      <c r="E36" s="87"/>
+      <c r="F36" s="87"/>
+      <c r="G36" s="87"/>
+      <c r="H36" s="87"/>
+      <c r="I36" s="87"/>
+    </row>
+    <row r="37" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A37" s="12" t="s">
         <v>57</v>
       </c>
@@ -2302,7 +2296,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="13" t="s">
         <v>63</v>
       </c>
@@ -2325,7 +2319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="13" t="s">
         <v>65</v>
       </c>
@@ -2348,7 +2342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
         <v>66</v>
       </c>
@@ -2373,7 +2367,7 @@
         <v>3.5316E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="13" t="s">
         <v>67</v>
       </c>
@@ -2398,7 +2392,7 @@
         <v>4.7088000000000005E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="13" t="s">
         <v>68</v>
       </c>
@@ -2423,7 +2417,7 @@
         <v>0.34531200000000006</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="13" t="s">
         <v>69</v>
       </c>
@@ -2448,7 +2442,7 @@
         <v>0.29430000000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="13" t="s">
         <v>70</v>
       </c>
@@ -2473,7 +2467,7 @@
         <v>0.47088000000000002</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="17" t="s">
         <v>71</v>
       </c>
@@ -2489,20 +2483,20 @@
         <v>1.1928960000000002</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="60" t="s">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A47" s="87" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="60"/>
-      <c r="C47" s="60"/>
-      <c r="D47" s="60"/>
-      <c r="E47" s="60"/>
-      <c r="F47" s="60"/>
-      <c r="G47" s="60"/>
-      <c r="H47" s="60"/>
-      <c r="I47" s="60"/>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B47" s="87"/>
+      <c r="C47" s="87"/>
+      <c r="D47" s="87"/>
+      <c r="E47" s="87"/>
+      <c r="F47" s="87"/>
+      <c r="G47" s="87"/>
+      <c r="H47" s="87"/>
+      <c r="I47" s="87"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>73</v>
       </c>
@@ -2511,7 +2505,7 @@
         <v>5.8860000000000003E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>74</v>
       </c>
@@ -2520,7 +2514,7 @@
         <v>0.15696000000000002</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="21" t="s">
         <v>75</v>
       </c>
@@ -2532,20 +2526,20 @@
         <v>76</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="60" t="s">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A52" s="87" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="60"/>
-      <c r="C52" s="60"/>
-      <c r="D52" s="60"/>
-      <c r="E52" s="60"/>
-      <c r="F52" s="60"/>
-      <c r="G52" s="60"/>
-      <c r="H52" s="60"/>
-      <c r="I52" s="60"/>
-    </row>
-    <row r="53" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B52" s="87"/>
+      <c r="C52" s="87"/>
+      <c r="D52" s="87"/>
+      <c r="E52" s="87"/>
+      <c r="F52" s="87"/>
+      <c r="G52" s="87"/>
+      <c r="H52" s="87"/>
+      <c r="I52" s="87"/>
+    </row>
+    <row r="53" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
         <v>78</v>
       </c>
@@ -2574,7 +2568,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" s="13" t="s">
         <v>87</v>
       </c>
@@ -2610,7 +2604,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" s="13" t="s">
         <v>88</v>
       </c>
@@ -2647,7 +2641,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" s="13" t="s">
         <v>89</v>
       </c>
@@ -2684,7 +2678,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="13" t="s">
         <v>90</v>
       </c>
@@ -2717,7 +2711,7 @@
       </c>
       <c r="I57" s="13"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" s="13" t="s">
         <v>91</v>
       </c>
@@ -2750,7 +2744,7 @@
       </c>
       <c r="I58" s="13"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" s="13" t="s">
         <v>92</v>
       </c>
@@ -2782,37 +2776,37 @@
       </c>
       <c r="I59" s="13"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>99</v>
       </c>
@@ -2846,7 +2840,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -2856,17 +2850,17 @@
     <col min="6" max="6" width="56" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="27" t="s">
         <v>102</v>
       </c>
@@ -2886,7 +2880,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
         <v>108</v>
       </c>
@@ -2906,7 +2900,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="66" x14ac:dyDescent="0.3">
       <c r="A6" s="28" t="s">
         <v>114</v>
       </c>
@@ -2926,7 +2920,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="66" x14ac:dyDescent="0.3">
       <c r="A7" s="28" t="s">
         <v>120</v>
       </c>
@@ -2946,7 +2940,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="66" x14ac:dyDescent="0.3">
       <c r="A8" s="28" t="s">
         <v>126</v>
       </c>
@@ -2966,7 +2960,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="66" x14ac:dyDescent="0.3">
       <c r="A9" s="28" t="s">
         <v>132</v>
       </c>
@@ -2986,7 +2980,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>138</v>
       </c>
@@ -3006,7 +3000,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="66" x14ac:dyDescent="0.3">
       <c r="A11" s="28" t="s">
         <v>144</v>
       </c>
@@ -3026,7 +3020,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A12" s="28" t="s">
         <v>150</v>
       </c>
@@ -3046,7 +3040,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="66" x14ac:dyDescent="0.3">
       <c r="A13" s="28" t="s">
         <v>156</v>
       </c>
@@ -3066,7 +3060,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A14" s="28" t="s">
         <v>162</v>
       </c>
@@ -3095,23 +3089,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03C3DC63-880C-4C7A-BD99-15B2870A7881}">
   <dimension ref="A1:Q70"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="59.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="66.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="59.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="66.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="44" t="s">
         <v>102</v>
       </c>
@@ -3146,7 +3140,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="42" t="s">
         <v>108</v>
       </c>
@@ -3160,8 +3154,8 @@
         <v>1</v>
       </c>
       <c r="E2" s="41"/>
-      <c r="F2" s="63" t="s">
-        <v>286</v>
+      <c r="F2" s="52" t="s">
+        <v>285</v>
       </c>
       <c r="G2" s="42"/>
       <c r="H2" s="42"/>
@@ -3169,10 +3163,10 @@
       <c r="J2" s="41"/>
       <c r="K2" s="41">
         <f>K3+K11+K41</f>
-        <v>1336.03</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1333.81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="36" t="s">
         <v>207</v>
       </c>
@@ -3194,7 +3188,7 @@
         <v>1094.8399999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="33" t="s">
         <v>205</v>
       </c>
@@ -3219,8 +3213,8 @@
       <c r="H4" s="39">
         <v>46237</v>
       </c>
-      <c r="I4" s="86" t="s">
-        <v>319</v>
+      <c r="I4" s="60" t="s">
+        <v>316</v>
       </c>
       <c r="J4" s="32">
         <v>2.4424999999999999</v>
@@ -3230,7 +3224,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="33" t="s">
         <v>203</v>
       </c>
@@ -3255,8 +3249,8 @@
       <c r="H5" s="39">
         <v>46237</v>
       </c>
-      <c r="I5" s="86" t="s">
-        <v>319</v>
+      <c r="I5" s="60" t="s">
+        <v>316</v>
       </c>
       <c r="J5" s="32">
         <v>2.4424999999999999</v>
@@ -3266,7 +3260,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="33" t="s">
         <v>201</v>
       </c>
@@ -3291,8 +3285,8 @@
       <c r="H6" s="39">
         <v>46213</v>
       </c>
-      <c r="I6" s="86" t="s">
-        <v>318</v>
+      <c r="I6" s="60" t="s">
+        <v>315</v>
       </c>
       <c r="J6" s="32">
         <v>2.4424999999999999</v>
@@ -3302,7 +3296,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="33" t="s">
         <v>199</v>
       </c>
@@ -3324,11 +3318,11 @@
       <c r="G7" s="38" t="s">
         <v>176</v>
       </c>
-      <c r="H7" s="87" t="s">
+      <c r="H7" s="61" t="s">
+        <v>314</v>
+      </c>
+      <c r="I7" s="62" t="s">
         <v>317</v>
-      </c>
-      <c r="I7" s="88" t="s">
-        <v>320</v>
       </c>
       <c r="J7" s="32">
         <v>11.07</v>
@@ -3338,7 +3332,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="33"/>
       <c r="B8" s="33"/>
       <c r="C8" s="34"/>
@@ -3351,7 +3345,7 @@
       <c r="J8" s="32"/>
       <c r="K8" s="32"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="33" t="s">
         <v>197</v>
       </c>
@@ -3376,10 +3370,10 @@
       <c r="H9" s="39">
         <v>46213</v>
       </c>
-      <c r="I9" s="86" t="s">
-        <v>316</v>
-      </c>
-      <c r="J9" s="61">
+      <c r="I9" s="60" t="s">
+        <v>313</v>
+      </c>
+      <c r="J9" s="51">
         <v>30</v>
       </c>
       <c r="K9" s="32">
@@ -3387,7 +3381,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="33" t="s">
         <v>256</v>
       </c>
@@ -3412,8 +3406,8 @@
       <c r="H10" s="39">
         <v>46237</v>
       </c>
-      <c r="I10" s="86" t="s">
-        <v>316</v>
+      <c r="I10" s="60" t="s">
+        <v>313</v>
       </c>
       <c r="J10" s="32">
         <v>2.4424999999999999</v>
@@ -3423,7 +3417,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="36" t="s">
         <v>196</v>
       </c>
@@ -3449,7 +3443,7 @@
         <v>135.47999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="33" t="s">
         <v>194</v>
       </c>
@@ -3477,7 +3471,7 @@
       <c r="I12" s="33">
         <v>1</v>
       </c>
-      <c r="J12" s="51">
+      <c r="J12" s="63">
         <v>7.68</v>
       </c>
       <c r="K12" s="32">
@@ -3485,20 +3479,20 @@
         <v>7.21</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="78"/>
-      <c r="B13" s="78"/>
-      <c r="C13" s="79"/>
-      <c r="D13" s="78"/>
-      <c r="E13" s="80"/>
-      <c r="F13" s="78"/>
-      <c r="G13" s="78"/>
-      <c r="H13" s="83"/>
-      <c r="I13" s="78"/>
-      <c r="J13" s="82"/>
-      <c r="K13" s="80"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="54"/>
+      <c r="B13" s="54"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="56"/>
+      <c r="F13" s="54"/>
+      <c r="G13" s="54"/>
+      <c r="H13" s="58"/>
+      <c r="I13" s="54"/>
+      <c r="J13" s="85"/>
+      <c r="K13" s="56"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="33" t="s">
         <v>193</v>
       </c>
@@ -3526,13 +3520,13 @@
       <c r="I14" s="33">
         <v>3</v>
       </c>
-      <c r="J14" s="52"/>
+      <c r="J14" s="86"/>
       <c r="K14" s="32">
         <f>I14*E14</f>
         <v>38.97</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="33" t="s">
         <v>192</v>
       </c>
@@ -3560,13 +3554,13 @@
       <c r="I15" s="33">
         <v>1</v>
       </c>
-      <c r="J15" s="52"/>
+      <c r="J15" s="86"/>
       <c r="K15" s="32">
         <f t="shared" ref="K15:K25" si="0">I15*E15</f>
         <v>9.99</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="33" t="s">
         <v>191</v>
       </c>
@@ -3594,26 +3588,26 @@
       <c r="I16" s="33">
         <v>1</v>
       </c>
-      <c r="J16" s="52"/>
+      <c r="J16" s="86"/>
       <c r="K16" s="32">
         <f t="shared" si="0"/>
         <v>9.7899999999999991</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="78"/>
-      <c r="B17" s="78"/>
-      <c r="C17" s="79"/>
-      <c r="D17" s="78"/>
-      <c r="E17" s="80"/>
-      <c r="F17" s="78"/>
-      <c r="G17" s="78"/>
-      <c r="H17" s="78"/>
-      <c r="I17" s="78"/>
-      <c r="J17" s="82"/>
-      <c r="K17" s="80"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="54"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="55"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="54"/>
+      <c r="G17" s="54"/>
+      <c r="H17" s="54"/>
+      <c r="I17" s="54"/>
+      <c r="J17" s="85"/>
+      <c r="K17" s="56"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="33" t="s">
         <v>190</v>
       </c>
@@ -3641,13 +3635,13 @@
       <c r="I18" s="33">
         <v>1</v>
       </c>
-      <c r="J18" s="52"/>
+      <c r="J18" s="86"/>
       <c r="K18" s="32">
         <f t="shared" si="0"/>
         <v>6.99</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="33" t="s">
         <v>189</v>
       </c>
@@ -3675,26 +3669,26 @@
       <c r="I19" s="33">
         <v>1</v>
       </c>
-      <c r="J19" s="52"/>
+      <c r="J19" s="86"/>
       <c r="K19" s="32">
         <f t="shared" si="0"/>
         <v>8.99</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="78"/>
-      <c r="B20" s="78"/>
-      <c r="C20" s="79"/>
-      <c r="D20" s="78"/>
-      <c r="E20" s="80"/>
-      <c r="F20" s="78"/>
-      <c r="G20" s="78"/>
-      <c r="H20" s="78"/>
-      <c r="I20" s="78"/>
-      <c r="J20" s="82"/>
-      <c r="K20" s="80"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="54"/>
+      <c r="B20" s="54"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="54"/>
+      <c r="E20" s="56"/>
+      <c r="F20" s="54"/>
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="54"/>
+      <c r="J20" s="85"/>
+      <c r="K20" s="56"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="47" t="s">
         <v>188</v>
       </c>
@@ -3722,13 +3716,13 @@
       <c r="I21" s="33">
         <v>2</v>
       </c>
-      <c r="J21" s="52"/>
+      <c r="J21" s="86"/>
       <c r="K21" s="32">
         <f t="shared" si="0"/>
         <v>15.58</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="47" t="s">
         <v>187</v>
       </c>
@@ -3741,28 +3735,28 @@
       <c r="D22" s="33">
         <v>9</v>
       </c>
-      <c r="E22" s="51">
+      <c r="E22" s="63">
         <v>22.99</v>
       </c>
       <c r="F22" s="47" t="s">
         <v>247</v>
       </c>
-      <c r="G22" s="56" t="s">
+      <c r="G22" s="79" t="s">
         <v>176</v>
       </c>
-      <c r="H22" s="58">
+      <c r="H22" s="81">
         <v>46230</v>
       </c>
-      <c r="I22" s="54">
+      <c r="I22" s="83">
         <v>1</v>
       </c>
-      <c r="J22" s="52"/>
-      <c r="K22" s="51">
+      <c r="J22" s="86"/>
+      <c r="K22" s="63">
         <f t="shared" si="0"/>
         <v>22.99</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="47" t="s">
         <v>186</v>
       </c>
@@ -3775,17 +3769,17 @@
       <c r="D23" s="33">
         <v>7</v>
       </c>
-      <c r="E23" s="53"/>
+      <c r="E23" s="64"/>
       <c r="F23" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G23" s="57"/>
-      <c r="H23" s="59"/>
-      <c r="I23" s="55"/>
-      <c r="J23" s="52"/>
-      <c r="K23" s="53"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G23" s="80"/>
+      <c r="H23" s="82"/>
+      <c r="I23" s="84"/>
+      <c r="J23" s="86"/>
+      <c r="K23" s="64"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="47" t="s">
         <v>185</v>
       </c>
@@ -3807,10 +3801,10 @@
         <v>248</v>
       </c>
       <c r="I24" s="33"/>
-      <c r="J24" s="52"/>
+      <c r="J24" s="86"/>
       <c r="K24" s="32"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="47" t="s">
         <v>218</v>
       </c>
@@ -3838,13 +3832,13 @@
       <c r="I25" s="33">
         <v>1</v>
       </c>
-      <c r="J25" s="52"/>
+      <c r="J25" s="86"/>
       <c r="K25" s="32">
         <f t="shared" si="0"/>
         <v>7.29</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="47" t="s">
         <v>219</v>
       </c>
@@ -3870,23 +3864,23 @@
         <v>248</v>
       </c>
       <c r="I26" s="33"/>
-      <c r="J26" s="53"/>
+      <c r="J26" s="64"/>
       <c r="K26" s="32"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="78"/>
-      <c r="B27" s="78"/>
-      <c r="C27" s="79"/>
-      <c r="D27" s="78"/>
-      <c r="E27" s="80"/>
-      <c r="F27" s="81"/>
-      <c r="G27" s="78"/>
-      <c r="H27" s="78"/>
-      <c r="I27" s="78"/>
-      <c r="J27" s="80"/>
-      <c r="K27" s="80"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" s="54"/>
+      <c r="B27" s="54"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="54"/>
+      <c r="E27" s="56"/>
+      <c r="F27" s="57"/>
+      <c r="G27" s="54"/>
+      <c r="H27" s="54"/>
+      <c r="I27" s="54"/>
+      <c r="J27" s="56"/>
+      <c r="K27" s="56"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="33" t="s">
         <v>220</v>
       </c>
@@ -3894,22 +3888,22 @@
         <v>3</v>
       </c>
       <c r="C28" s="50" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D28" s="33">
         <v>1</v>
       </c>
       <c r="E28" s="32"/>
-      <c r="F28" s="64" t="s">
+      <c r="F28" s="65" t="s">
         <v>233</v>
       </c>
-      <c r="G28" s="65"/>
-      <c r="H28" s="65"/>
-      <c r="I28" s="65"/>
-      <c r="J28" s="65"/>
-      <c r="K28" s="66"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G28" s="66"/>
+      <c r="H28" s="66"/>
+      <c r="I28" s="66"/>
+      <c r="J28" s="66"/>
+      <c r="K28" s="67"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="33" t="s">
         <v>222</v>
       </c>
@@ -3917,20 +3911,20 @@
         <v>3</v>
       </c>
       <c r="C29" s="50" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D29" s="33">
         <v>1</v>
       </c>
       <c r="E29" s="32"/>
-      <c r="F29" s="67"/>
-      <c r="G29" s="68"/>
-      <c r="H29" s="68"/>
-      <c r="I29" s="68"/>
-      <c r="J29" s="68"/>
-      <c r="K29" s="69"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F29" s="68"/>
+      <c r="G29" s="69"/>
+      <c r="H29" s="69"/>
+      <c r="I29" s="69"/>
+      <c r="J29" s="69"/>
+      <c r="K29" s="70"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="33" t="s">
         <v>223</v>
       </c>
@@ -3938,20 +3932,20 @@
         <v>3</v>
       </c>
       <c r="C30" s="50" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D30" s="33">
         <v>78</v>
       </c>
       <c r="E30" s="32"/>
-      <c r="F30" s="67"/>
-      <c r="G30" s="68"/>
-      <c r="H30" s="68"/>
-      <c r="I30" s="68"/>
-      <c r="J30" s="68"/>
-      <c r="K30" s="69"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F30" s="68"/>
+      <c r="G30" s="69"/>
+      <c r="H30" s="69"/>
+      <c r="I30" s="69"/>
+      <c r="J30" s="69"/>
+      <c r="K30" s="70"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="33" t="s">
         <v>224</v>
       </c>
@@ -3959,20 +3953,20 @@
         <v>3</v>
       </c>
       <c r="C31" s="50" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D31" s="33">
         <v>39</v>
       </c>
       <c r="E31" s="32"/>
-      <c r="F31" s="67"/>
-      <c r="G31" s="68"/>
-      <c r="H31" s="68"/>
-      <c r="I31" s="68"/>
-      <c r="J31" s="68"/>
-      <c r="K31" s="69"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F31" s="68"/>
+      <c r="G31" s="69"/>
+      <c r="H31" s="69"/>
+      <c r="I31" s="69"/>
+      <c r="J31" s="69"/>
+      <c r="K31" s="70"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="33" t="s">
         <v>225</v>
       </c>
@@ -3980,20 +3974,20 @@
         <v>3</v>
       </c>
       <c r="C32" s="50" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D32" s="33">
         <v>2</v>
       </c>
       <c r="E32" s="32"/>
-      <c r="F32" s="67"/>
-      <c r="G32" s="68"/>
-      <c r="H32" s="68"/>
-      <c r="I32" s="68"/>
-      <c r="J32" s="68"/>
-      <c r="K32" s="69"/>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F32" s="68"/>
+      <c r="G32" s="69"/>
+      <c r="H32" s="69"/>
+      <c r="I32" s="69"/>
+      <c r="J32" s="69"/>
+      <c r="K32" s="70"/>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A33" s="33" t="s">
         <v>226</v>
       </c>
@@ -4001,20 +3995,20 @@
         <v>3</v>
       </c>
       <c r="C33" s="50" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D33" s="33">
         <v>2</v>
       </c>
       <c r="E33" s="32"/>
-      <c r="F33" s="67"/>
-      <c r="G33" s="68"/>
-      <c r="H33" s="68"/>
-      <c r="I33" s="68"/>
-      <c r="J33" s="68"/>
-      <c r="K33" s="69"/>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F33" s="68"/>
+      <c r="G33" s="69"/>
+      <c r="H33" s="69"/>
+      <c r="I33" s="69"/>
+      <c r="J33" s="69"/>
+      <c r="K33" s="70"/>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A34" s="33" t="s">
         <v>227</v>
       </c>
@@ -4022,20 +4016,20 @@
         <v>3</v>
       </c>
       <c r="C34" s="50" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D34" s="33">
         <v>1</v>
       </c>
       <c r="E34" s="32"/>
-      <c r="F34" s="67"/>
-      <c r="G34" s="68"/>
-      <c r="H34" s="68"/>
-      <c r="I34" s="68"/>
-      <c r="J34" s="68"/>
-      <c r="K34" s="69"/>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F34" s="68"/>
+      <c r="G34" s="69"/>
+      <c r="H34" s="69"/>
+      <c r="I34" s="69"/>
+      <c r="J34" s="69"/>
+      <c r="K34" s="70"/>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35" s="33" t="s">
         <v>228</v>
       </c>
@@ -4043,20 +4037,20 @@
         <v>3</v>
       </c>
       <c r="C35" s="50" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D35" s="33">
         <v>1</v>
       </c>
       <c r="E35" s="32"/>
-      <c r="F35" s="67"/>
-      <c r="G35" s="68"/>
-      <c r="H35" s="68"/>
-      <c r="I35" s="68"/>
-      <c r="J35" s="68"/>
-      <c r="K35" s="69"/>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F35" s="68"/>
+      <c r="G35" s="69"/>
+      <c r="H35" s="69"/>
+      <c r="I35" s="69"/>
+      <c r="J35" s="69"/>
+      <c r="K35" s="70"/>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36" s="33" t="s">
         <v>229</v>
       </c>
@@ -4064,20 +4058,20 @@
         <v>3</v>
       </c>
       <c r="C36" s="50" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D36" s="33">
         <v>1</v>
       </c>
       <c r="E36" s="32"/>
-      <c r="F36" s="67"/>
-      <c r="G36" s="68"/>
-      <c r="H36" s="68"/>
-      <c r="I36" s="68"/>
-      <c r="J36" s="68"/>
-      <c r="K36" s="69"/>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F36" s="68"/>
+      <c r="G36" s="69"/>
+      <c r="H36" s="69"/>
+      <c r="I36" s="69"/>
+      <c r="J36" s="69"/>
+      <c r="K36" s="70"/>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A37" s="33" t="s">
         <v>231</v>
       </c>
@@ -4085,21 +4079,21 @@
         <v>3</v>
       </c>
       <c r="C37" s="50" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D37" s="33">
         <v>1</v>
       </c>
       <c r="E37" s="32"/>
-      <c r="F37" s="67"/>
-      <c r="G37" s="68"/>
-      <c r="H37" s="68"/>
-      <c r="I37" s="68"/>
-      <c r="J37" s="68"/>
-      <c r="K37" s="69"/>
+      <c r="F37" s="68"/>
+      <c r="G37" s="69"/>
+      <c r="H37" s="69"/>
+      <c r="I37" s="69"/>
+      <c r="J37" s="69"/>
+      <c r="K37" s="70"/>
       <c r="Q37" s="48"/>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A38" s="33" t="s">
         <v>232</v>
       </c>
@@ -4107,20 +4101,20 @@
         <v>3</v>
       </c>
       <c r="C38" s="50" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D38" s="33">
         <v>1</v>
       </c>
       <c r="E38" s="32"/>
-      <c r="F38" s="67"/>
-      <c r="G38" s="68"/>
-      <c r="H38" s="68"/>
-      <c r="I38" s="68"/>
-      <c r="J38" s="68"/>
-      <c r="K38" s="69"/>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F38" s="68"/>
+      <c r="G38" s="69"/>
+      <c r="H38" s="69"/>
+      <c r="I38" s="69"/>
+      <c r="J38" s="69"/>
+      <c r="K38" s="70"/>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A39" s="33" t="s">
         <v>244</v>
       </c>
@@ -4128,20 +4122,20 @@
         <v>3</v>
       </c>
       <c r="C39" s="50" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D39" s="33">
         <v>1</v>
       </c>
       <c r="E39" s="32"/>
-      <c r="F39" s="67"/>
-      <c r="G39" s="68"/>
-      <c r="H39" s="68"/>
-      <c r="I39" s="68"/>
-      <c r="J39" s="68"/>
-      <c r="K39" s="69"/>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F39" s="68"/>
+      <c r="G39" s="69"/>
+      <c r="H39" s="69"/>
+      <c r="I39" s="69"/>
+      <c r="J39" s="69"/>
+      <c r="K39" s="70"/>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A40" s="33" t="s">
         <v>245</v>
       </c>
@@ -4149,20 +4143,20 @@
         <v>3</v>
       </c>
       <c r="C40" s="50" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D40" s="33">
         <v>1</v>
       </c>
       <c r="E40" s="32"/>
-      <c r="F40" s="70"/>
-      <c r="G40" s="71"/>
-      <c r="H40" s="71"/>
-      <c r="I40" s="71"/>
-      <c r="J40" s="71"/>
-      <c r="K40" s="72"/>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F40" s="71"/>
+      <c r="G40" s="72"/>
+      <c r="H40" s="72"/>
+      <c r="I40" s="72"/>
+      <c r="J40" s="72"/>
+      <c r="K40" s="73"/>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A41" s="36">
         <v>1.3</v>
       </c>
@@ -4185,10 +4179,10 @@
       <c r="J41" s="35"/>
       <c r="K41" s="35">
         <f>SUM(K42:K56)+SUM(J42:J56)</f>
-        <v>105.71</v>
-      </c>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+        <v>103.49</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A42" s="47" t="s">
         <v>184</v>
       </c>
@@ -4210,34 +4204,34 @@
       <c r="G42" s="45" t="s">
         <v>176</v>
       </c>
-      <c r="H42" s="62" t="s">
-        <v>261</v>
+      <c r="H42" s="88">
+        <v>46237</v>
       </c>
       <c r="I42" s="33">
         <v>1</v>
       </c>
-      <c r="J42" s="75" t="s">
-        <v>293</v>
+      <c r="J42" s="75">
+        <v>5.87</v>
       </c>
       <c r="K42" s="32">
         <f>I42*E42</f>
         <v>7.21</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A43" s="78"/>
-      <c r="B43" s="78"/>
-      <c r="C43" s="79"/>
-      <c r="D43" s="78"/>
-      <c r="E43" s="80"/>
-      <c r="F43" s="78"/>
-      <c r="G43" s="78"/>
-      <c r="H43" s="83"/>
-      <c r="I43" s="78"/>
-      <c r="J43" s="84"/>
-      <c r="K43" s="80"/>
-    </row>
-    <row r="44" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A43" s="54"/>
+      <c r="B43" s="54"/>
+      <c r="C43" s="55"/>
+      <c r="D43" s="54"/>
+      <c r="E43" s="56"/>
+      <c r="F43" s="54"/>
+      <c r="G43" s="54"/>
+      <c r="H43" s="58"/>
+      <c r="I43" s="54"/>
+      <c r="J43" s="76"/>
+      <c r="K43" s="56"/>
+    </row>
+    <row r="44" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="47" t="s">
         <v>182</v>
       </c>
@@ -4253,25 +4247,25 @@
       <c r="E44" s="32">
         <v>12.99</v>
       </c>
-      <c r="F44" s="73" t="s">
-        <v>291</v>
+      <c r="F44" s="53" t="s">
+        <v>289</v>
       </c>
       <c r="G44" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="H44" s="62" t="s">
-        <v>261</v>
+      <c r="H44" s="88">
+        <v>46237</v>
       </c>
       <c r="I44" s="33">
         <v>3</v>
       </c>
-      <c r="J44" s="76"/>
+      <c r="J44" s="77"/>
       <c r="K44" s="32">
         <f>I44*E44</f>
         <v>38.97</v>
       </c>
     </row>
-    <row r="45" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="47" t="s">
         <v>179</v>
       </c>
@@ -4287,27 +4281,27 @@
       <c r="E45" s="32">
         <v>8.09</v>
       </c>
-      <c r="F45" s="73" t="s">
-        <v>290</v>
+      <c r="F45" s="53" t="s">
+        <v>318</v>
       </c>
       <c r="G45" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="H45" s="62" t="s">
-        <v>261</v>
+      <c r="H45" s="88">
+        <v>46237</v>
       </c>
       <c r="I45" s="33">
-        <v>2</v>
-      </c>
-      <c r="J45" s="76"/>
+        <v>1</v>
+      </c>
+      <c r="J45" s="77"/>
       <c r="K45" s="32">
-        <f t="shared" ref="K45:K55" si="1">I45*E45</f>
-        <v>16.18</v>
-      </c>
-    </row>
-    <row r="46" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" ref="K45:K46" si="1">I45*E45</f>
+        <v>8.09</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46" s="47" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="B46" s="33">
         <v>3</v>
@@ -4321,40 +4315,40 @@
       <c r="E46" s="32">
         <v>9.99</v>
       </c>
-      <c r="F46" s="73" t="s">
-        <v>289</v>
+      <c r="F46" s="53" t="s">
+        <v>288</v>
       </c>
       <c r="G46" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="H46" s="62" t="s">
-        <v>261</v>
+      <c r="H46" s="88">
+        <v>46237</v>
       </c>
       <c r="I46" s="33">
         <v>1</v>
       </c>
-      <c r="J46" s="76"/>
+      <c r="J46" s="77"/>
       <c r="K46" s="32">
         <f t="shared" si="1"/>
         <v>9.99</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A47" s="78"/>
-      <c r="B47" s="78"/>
-      <c r="C47" s="79"/>
-      <c r="D47" s="78"/>
-      <c r="E47" s="80"/>
-      <c r="F47" s="78"/>
-      <c r="G47" s="78"/>
-      <c r="H47" s="78"/>
-      <c r="I47" s="78"/>
-      <c r="J47" s="84"/>
-      <c r="K47" s="80"/>
-    </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A47" s="54"/>
+      <c r="B47" s="54"/>
+      <c r="C47" s="55"/>
+      <c r="D47" s="54"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="54"/>
+      <c r="G47" s="54"/>
+      <c r="H47" s="54"/>
+      <c r="I47" s="54"/>
+      <c r="J47" s="76"/>
+      <c r="K47" s="56"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A48" s="47" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B48" s="33">
         <v>3</v>
@@ -4378,15 +4372,15 @@
         <v>259</v>
       </c>
       <c r="I48" s="33"/>
-      <c r="J48" s="76"/>
+      <c r="J48" s="77"/>
       <c r="K48" s="32">
-        <f t="shared" ref="K48:K58" si="2">I48*E48</f>
+        <f t="shared" ref="K48:K55" si="2">I48*E48</f>
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A49" s="47" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B49" s="33">
         <v>3</v>
@@ -4410,28 +4404,28 @@
         <v>259</v>
       </c>
       <c r="I49" s="33"/>
-      <c r="J49" s="76"/>
+      <c r="J49" s="77"/>
       <c r="K49" s="32">
         <f>I49*E49</f>
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A50" s="85"/>
-      <c r="B50" s="78"/>
-      <c r="C50" s="79"/>
-      <c r="D50" s="78"/>
-      <c r="E50" s="80"/>
-      <c r="F50" s="78"/>
-      <c r="G50" s="78"/>
-      <c r="H50" s="78"/>
-      <c r="I50" s="78"/>
-      <c r="J50" s="84"/>
-      <c r="K50" s="80"/>
-    </row>
-    <row r="51" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A50" s="59"/>
+      <c r="B50" s="54"/>
+      <c r="C50" s="55"/>
+      <c r="D50" s="54"/>
+      <c r="E50" s="56"/>
+      <c r="F50" s="54"/>
+      <c r="G50" s="54"/>
+      <c r="H50" s="54"/>
+      <c r="I50" s="54"/>
+      <c r="J50" s="76"/>
+      <c r="K50" s="56"/>
+    </row>
+    <row r="51" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="47" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B51" s="33">
         <v>3</v>
@@ -4445,28 +4439,28 @@
       <c r="E51" s="32">
         <v>7.79</v>
       </c>
-      <c r="F51" s="73" t="s">
-        <v>288</v>
+      <c r="F51" s="53" t="s">
+        <v>287</v>
       </c>
       <c r="G51" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="H51" s="62" t="s">
-        <v>261</v>
+      <c r="H51" s="88">
+        <v>46237</v>
       </c>
       <c r="I51" s="33">
         <v>3</v>
       </c>
-      <c r="J51" s="76"/>
+      <c r="J51" s="77"/>
       <c r="K51" s="32">
-        <f t="shared" ref="K51:K61" si="3">I51*E51</f>
+        <f t="shared" ref="K51:K52" si="3">I51*E51</f>
         <v>23.37</v>
       </c>
       <c r="Q51" s="31"/>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A52" s="47" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B52" s="33">
         <v>3</v>
@@ -4477,28 +4471,28 @@
       <c r="D52" s="33">
         <v>9</v>
       </c>
-      <c r="E52" s="51">
+      <c r="E52" s="63">
         <v>22.99</v>
       </c>
       <c r="F52" s="47" t="s">
         <v>260</v>
       </c>
-      <c r="G52" s="56" t="s">
+      <c r="G52" s="79" t="s">
         <v>176</v>
       </c>
-      <c r="H52" s="58" t="s">
+      <c r="H52" s="81" t="s">
         <v>259</v>
       </c>
-      <c r="I52" s="54"/>
-      <c r="J52" s="76"/>
-      <c r="K52" s="51">
+      <c r="I52" s="83"/>
+      <c r="J52" s="77"/>
+      <c r="K52" s="63">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A53" s="47" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B53" s="33">
         <v>3</v>
@@ -4509,19 +4503,19 @@
       <c r="D53" s="33">
         <v>7</v>
       </c>
-      <c r="E53" s="53"/>
+      <c r="E53" s="64"/>
       <c r="F53" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G53" s="57"/>
-      <c r="H53" s="59"/>
-      <c r="I53" s="55"/>
-      <c r="J53" s="76"/>
-      <c r="K53" s="53"/>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="G53" s="80"/>
+      <c r="H53" s="82"/>
+      <c r="I53" s="84"/>
+      <c r="J53" s="77"/>
+      <c r="K53" s="64"/>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A54" s="47" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B54" s="33">
         <v>3</v>
@@ -4541,21 +4535,21 @@
       <c r="G54" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="H54" s="62" t="s">
-        <v>261</v>
+      <c r="H54" s="88">
+        <v>46237</v>
       </c>
       <c r="I54" s="33">
         <v>1</v>
       </c>
-      <c r="J54" s="76"/>
+      <c r="J54" s="77"/>
       <c r="K54" s="32">
         <f>I54*E54</f>
         <v>9.99</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A55" s="47" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="B55" s="33">
         <v>3</v>
@@ -4579,15 +4573,15 @@
         <v>258</v>
       </c>
       <c r="I55" s="47"/>
-      <c r="J55" s="76"/>
+      <c r="J55" s="77"/>
       <c r="K55" s="32">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A56" s="47" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B56" s="33">
         <v>3</v>
@@ -4602,7 +4596,7 @@
         <v>21.45</v>
       </c>
       <c r="F56" s="47" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G56" s="46" t="s">
         <v>176</v>
@@ -4611,299 +4605,305 @@
         <v>248</v>
       </c>
       <c r="I56" s="33"/>
-      <c r="J56" s="77"/>
+      <c r="J56" s="78"/>
       <c r="K56" s="32"/>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A57" s="78"/>
-      <c r="B57" s="78"/>
-      <c r="C57" s="79"/>
-      <c r="D57" s="78"/>
-      <c r="E57" s="80"/>
-      <c r="F57" s="81"/>
-      <c r="G57" s="78"/>
-      <c r="H57" s="78"/>
-      <c r="I57" s="78"/>
-      <c r="J57" s="80"/>
-      <c r="K57" s="80"/>
-    </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A57" s="54"/>
+      <c r="B57" s="54"/>
+      <c r="C57" s="55"/>
+      <c r="D57" s="54"/>
+      <c r="E57" s="56"/>
+      <c r="F57" s="57"/>
+      <c r="G57" s="54"/>
+      <c r="H57" s="54"/>
+      <c r="I57" s="54"/>
+      <c r="J57" s="56"/>
+      <c r="K57" s="56"/>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A58" s="47" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B58" s="33">
         <v>3</v>
       </c>
       <c r="C58" s="50" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D58" s="33">
         <v>1</v>
       </c>
       <c r="E58" s="32"/>
       <c r="F58" s="74" t="s">
-        <v>292</v>
-      </c>
-      <c r="G58" s="65"/>
-      <c r="H58" s="65"/>
-      <c r="I58" s="65"/>
-      <c r="J58" s="65"/>
-      <c r="K58" s="66"/>
-    </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
+        <v>290</v>
+      </c>
+      <c r="G58" s="66"/>
+      <c r="H58" s="66"/>
+      <c r="I58" s="66"/>
+      <c r="J58" s="66"/>
+      <c r="K58" s="67"/>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A59" s="47" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B59" s="33">
         <v>3</v>
       </c>
       <c r="C59" s="50" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D59" s="33">
         <v>1</v>
       </c>
       <c r="E59" s="32"/>
-      <c r="F59" s="67"/>
-      <c r="G59" s="68"/>
-      <c r="H59" s="68"/>
-      <c r="I59" s="68"/>
-      <c r="J59" s="68"/>
-      <c r="K59" s="69"/>
-    </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F59" s="68"/>
+      <c r="G59" s="69"/>
+      <c r="H59" s="69"/>
+      <c r="I59" s="69"/>
+      <c r="J59" s="69"/>
+      <c r="K59" s="70"/>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A60" s="47" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B60" s="33">
         <v>3</v>
       </c>
       <c r="C60" s="50" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D60" s="33">
         <v>44</v>
       </c>
       <c r="E60" s="32"/>
-      <c r="F60" s="67"/>
-      <c r="G60" s="68"/>
-      <c r="H60" s="68"/>
-      <c r="I60" s="68"/>
-      <c r="J60" s="68"/>
-      <c r="K60" s="69"/>
-    </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F60" s="68"/>
+      <c r="G60" s="69"/>
+      <c r="H60" s="69"/>
+      <c r="I60" s="69"/>
+      <c r="J60" s="69"/>
+      <c r="K60" s="70"/>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A61" s="47" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B61" s="33">
         <v>3</v>
       </c>
       <c r="C61" s="50" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D61" s="33">
         <v>22</v>
       </c>
       <c r="E61" s="32"/>
-      <c r="F61" s="67"/>
-      <c r="G61" s="68"/>
-      <c r="H61" s="68"/>
-      <c r="I61" s="68"/>
-      <c r="J61" s="68"/>
-      <c r="K61" s="69"/>
-    </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F61" s="68"/>
+      <c r="G61" s="69"/>
+      <c r="H61" s="69"/>
+      <c r="I61" s="69"/>
+      <c r="J61" s="69"/>
+      <c r="K61" s="70"/>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A62" s="47" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="B62" s="33">
         <v>3</v>
       </c>
       <c r="C62" s="50" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D62" s="33">
         <v>2</v>
       </c>
       <c r="E62" s="32"/>
-      <c r="F62" s="67"/>
-      <c r="G62" s="68"/>
-      <c r="H62" s="68"/>
-      <c r="I62" s="68"/>
-      <c r="J62" s="68"/>
-      <c r="K62" s="69"/>
-    </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F62" s="68"/>
+      <c r="G62" s="69"/>
+      <c r="H62" s="69"/>
+      <c r="I62" s="69"/>
+      <c r="J62" s="69"/>
+      <c r="K62" s="70"/>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A63" s="47" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B63" s="33">
         <v>3</v>
       </c>
       <c r="C63" s="50" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D63" s="33">
         <v>2</v>
       </c>
       <c r="E63" s="32"/>
-      <c r="F63" s="67"/>
-      <c r="G63" s="68"/>
-      <c r="H63" s="68"/>
-      <c r="I63" s="68"/>
-      <c r="J63" s="68"/>
-      <c r="K63" s="69"/>
-    </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F63" s="68"/>
+      <c r="G63" s="69"/>
+      <c r="H63" s="69"/>
+      <c r="I63" s="69"/>
+      <c r="J63" s="69"/>
+      <c r="K63" s="70"/>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A64" s="47" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B64" s="33">
         <v>3</v>
       </c>
       <c r="C64" s="50" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D64" s="33">
         <v>1</v>
       </c>
       <c r="E64" s="32"/>
-      <c r="F64" s="67"/>
-      <c r="G64" s="68"/>
-      <c r="H64" s="68"/>
-      <c r="I64" s="68"/>
-      <c r="J64" s="68"/>
-      <c r="K64" s="69"/>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F64" s="68"/>
+      <c r="G64" s="69"/>
+      <c r="H64" s="69"/>
+      <c r="I64" s="69"/>
+      <c r="J64" s="69"/>
+      <c r="K64" s="70"/>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65" s="47" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B65" s="33">
         <v>3</v>
       </c>
       <c r="C65" s="50" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D65" s="33">
         <v>1</v>
       </c>
       <c r="E65" s="32"/>
-      <c r="F65" s="67"/>
-      <c r="G65" s="68"/>
-      <c r="H65" s="68"/>
-      <c r="I65" s="68"/>
-      <c r="J65" s="68"/>
-      <c r="K65" s="69"/>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F65" s="68"/>
+      <c r="G65" s="69"/>
+      <c r="H65" s="69"/>
+      <c r="I65" s="69"/>
+      <c r="J65" s="69"/>
+      <c r="K65" s="70"/>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66" s="47" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B66" s="33">
         <v>3</v>
       </c>
       <c r="C66" s="50" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D66" s="33">
         <v>1</v>
       </c>
       <c r="E66" s="32"/>
-      <c r="F66" s="67"/>
-      <c r="G66" s="68"/>
-      <c r="H66" s="68"/>
-      <c r="I66" s="68"/>
-      <c r="J66" s="68"/>
-      <c r="K66" s="69"/>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F66" s="68"/>
+      <c r="G66" s="69"/>
+      <c r="H66" s="69"/>
+      <c r="I66" s="69"/>
+      <c r="J66" s="69"/>
+      <c r="K66" s="70"/>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67" s="47" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B67" s="33">
         <v>3</v>
       </c>
       <c r="C67" s="50" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D67" s="33">
         <v>1</v>
       </c>
       <c r="E67" s="32"/>
-      <c r="F67" s="67"/>
-      <c r="G67" s="68"/>
-      <c r="H67" s="68"/>
-      <c r="I67" s="68"/>
-      <c r="J67" s="68"/>
-      <c r="K67" s="69"/>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F67" s="68"/>
+      <c r="G67" s="69"/>
+      <c r="H67" s="69"/>
+      <c r="I67" s="69"/>
+      <c r="J67" s="69"/>
+      <c r="K67" s="70"/>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68" s="47" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="B68" s="33">
         <v>3</v>
       </c>
       <c r="C68" s="50" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D68" s="33">
         <v>1</v>
       </c>
       <c r="E68" s="32"/>
-      <c r="F68" s="67"/>
-      <c r="G68" s="68"/>
-      <c r="H68" s="68"/>
-      <c r="I68" s="68"/>
-      <c r="J68" s="68"/>
-      <c r="K68" s="69"/>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F68" s="68"/>
+      <c r="G68" s="69"/>
+      <c r="H68" s="69"/>
+      <c r="I68" s="69"/>
+      <c r="J68" s="69"/>
+      <c r="K68" s="70"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69" s="47" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B69" s="33">
         <v>3</v>
       </c>
       <c r="C69" s="50" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D69" s="33">
         <v>1</v>
       </c>
       <c r="E69" s="32"/>
-      <c r="F69" s="67"/>
-      <c r="G69" s="68"/>
-      <c r="H69" s="68"/>
-      <c r="I69" s="68"/>
-      <c r="J69" s="68"/>
-      <c r="K69" s="69"/>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F69" s="68"/>
+      <c r="G69" s="69"/>
+      <c r="H69" s="69"/>
+      <c r="I69" s="69"/>
+      <c r="J69" s="69"/>
+      <c r="K69" s="70"/>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70" s="47" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="B70" s="33">
         <v>3</v>
       </c>
       <c r="C70" s="50" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D70" s="33">
         <v>1</v>
       </c>
       <c r="E70" s="32"/>
-      <c r="F70" s="67"/>
-      <c r="G70" s="68"/>
-      <c r="H70" s="68"/>
-      <c r="I70" s="68"/>
-      <c r="J70" s="68"/>
-      <c r="K70" s="69"/>
+      <c r="F70" s="68"/>
+      <c r="G70" s="69"/>
+      <c r="H70" s="69"/>
+      <c r="I70" s="69"/>
+      <c r="J70" s="69"/>
+      <c r="K70" s="70"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="J12:J26"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="E22:E23"/>
     <mergeCell ref="K52:K53"/>
     <mergeCell ref="F28:K40"/>
     <mergeCell ref="F58:K70"/>
@@ -4912,12 +4912,6 @@
     <mergeCell ref="G52:G53"/>
     <mergeCell ref="H52:H53"/>
     <mergeCell ref="I52:I53"/>
-    <mergeCell ref="J12:J26"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="K22:K23"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <hyperlinks>
@@ -4935,16 +4929,16 @@
     <hyperlink ref="G26" r:id="rId12" xr:uid="{DEBF1BA2-46DF-49AD-9E35-D39C010E82A9}"/>
     <hyperlink ref="G21" r:id="rId13" xr:uid="{1412C55E-6A1A-4053-A18E-D6A0EE5D9AF0}"/>
     <hyperlink ref="G10" r:id="rId14" xr:uid="{BB939D89-68F1-407A-8961-161DEA665F6A}"/>
-    <hyperlink ref="G46" r:id="rId15" xr:uid="{B027617C-3F89-419E-A842-31851D15B3A1}"/>
-    <hyperlink ref="G48" r:id="rId16" xr:uid="{CF4E87A8-2CD6-44E7-B022-0B1B179E9C9B}"/>
-    <hyperlink ref="G49" r:id="rId17" xr:uid="{E7EE2972-5E2C-4E50-B232-CF0017396C34}"/>
-    <hyperlink ref="G44" r:id="rId18" xr:uid="{3BE946ED-0C3E-4843-8774-E4F93E18E598}"/>
-    <hyperlink ref="G42" r:id="rId19" xr:uid="{F408121A-1D17-44CD-9FA6-54DD50AB9900}"/>
-    <hyperlink ref="G55" r:id="rId20" xr:uid="{FEA4F571-F1A3-49CD-8ADA-35A12B26F775}"/>
-    <hyperlink ref="G56" r:id="rId21" xr:uid="{F758FAF3-7978-4F47-B4FF-CA876A9FFDA1}"/>
-    <hyperlink ref="G45" r:id="rId22" xr:uid="{5E52BE69-7A7F-4A75-A558-F821970562D3}"/>
-    <hyperlink ref="G51" r:id="rId23" xr:uid="{181C5DE6-9473-4241-B12C-D25DC1804061}"/>
-    <hyperlink ref="G54" r:id="rId24" xr:uid="{19AC5AEB-C68E-4393-AAB8-3C0E0C06A444}"/>
+    <hyperlink ref="G48" r:id="rId15" xr:uid="{CF4E87A8-2CD6-44E7-B022-0B1B179E9C9B}"/>
+    <hyperlink ref="G49" r:id="rId16" xr:uid="{E7EE2972-5E2C-4E50-B232-CF0017396C34}"/>
+    <hyperlink ref="G44" r:id="rId17" xr:uid="{3BE946ED-0C3E-4843-8774-E4F93E18E598}"/>
+    <hyperlink ref="G42" r:id="rId18" xr:uid="{F408121A-1D17-44CD-9FA6-54DD50AB9900}"/>
+    <hyperlink ref="G55" r:id="rId19" xr:uid="{FEA4F571-F1A3-49CD-8ADA-35A12B26F775}"/>
+    <hyperlink ref="G56" r:id="rId20" xr:uid="{F758FAF3-7978-4F47-B4FF-CA876A9FFDA1}"/>
+    <hyperlink ref="G45" r:id="rId21" xr:uid="{5E52BE69-7A7F-4A75-A558-F821970562D3}"/>
+    <hyperlink ref="G51" r:id="rId22" xr:uid="{181C5DE6-9473-4241-B12C-D25DC1804061}"/>
+    <hyperlink ref="G54" r:id="rId23" xr:uid="{19AC5AEB-C68E-4393-AAB8-3C0E0C06A444}"/>
+    <hyperlink ref="G46" r:id="rId24" xr:uid="{B027617C-3F89-419E-A842-31851D15B3A1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId25"/>

</xml_diff>

<commit_message>
Starting 6-DOF arm assembly
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADBA8DFD-6C6E-4C1A-AA6F-0940B37E4555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1230963E-BD47-49E0-B776-60988303A4C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Torque Budget" sheetId="1" r:id="rId1"/>
@@ -1014,7 +1014,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1125,6 +1125,12 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1345,7 +1351,7 @@
     <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1499,10 +1505,39 @@
     <xf numFmtId="49" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1546,34 +1581,6 @@
     </xf>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1869,9 +1876,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I67"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.88671875" customWidth="1"/>
+    <col min="1" max="1" width="45.85546875" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
@@ -1881,30 +1888,30 @@
     <col min="9" max="9" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="87" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="87"/>
-      <c r="C4" s="87"/>
-      <c r="D4" s="87"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B4" s="65"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1915,7 +1922,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
@@ -1926,7 +1933,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -1940,7 +1947,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
@@ -1954,7 +1961,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -1969,25 +1976,25 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="87" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="87"/>
-      <c r="C11" s="87"/>
-      <c r="D11" s="87"/>
-      <c r="E11" s="87"/>
-      <c r="F11" s="87"/>
-      <c r="G11" s="87"/>
-      <c r="H11" s="87"/>
-      <c r="I11" s="87"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="65"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="65"/>
+      <c r="I11" s="65"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="4">
-        <v>0.35</v>
+        <v>0.9</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>14</v>
@@ -1996,7 +2003,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>16</v>
       </c>
@@ -2010,7 +2017,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -2024,7 +2031,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>20</v>
       </c>
@@ -2038,7 +2045,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>22</v>
       </c>
@@ -2052,7 +2059,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -2063,7 +2070,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>25</v>
       </c>
@@ -2077,20 +2084,20 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="87" t="s">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="87"/>
-      <c r="C20" s="87"/>
-      <c r="D20" s="87"/>
-      <c r="E20" s="87"/>
-      <c r="F20" s="87"/>
-      <c r="G20" s="87"/>
-      <c r="H20" s="87"/>
-      <c r="I20" s="87"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B20" s="65"/>
+      <c r="C20" s="65"/>
+      <c r="D20" s="65"/>
+      <c r="E20" s="65"/>
+      <c r="F20" s="65"/>
+      <c r="G20" s="65"/>
+      <c r="H20" s="65"/>
+      <c r="I20" s="65"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>28</v>
       </c>
@@ -2101,7 +2108,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>30</v>
       </c>
@@ -2112,20 +2119,20 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="87" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="65" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="87"/>
-      <c r="C24" s="87"/>
-      <c r="D24" s="87"/>
-      <c r="E24" s="87"/>
-      <c r="F24" s="87"/>
-      <c r="G24" s="87"/>
-      <c r="H24" s="87"/>
-      <c r="I24" s="87"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B24" s="65"/>
+      <c r="C24" s="65"/>
+      <c r="D24" s="65"/>
+      <c r="E24" s="65"/>
+      <c r="F24" s="65"/>
+      <c r="G24" s="65"/>
+      <c r="H24" s="65"/>
+      <c r="I24" s="65"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>33</v>
       </c>
@@ -2139,7 +2146,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>36</v>
       </c>
@@ -2153,7 +2160,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>38</v>
       </c>
@@ -2167,7 +2174,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>41</v>
       </c>
@@ -2181,7 +2188,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>44</v>
       </c>
@@ -2195,7 +2202,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>47</v>
       </c>
@@ -2209,11 +2216,11 @@
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="64">
         <v>15</v>
       </c>
       <c r="C31" s="3" t="s">
@@ -2223,7 +2230,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>51</v>
       </c>
@@ -2237,12 +2244,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>53</v>
       </c>
       <c r="B33" s="9">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>45</v>
@@ -2251,7 +2258,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>55</v>
       </c>
@@ -2262,20 +2269,20 @@
         <v>42</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="87" t="s">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="65" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="87"/>
-      <c r="C36" s="87"/>
-      <c r="D36" s="87"/>
-      <c r="E36" s="87"/>
-      <c r="F36" s="87"/>
-      <c r="G36" s="87"/>
-      <c r="H36" s="87"/>
-      <c r="I36" s="87"/>
-    </row>
-    <row r="37" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B36" s="65"/>
+      <c r="C36" s="65"/>
+      <c r="D36" s="65"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="65"/>
+      <c r="G36" s="65"/>
+      <c r="H36" s="65"/>
+      <c r="I36" s="65"/>
+    </row>
+    <row r="37" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
         <v>57</v>
       </c>
@@ -2296,7 +2303,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
         <v>63</v>
       </c>
@@ -2319,13 +2326,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
         <v>65</v>
       </c>
       <c r="B39" s="14">
         <f>B12</f>
-        <v>0.35</v>
+        <v>0.9</v>
       </c>
       <c r="D39" s="14">
         <f>B5</f>
@@ -2335,14 +2342,14 @@
         <v>64</v>
       </c>
       <c r="F39" s="16">
-        <f t="shared" si="0"/>
-        <v>0.54935999999999996</v>
+        <f>B39*$B$21*D39</f>
+        <v>1.4126400000000001</v>
       </c>
       <c r="G39" s="16">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
         <v>66</v>
       </c>
@@ -2367,7 +2374,7 @@
         <v>3.5316E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
         <v>67</v>
       </c>
@@ -2392,7 +2399,7 @@
         <v>4.7088000000000005E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
         <v>68</v>
       </c>
@@ -2417,7 +2424,7 @@
         <v>0.34531200000000006</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
         <v>69</v>
       </c>
@@ -2442,7 +2449,7 @@
         <v>0.29430000000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
         <v>70</v>
       </c>
@@ -2467,7 +2474,7 @@
         <v>0.47088000000000002</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="17" t="s">
         <v>71</v>
       </c>
@@ -2476,27 +2483,27 @@
       <c r="E45" s="18"/>
       <c r="F45" s="19">
         <f>SUM(F38:F44)</f>
-        <v>2.9665440000000003</v>
+        <v>3.8298240000000003</v>
       </c>
       <c r="G45" s="19">
         <f>SUM(G38:G44)</f>
         <v>1.1928960000000002</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" s="87" t="s">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="65" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="87"/>
-      <c r="C47" s="87"/>
-      <c r="D47" s="87"/>
-      <c r="E47" s="87"/>
-      <c r="F47" s="87"/>
-      <c r="G47" s="87"/>
-      <c r="H47" s="87"/>
-      <c r="I47" s="87"/>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B47" s="65"/>
+      <c r="C47" s="65"/>
+      <c r="D47" s="65"/>
+      <c r="E47" s="65"/>
+      <c r="F47" s="65"/>
+      <c r="G47" s="65"/>
+      <c r="H47" s="65"/>
+      <c r="I47" s="65"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>73</v>
       </c>
@@ -2505,7 +2512,7 @@
         <v>5.8860000000000003E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>74</v>
       </c>
@@ -2514,7 +2521,7 @@
         <v>0.15696000000000002</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="21" t="s">
         <v>75</v>
       </c>
@@ -2526,20 +2533,20 @@
         <v>76</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A52" s="87" t="s">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="87"/>
-      <c r="C52" s="87"/>
-      <c r="D52" s="87"/>
-      <c r="E52" s="87"/>
-      <c r="F52" s="87"/>
-      <c r="G52" s="87"/>
-      <c r="H52" s="87"/>
-      <c r="I52" s="87"/>
-    </row>
-    <row r="53" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B52" s="65"/>
+      <c r="C52" s="65"/>
+      <c r="D52" s="65"/>
+      <c r="E52" s="65"/>
+      <c r="F52" s="65"/>
+      <c r="G52" s="65"/>
+      <c r="H52" s="65"/>
+      <c r="I52" s="65"/>
+    </row>
+    <row r="53" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
         <v>78</v>
       </c>
@@ -2568,7 +2575,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="13" t="s">
         <v>87</v>
       </c>
@@ -2604,17 +2611,17 @@
         <v>96</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
         <v>88</v>
       </c>
       <c r="B55" s="16">
         <f>F45</f>
-        <v>2.9665440000000003</v>
+        <v>3.8298240000000003</v>
       </c>
       <c r="C55" s="16">
         <f t="shared" si="1"/>
-        <v>4.4498160000000002</v>
+        <v>5.7447360000000005</v>
       </c>
       <c r="D55" s="24">
         <f>B30</f>
@@ -2626,11 +2633,11 @@
       </c>
       <c r="F55" s="16">
         <f t="shared" si="2"/>
-        <v>1.2135333236250665</v>
+        <v>0.9399909760866294</v>
       </c>
       <c r="G55" s="25" t="str">
         <f t="shared" si="3"/>
-        <v>PASS</v>
+        <v>MARGINAL</v>
       </c>
       <c r="H55" s="26">
         <f>B26*B30*B28</f>
@@ -2641,7 +2648,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="13" t="s">
         <v>89</v>
       </c>
@@ -2678,7 +2685,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="13" t="s">
         <v>90</v>
       </c>
@@ -2692,15 +2699,15 @@
       </c>
       <c r="D57" s="24">
         <f>B33</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E57" s="16">
         <f>B32*B33*B34</f>
-        <v>0.85</v>
+        <v>1.36</v>
       </c>
       <c r="F57" s="16">
         <f t="shared" si="2"/>
-        <v>2.6256448274796895</v>
+        <v>4.2010317239675041</v>
       </c>
       <c r="G57" s="25" t="str">
         <f t="shared" si="3"/>
@@ -2711,7 +2718,7 @@
       </c>
       <c r="I57" s="13"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="13" t="s">
         <v>91</v>
       </c>
@@ -2725,15 +2732,15 @@
       </c>
       <c r="D58" s="24">
         <f>B33</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E58" s="16">
         <f>B32*B33*B34</f>
-        <v>0.85</v>
+        <v>1.36</v>
       </c>
       <c r="F58" s="16">
         <f t="shared" si="2"/>
-        <v>2.6256448274796895</v>
+        <v>4.2010317239675041</v>
       </c>
       <c r="G58" s="25" t="str">
         <f t="shared" si="3"/>
@@ -2744,7 +2751,7 @@
       </c>
       <c r="I58" s="13"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
         <v>92</v>
       </c>
@@ -2757,15 +2764,15 @@
       </c>
       <c r="D59" s="24">
         <f>B33</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E59" s="16">
         <f>B32*B33*B34</f>
-        <v>0.85</v>
+        <v>1.36</v>
       </c>
       <c r="F59" s="16">
         <f t="shared" si="2"/>
-        <v>3.7777777777777781</v>
+        <v>6.0444444444444452</v>
       </c>
       <c r="G59" s="25" t="str">
         <f t="shared" si="3"/>
@@ -2776,37 +2783,37 @@
       </c>
       <c r="I59" s="13"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>99</v>
       </c>
@@ -2840,7 +2847,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -2850,17 +2857,17 @@
     <col min="6" max="6" width="56" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
         <v>102</v>
       </c>
@@ -2880,7 +2887,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A5" s="28" t="s">
         <v>108</v>
       </c>
@@ -2900,7 +2907,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="66" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A6" s="28" t="s">
         <v>114</v>
       </c>
@@ -2920,7 +2927,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="66" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A7" s="28" t="s">
         <v>120</v>
       </c>
@@ -2940,7 +2947,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="66" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A8" s="28" t="s">
         <v>126</v>
       </c>
@@ -2960,7 +2967,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="66" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>132</v>
       </c>
@@ -2980,7 +2987,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A10" s="28" t="s">
         <v>138</v>
       </c>
@@ -3000,7 +3007,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="66" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A11" s="28" t="s">
         <v>144</v>
       </c>
@@ -3020,7 +3027,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A12" s="28" t="s">
         <v>150</v>
       </c>
@@ -3040,7 +3047,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="66" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A13" s="28" t="s">
         <v>156</v>
       </c>
@@ -3060,7 +3067,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A14" s="28" t="s">
         <v>162</v>
       </c>
@@ -3089,23 +3096,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03C3DC63-880C-4C7A-BD99-15B2870A7881}">
   <dimension ref="A1:Q70"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="59.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="66.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="59.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="66.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="44" t="s">
         <v>102</v>
       </c>
@@ -3140,7 +3147,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
         <v>108</v>
       </c>
@@ -3166,7 +3173,7 @@
         <v>1333.81</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="36" t="s">
         <v>207</v>
       </c>
@@ -3188,7 +3195,7 @@
         <v>1094.8399999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>205</v>
       </c>
@@ -3224,7 +3231,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>203</v>
       </c>
@@ -3260,7 +3267,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
         <v>201</v>
       </c>
@@ -3296,7 +3303,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
         <v>199</v>
       </c>
@@ -3332,7 +3339,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="33"/>
       <c r="B8" s="33"/>
       <c r="C8" s="34"/>
@@ -3345,7 +3352,7 @@
       <c r="J8" s="32"/>
       <c r="K8" s="32"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
         <v>197</v>
       </c>
@@ -3364,7 +3371,7 @@
       <c r="F9" s="33" t="s">
         <v>180</v>
       </c>
-      <c r="G9" s="38" t="s">
+      <c r="G9" s="46" t="s">
         <v>176</v>
       </c>
       <c r="H9" s="39">
@@ -3381,7 +3388,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
         <v>256</v>
       </c>
@@ -3417,7 +3424,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="36" t="s">
         <v>196</v>
       </c>
@@ -3443,7 +3450,7 @@
         <v>135.47999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
         <v>194</v>
       </c>
@@ -3471,7 +3478,7 @@
       <c r="I12" s="33">
         <v>1</v>
       </c>
-      <c r="J12" s="63">
+      <c r="J12" s="66">
         <v>7.68</v>
       </c>
       <c r="K12" s="32">
@@ -3479,7 +3486,7 @@
         <v>7.21</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="54"/>
       <c r="B13" s="54"/>
       <c r="C13" s="55"/>
@@ -3489,10 +3496,10 @@
       <c r="G13" s="54"/>
       <c r="H13" s="58"/>
       <c r="I13" s="54"/>
-      <c r="J13" s="85"/>
+      <c r="J13" s="68"/>
       <c r="K13" s="56"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="33" t="s">
         <v>193</v>
       </c>
@@ -3520,13 +3527,13 @@
       <c r="I14" s="33">
         <v>3</v>
       </c>
-      <c r="J14" s="86"/>
+      <c r="J14" s="69"/>
       <c r="K14" s="32">
         <f>I14*E14</f>
         <v>38.97</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
         <v>192</v>
       </c>
@@ -3554,13 +3561,13 @@
       <c r="I15" s="33">
         <v>1</v>
       </c>
-      <c r="J15" s="86"/>
+      <c r="J15" s="69"/>
       <c r="K15" s="32">
         <f t="shared" ref="K15:K25" si="0">I15*E15</f>
         <v>9.99</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
         <v>191</v>
       </c>
@@ -3588,13 +3595,13 @@
       <c r="I16" s="33">
         <v>1</v>
       </c>
-      <c r="J16" s="86"/>
+      <c r="J16" s="69"/>
       <c r="K16" s="32">
         <f t="shared" si="0"/>
         <v>9.7899999999999991</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="54"/>
       <c r="B17" s="54"/>
       <c r="C17" s="55"/>
@@ -3604,10 +3611,10 @@
       <c r="G17" s="54"/>
       <c r="H17" s="54"/>
       <c r="I17" s="54"/>
-      <c r="J17" s="85"/>
+      <c r="J17" s="68"/>
       <c r="K17" s="56"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="33" t="s">
         <v>190</v>
       </c>
@@ -3635,13 +3642,13 @@
       <c r="I18" s="33">
         <v>1</v>
       </c>
-      <c r="J18" s="86"/>
+      <c r="J18" s="69"/>
       <c r="K18" s="32">
         <f t="shared" si="0"/>
         <v>6.99</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="33" t="s">
         <v>189</v>
       </c>
@@ -3669,13 +3676,13 @@
       <c r="I19" s="33">
         <v>1</v>
       </c>
-      <c r="J19" s="86"/>
+      <c r="J19" s="69"/>
       <c r="K19" s="32">
         <f t="shared" si="0"/>
         <v>8.99</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="54"/>
       <c r="B20" s="54"/>
       <c r="C20" s="55"/>
@@ -3685,10 +3692,10 @@
       <c r="G20" s="54"/>
       <c r="H20" s="54"/>
       <c r="I20" s="54"/>
-      <c r="J20" s="85"/>
+      <c r="J20" s="68"/>
       <c r="K20" s="56"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="47" t="s">
         <v>188</v>
       </c>
@@ -3716,13 +3723,13 @@
       <c r="I21" s="33">
         <v>2</v>
       </c>
-      <c r="J21" s="86"/>
+      <c r="J21" s="69"/>
       <c r="K21" s="32">
         <f t="shared" si="0"/>
         <v>15.58</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="47" t="s">
         <v>187</v>
       </c>
@@ -3735,28 +3742,28 @@
       <c r="D22" s="33">
         <v>9</v>
       </c>
-      <c r="E22" s="63">
+      <c r="E22" s="66">
         <v>22.99</v>
       </c>
       <c r="F22" s="47" t="s">
         <v>247</v>
       </c>
-      <c r="G22" s="79" t="s">
+      <c r="G22" s="72" t="s">
         <v>176</v>
       </c>
-      <c r="H22" s="81">
+      <c r="H22" s="70">
         <v>46230</v>
       </c>
-      <c r="I22" s="83">
+      <c r="I22" s="74">
         <v>1</v>
       </c>
-      <c r="J22" s="86"/>
-      <c r="K22" s="63">
+      <c r="J22" s="69"/>
+      <c r="K22" s="66">
         <f t="shared" si="0"/>
         <v>22.99</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="47" t="s">
         <v>186</v>
       </c>
@@ -3769,17 +3776,17 @@
       <c r="D23" s="33">
         <v>7</v>
       </c>
-      <c r="E23" s="64"/>
+      <c r="E23" s="67"/>
       <c r="F23" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G23" s="80"/>
-      <c r="H23" s="82"/>
-      <c r="I23" s="84"/>
-      <c r="J23" s="86"/>
-      <c r="K23" s="64"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G23" s="73"/>
+      <c r="H23" s="71"/>
+      <c r="I23" s="75"/>
+      <c r="J23" s="69"/>
+      <c r="K23" s="67"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="47" t="s">
         <v>185</v>
       </c>
@@ -3801,10 +3808,10 @@
         <v>248</v>
       </c>
       <c r="I24" s="33"/>
-      <c r="J24" s="86"/>
+      <c r="J24" s="69"/>
       <c r="K24" s="32"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="47" t="s">
         <v>218</v>
       </c>
@@ -3832,13 +3839,13 @@
       <c r="I25" s="33">
         <v>1</v>
       </c>
-      <c r="J25" s="86"/>
+      <c r="J25" s="69"/>
       <c r="K25" s="32">
         <f t="shared" si="0"/>
         <v>7.29</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="47" t="s">
         <v>219</v>
       </c>
@@ -3864,10 +3871,10 @@
         <v>248</v>
       </c>
       <c r="I26" s="33"/>
-      <c r="J26" s="64"/>
+      <c r="J26" s="67"/>
       <c r="K26" s="32"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="54"/>
       <c r="B27" s="54"/>
       <c r="C27" s="55"/>
@@ -3880,7 +3887,7 @@
       <c r="J27" s="56"/>
       <c r="K27" s="56"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="33" t="s">
         <v>220</v>
       </c>
@@ -3894,16 +3901,16 @@
         <v>1</v>
       </c>
       <c r="E28" s="32"/>
-      <c r="F28" s="65" t="s">
+      <c r="F28" s="76" t="s">
         <v>233</v>
       </c>
-      <c r="G28" s="66"/>
-      <c r="H28" s="66"/>
-      <c r="I28" s="66"/>
-      <c r="J28" s="66"/>
-      <c r="K28" s="67"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G28" s="77"/>
+      <c r="H28" s="77"/>
+      <c r="I28" s="77"/>
+      <c r="J28" s="77"/>
+      <c r="K28" s="78"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="33" t="s">
         <v>222</v>
       </c>
@@ -3917,14 +3924,14 @@
         <v>1</v>
       </c>
       <c r="E29" s="32"/>
-      <c r="F29" s="68"/>
-      <c r="G29" s="69"/>
-      <c r="H29" s="69"/>
-      <c r="I29" s="69"/>
-      <c r="J29" s="69"/>
-      <c r="K29" s="70"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F29" s="79"/>
+      <c r="G29" s="80"/>
+      <c r="H29" s="80"/>
+      <c r="I29" s="80"/>
+      <c r="J29" s="80"/>
+      <c r="K29" s="81"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="33" t="s">
         <v>223</v>
       </c>
@@ -3938,14 +3945,14 @@
         <v>78</v>
       </c>
       <c r="E30" s="32"/>
-      <c r="F30" s="68"/>
-      <c r="G30" s="69"/>
-      <c r="H30" s="69"/>
-      <c r="I30" s="69"/>
-      <c r="J30" s="69"/>
-      <c r="K30" s="70"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F30" s="79"/>
+      <c r="G30" s="80"/>
+      <c r="H30" s="80"/>
+      <c r="I30" s="80"/>
+      <c r="J30" s="80"/>
+      <c r="K30" s="81"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="33" t="s">
         <v>224</v>
       </c>
@@ -3959,14 +3966,14 @@
         <v>39</v>
       </c>
       <c r="E31" s="32"/>
-      <c r="F31" s="68"/>
-      <c r="G31" s="69"/>
-      <c r="H31" s="69"/>
-      <c r="I31" s="69"/>
-      <c r="J31" s="69"/>
-      <c r="K31" s="70"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F31" s="79"/>
+      <c r="G31" s="80"/>
+      <c r="H31" s="80"/>
+      <c r="I31" s="80"/>
+      <c r="J31" s="80"/>
+      <c r="K31" s="81"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="33" t="s">
         <v>225</v>
       </c>
@@ -3980,14 +3987,14 @@
         <v>2</v>
       </c>
       <c r="E32" s="32"/>
-      <c r="F32" s="68"/>
-      <c r="G32" s="69"/>
-      <c r="H32" s="69"/>
-      <c r="I32" s="69"/>
-      <c r="J32" s="69"/>
-      <c r="K32" s="70"/>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="80"/>
+      <c r="I32" s="80"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="81"/>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="33" t="s">
         <v>226</v>
       </c>
@@ -4001,14 +4008,14 @@
         <v>2</v>
       </c>
       <c r="E33" s="32"/>
-      <c r="F33" s="68"/>
-      <c r="G33" s="69"/>
-      <c r="H33" s="69"/>
-      <c r="I33" s="69"/>
-      <c r="J33" s="69"/>
-      <c r="K33" s="70"/>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F33" s="79"/>
+      <c r="G33" s="80"/>
+      <c r="H33" s="80"/>
+      <c r="I33" s="80"/>
+      <c r="J33" s="80"/>
+      <c r="K33" s="81"/>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="33" t="s">
         <v>227</v>
       </c>
@@ -4022,14 +4029,14 @@
         <v>1</v>
       </c>
       <c r="E34" s="32"/>
-      <c r="F34" s="68"/>
-      <c r="G34" s="69"/>
-      <c r="H34" s="69"/>
-      <c r="I34" s="69"/>
-      <c r="J34" s="69"/>
-      <c r="K34" s="70"/>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F34" s="79"/>
+      <c r="G34" s="80"/>
+      <c r="H34" s="80"/>
+      <c r="I34" s="80"/>
+      <c r="J34" s="80"/>
+      <c r="K34" s="81"/>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="33" t="s">
         <v>228</v>
       </c>
@@ -4043,14 +4050,14 @@
         <v>1</v>
       </c>
       <c r="E35" s="32"/>
-      <c r="F35" s="68"/>
-      <c r="G35" s="69"/>
-      <c r="H35" s="69"/>
-      <c r="I35" s="69"/>
-      <c r="J35" s="69"/>
-      <c r="K35" s="70"/>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F35" s="79"/>
+      <c r="G35" s="80"/>
+      <c r="H35" s="80"/>
+      <c r="I35" s="80"/>
+      <c r="J35" s="80"/>
+      <c r="K35" s="81"/>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="33" t="s">
         <v>229</v>
       </c>
@@ -4064,14 +4071,14 @@
         <v>1</v>
       </c>
       <c r="E36" s="32"/>
-      <c r="F36" s="68"/>
-      <c r="G36" s="69"/>
-      <c r="H36" s="69"/>
-      <c r="I36" s="69"/>
-      <c r="J36" s="69"/>
-      <c r="K36" s="70"/>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F36" s="79"/>
+      <c r="G36" s="80"/>
+      <c r="H36" s="80"/>
+      <c r="I36" s="80"/>
+      <c r="J36" s="80"/>
+      <c r="K36" s="81"/>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="33" t="s">
         <v>231</v>
       </c>
@@ -4085,15 +4092,15 @@
         <v>1</v>
       </c>
       <c r="E37" s="32"/>
-      <c r="F37" s="68"/>
-      <c r="G37" s="69"/>
-      <c r="H37" s="69"/>
-      <c r="I37" s="69"/>
-      <c r="J37" s="69"/>
-      <c r="K37" s="70"/>
+      <c r="F37" s="79"/>
+      <c r="G37" s="80"/>
+      <c r="H37" s="80"/>
+      <c r="I37" s="80"/>
+      <c r="J37" s="80"/>
+      <c r="K37" s="81"/>
       <c r="Q37" s="48"/>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="33" t="s">
         <v>232</v>
       </c>
@@ -4107,14 +4114,14 @@
         <v>1</v>
       </c>
       <c r="E38" s="32"/>
-      <c r="F38" s="68"/>
-      <c r="G38" s="69"/>
-      <c r="H38" s="69"/>
-      <c r="I38" s="69"/>
-      <c r="J38" s="69"/>
-      <c r="K38" s="70"/>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F38" s="79"/>
+      <c r="G38" s="80"/>
+      <c r="H38" s="80"/>
+      <c r="I38" s="80"/>
+      <c r="J38" s="80"/>
+      <c r="K38" s="81"/>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="33" t="s">
         <v>244</v>
       </c>
@@ -4128,14 +4135,14 @@
         <v>1</v>
       </c>
       <c r="E39" s="32"/>
-      <c r="F39" s="68"/>
-      <c r="G39" s="69"/>
-      <c r="H39" s="69"/>
-      <c r="I39" s="69"/>
-      <c r="J39" s="69"/>
-      <c r="K39" s="70"/>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F39" s="79"/>
+      <c r="G39" s="80"/>
+      <c r="H39" s="80"/>
+      <c r="I39" s="80"/>
+      <c r="J39" s="80"/>
+      <c r="K39" s="81"/>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="33" t="s">
         <v>245</v>
       </c>
@@ -4149,14 +4156,14 @@
         <v>1</v>
       </c>
       <c r="E40" s="32"/>
-      <c r="F40" s="71"/>
-      <c r="G40" s="72"/>
-      <c r="H40" s="72"/>
-      <c r="I40" s="72"/>
-      <c r="J40" s="72"/>
-      <c r="K40" s="73"/>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F40" s="82"/>
+      <c r="G40" s="83"/>
+      <c r="H40" s="83"/>
+      <c r="I40" s="83"/>
+      <c r="J40" s="83"/>
+      <c r="K40" s="84"/>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="36">
         <v>1.3</v>
       </c>
@@ -4182,7 +4189,7 @@
         <v>103.49</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="47" t="s">
         <v>184</v>
       </c>
@@ -4204,13 +4211,13 @@
       <c r="G42" s="45" t="s">
         <v>176</v>
       </c>
-      <c r="H42" s="88">
+      <c r="H42" s="63">
         <v>46237</v>
       </c>
       <c r="I42" s="33">
         <v>1</v>
       </c>
-      <c r="J42" s="75">
+      <c r="J42" s="86">
         <v>5.87</v>
       </c>
       <c r="K42" s="32">
@@ -4218,7 +4225,7 @@
         <v>7.21</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="54"/>
       <c r="B43" s="54"/>
       <c r="C43" s="55"/>
@@ -4228,10 +4235,10 @@
       <c r="G43" s="54"/>
       <c r="H43" s="58"/>
       <c r="I43" s="54"/>
-      <c r="J43" s="76"/>
+      <c r="J43" s="87"/>
       <c r="K43" s="56"/>
     </row>
-    <row r="44" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="47" t="s">
         <v>182</v>
       </c>
@@ -4253,19 +4260,19 @@
       <c r="G44" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="H44" s="88">
+      <c r="H44" s="63">
         <v>46237</v>
       </c>
       <c r="I44" s="33">
         <v>3</v>
       </c>
-      <c r="J44" s="77"/>
+      <c r="J44" s="88"/>
       <c r="K44" s="32">
         <f>I44*E44</f>
         <v>38.97</v>
       </c>
     </row>
-    <row r="45" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="47" t="s">
         <v>179</v>
       </c>
@@ -4287,19 +4294,19 @@
       <c r="G45" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="H45" s="88">
+      <c r="H45" s="63">
         <v>46237</v>
       </c>
       <c r="I45" s="33">
         <v>1</v>
       </c>
-      <c r="J45" s="77"/>
+      <c r="J45" s="88"/>
       <c r="K45" s="32">
         <f t="shared" ref="K45:K46" si="1">I45*E45</f>
         <v>8.09</v>
       </c>
     </row>
-    <row r="46" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="47" t="s">
         <v>291</v>
       </c>
@@ -4321,19 +4328,19 @@
       <c r="G46" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="H46" s="88">
+      <c r="H46" s="63">
         <v>46237</v>
       </c>
       <c r="I46" s="33">
         <v>1</v>
       </c>
-      <c r="J46" s="77"/>
+      <c r="J46" s="88"/>
       <c r="K46" s="32">
         <f t="shared" si="1"/>
         <v>9.99</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="54"/>
       <c r="B47" s="54"/>
       <c r="C47" s="55"/>
@@ -4343,10 +4350,10 @@
       <c r="G47" s="54"/>
       <c r="H47" s="54"/>
       <c r="I47" s="54"/>
-      <c r="J47" s="76"/>
+      <c r="J47" s="87"/>
       <c r="K47" s="56"/>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="47" t="s">
         <v>292</v>
       </c>
@@ -4372,13 +4379,13 @@
         <v>259</v>
       </c>
       <c r="I48" s="33"/>
-      <c r="J48" s="77"/>
+      <c r="J48" s="88"/>
       <c r="K48" s="32">
         <f t="shared" ref="K48:K55" si="2">I48*E48</f>
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="47" t="s">
         <v>293</v>
       </c>
@@ -4404,13 +4411,13 @@
         <v>259</v>
       </c>
       <c r="I49" s="33"/>
-      <c r="J49" s="77"/>
+      <c r="J49" s="88"/>
       <c r="K49" s="32">
         <f>I49*E49</f>
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59"/>
       <c r="B50" s="54"/>
       <c r="C50" s="55"/>
@@ -4420,10 +4427,10 @@
       <c r="G50" s="54"/>
       <c r="H50" s="54"/>
       <c r="I50" s="54"/>
-      <c r="J50" s="76"/>
+      <c r="J50" s="87"/>
       <c r="K50" s="56"/>
     </row>
-    <row r="51" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="47" t="s">
         <v>294</v>
       </c>
@@ -4445,20 +4452,20 @@
       <c r="G51" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="H51" s="88">
+      <c r="H51" s="63">
         <v>46237</v>
       </c>
       <c r="I51" s="33">
         <v>3</v>
       </c>
-      <c r="J51" s="77"/>
+      <c r="J51" s="88"/>
       <c r="K51" s="32">
         <f t="shared" ref="K51:K52" si="3">I51*E51</f>
         <v>23.37</v>
       </c>
       <c r="Q51" s="31"/>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="47" t="s">
         <v>295</v>
       </c>
@@ -4471,26 +4478,26 @@
       <c r="D52" s="33">
         <v>9</v>
       </c>
-      <c r="E52" s="63">
+      <c r="E52" s="66">
         <v>22.99</v>
       </c>
       <c r="F52" s="47" t="s">
         <v>260</v>
       </c>
-      <c r="G52" s="79" t="s">
+      <c r="G52" s="72" t="s">
         <v>176</v>
       </c>
-      <c r="H52" s="81" t="s">
+      <c r="H52" s="70" t="s">
         <v>259</v>
       </c>
-      <c r="I52" s="83"/>
-      <c r="J52" s="77"/>
-      <c r="K52" s="63">
+      <c r="I52" s="74"/>
+      <c r="J52" s="88"/>
+      <c r="K52" s="66">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="47" t="s">
         <v>296</v>
       </c>
@@ -4503,17 +4510,17 @@
       <c r="D53" s="33">
         <v>7</v>
       </c>
-      <c r="E53" s="64"/>
+      <c r="E53" s="67"/>
       <c r="F53" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G53" s="80"/>
-      <c r="H53" s="82"/>
-      <c r="I53" s="84"/>
-      <c r="J53" s="77"/>
-      <c r="K53" s="64"/>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="G53" s="73"/>
+      <c r="H53" s="71"/>
+      <c r="I53" s="75"/>
+      <c r="J53" s="88"/>
+      <c r="K53" s="67"/>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="47" t="s">
         <v>297</v>
       </c>
@@ -4535,19 +4542,19 @@
       <c r="G54" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="H54" s="88">
+      <c r="H54" s="63">
         <v>46237</v>
       </c>
       <c r="I54" s="33">
         <v>1</v>
       </c>
-      <c r="J54" s="77"/>
+      <c r="J54" s="88"/>
       <c r="K54" s="32">
         <f>I54*E54</f>
         <v>9.99</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="47" t="s">
         <v>298</v>
       </c>
@@ -4573,13 +4580,13 @@
         <v>258</v>
       </c>
       <c r="I55" s="47"/>
-      <c r="J55" s="77"/>
+      <c r="J55" s="88"/>
       <c r="K55" s="32">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="47" t="s">
         <v>299</v>
       </c>
@@ -4605,10 +4612,10 @@
         <v>248</v>
       </c>
       <c r="I56" s="33"/>
-      <c r="J56" s="78"/>
+      <c r="J56" s="89"/>
       <c r="K56" s="32"/>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="54"/>
       <c r="B57" s="54"/>
       <c r="C57" s="55"/>
@@ -4621,7 +4628,7 @@
       <c r="J57" s="56"/>
       <c r="K57" s="56"/>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="47" t="s">
         <v>300</v>
       </c>
@@ -4635,16 +4642,16 @@
         <v>1</v>
       </c>
       <c r="E58" s="32"/>
-      <c r="F58" s="74" t="s">
+      <c r="F58" s="85" t="s">
         <v>290</v>
       </c>
-      <c r="G58" s="66"/>
-      <c r="H58" s="66"/>
-      <c r="I58" s="66"/>
-      <c r="J58" s="66"/>
-      <c r="K58" s="67"/>
-    </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="G58" s="77"/>
+      <c r="H58" s="77"/>
+      <c r="I58" s="77"/>
+      <c r="J58" s="77"/>
+      <c r="K58" s="78"/>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="47" t="s">
         <v>301</v>
       </c>
@@ -4658,14 +4665,14 @@
         <v>1</v>
       </c>
       <c r="E59" s="32"/>
-      <c r="F59" s="68"/>
-      <c r="G59" s="69"/>
-      <c r="H59" s="69"/>
-      <c r="I59" s="69"/>
-      <c r="J59" s="69"/>
-      <c r="K59" s="70"/>
-    </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F59" s="79"/>
+      <c r="G59" s="80"/>
+      <c r="H59" s="80"/>
+      <c r="I59" s="80"/>
+      <c r="J59" s="80"/>
+      <c r="K59" s="81"/>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="47" t="s">
         <v>302</v>
       </c>
@@ -4679,14 +4686,14 @@
         <v>44</v>
       </c>
       <c r="E60" s="32"/>
-      <c r="F60" s="68"/>
-      <c r="G60" s="69"/>
-      <c r="H60" s="69"/>
-      <c r="I60" s="69"/>
-      <c r="J60" s="69"/>
-      <c r="K60" s="70"/>
-    </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F60" s="79"/>
+      <c r="G60" s="80"/>
+      <c r="H60" s="80"/>
+      <c r="I60" s="80"/>
+      <c r="J60" s="80"/>
+      <c r="K60" s="81"/>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="47" t="s">
         <v>303</v>
       </c>
@@ -4700,14 +4707,14 @@
         <v>22</v>
       </c>
       <c r="E61" s="32"/>
-      <c r="F61" s="68"/>
-      <c r="G61" s="69"/>
-      <c r="H61" s="69"/>
-      <c r="I61" s="69"/>
-      <c r="J61" s="69"/>
-      <c r="K61" s="70"/>
-    </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F61" s="79"/>
+      <c r="G61" s="80"/>
+      <c r="H61" s="80"/>
+      <c r="I61" s="80"/>
+      <c r="J61" s="80"/>
+      <c r="K61" s="81"/>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="47" t="s">
         <v>304</v>
       </c>
@@ -4721,14 +4728,14 @@
         <v>2</v>
       </c>
       <c r="E62" s="32"/>
-      <c r="F62" s="68"/>
-      <c r="G62" s="69"/>
-      <c r="H62" s="69"/>
-      <c r="I62" s="69"/>
-      <c r="J62" s="69"/>
-      <c r="K62" s="70"/>
-    </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F62" s="79"/>
+      <c r="G62" s="80"/>
+      <c r="H62" s="80"/>
+      <c r="I62" s="80"/>
+      <c r="J62" s="80"/>
+      <c r="K62" s="81"/>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="47" t="s">
         <v>305</v>
       </c>
@@ -4742,14 +4749,14 @@
         <v>2</v>
       </c>
       <c r="E63" s="32"/>
-      <c r="F63" s="68"/>
-      <c r="G63" s="69"/>
-      <c r="H63" s="69"/>
-      <c r="I63" s="69"/>
-      <c r="J63" s="69"/>
-      <c r="K63" s="70"/>
-    </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F63" s="79"/>
+      <c r="G63" s="80"/>
+      <c r="H63" s="80"/>
+      <c r="I63" s="80"/>
+      <c r="J63" s="80"/>
+      <c r="K63" s="81"/>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="47" t="s">
         <v>306</v>
       </c>
@@ -4763,14 +4770,14 @@
         <v>1</v>
       </c>
       <c r="E64" s="32"/>
-      <c r="F64" s="68"/>
-      <c r="G64" s="69"/>
-      <c r="H64" s="69"/>
-      <c r="I64" s="69"/>
-      <c r="J64" s="69"/>
-      <c r="K64" s="70"/>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F64" s="79"/>
+      <c r="G64" s="80"/>
+      <c r="H64" s="80"/>
+      <c r="I64" s="80"/>
+      <c r="J64" s="80"/>
+      <c r="K64" s="81"/>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="47" t="s">
         <v>307</v>
       </c>
@@ -4784,14 +4791,14 @@
         <v>1</v>
       </c>
       <c r="E65" s="32"/>
-      <c r="F65" s="68"/>
-      <c r="G65" s="69"/>
-      <c r="H65" s="69"/>
-      <c r="I65" s="69"/>
-      <c r="J65" s="69"/>
-      <c r="K65" s="70"/>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F65" s="79"/>
+      <c r="G65" s="80"/>
+      <c r="H65" s="80"/>
+      <c r="I65" s="80"/>
+      <c r="J65" s="80"/>
+      <c r="K65" s="81"/>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="47" t="s">
         <v>308</v>
       </c>
@@ -4805,14 +4812,14 @@
         <v>1</v>
       </c>
       <c r="E66" s="32"/>
-      <c r="F66" s="68"/>
-      <c r="G66" s="69"/>
-      <c r="H66" s="69"/>
-      <c r="I66" s="69"/>
-      <c r="J66" s="69"/>
-      <c r="K66" s="70"/>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F66" s="79"/>
+      <c r="G66" s="80"/>
+      <c r="H66" s="80"/>
+      <c r="I66" s="80"/>
+      <c r="J66" s="80"/>
+      <c r="K66" s="81"/>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="47" t="s">
         <v>309</v>
       </c>
@@ -4826,14 +4833,14 @@
         <v>1</v>
       </c>
       <c r="E67" s="32"/>
-      <c r="F67" s="68"/>
-      <c r="G67" s="69"/>
-      <c r="H67" s="69"/>
-      <c r="I67" s="69"/>
-      <c r="J67" s="69"/>
-      <c r="K67" s="70"/>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F67" s="79"/>
+      <c r="G67" s="80"/>
+      <c r="H67" s="80"/>
+      <c r="I67" s="80"/>
+      <c r="J67" s="80"/>
+      <c r="K67" s="81"/>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="47" t="s">
         <v>310</v>
       </c>
@@ -4847,14 +4854,14 @@
         <v>1</v>
       </c>
       <c r="E68" s="32"/>
-      <c r="F68" s="68"/>
-      <c r="G68" s="69"/>
-      <c r="H68" s="69"/>
-      <c r="I68" s="69"/>
-      <c r="J68" s="69"/>
-      <c r="K68" s="70"/>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F68" s="79"/>
+      <c r="G68" s="80"/>
+      <c r="H68" s="80"/>
+      <c r="I68" s="80"/>
+      <c r="J68" s="80"/>
+      <c r="K68" s="81"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="47" t="s">
         <v>311</v>
       </c>
@@ -4868,14 +4875,14 @@
         <v>1</v>
       </c>
       <c r="E69" s="32"/>
-      <c r="F69" s="68"/>
-      <c r="G69" s="69"/>
-      <c r="H69" s="69"/>
-      <c r="I69" s="69"/>
-      <c r="J69" s="69"/>
-      <c r="K69" s="70"/>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F69" s="79"/>
+      <c r="G69" s="80"/>
+      <c r="H69" s="80"/>
+      <c r="I69" s="80"/>
+      <c r="J69" s="80"/>
+      <c r="K69" s="81"/>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="47" t="s">
         <v>312</v>
       </c>
@@ -4889,20 +4896,15 @@
         <v>1</v>
       </c>
       <c r="E70" s="32"/>
-      <c r="F70" s="68"/>
-      <c r="G70" s="69"/>
-      <c r="H70" s="69"/>
-      <c r="I70" s="69"/>
-      <c r="J70" s="69"/>
-      <c r="K70" s="70"/>
+      <c r="F70" s="79"/>
+      <c r="G70" s="80"/>
+      <c r="H70" s="80"/>
+      <c r="I70" s="80"/>
+      <c r="J70" s="80"/>
+      <c r="K70" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="K22:K23"/>
-    <mergeCell ref="J12:J26"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="I22:I23"/>
     <mergeCell ref="E22:E23"/>
     <mergeCell ref="K52:K53"/>
     <mergeCell ref="F28:K40"/>
@@ -4912,6 +4914,11 @@
     <mergeCell ref="G52:G53"/>
     <mergeCell ref="H52:H53"/>
     <mergeCell ref="I52:I53"/>
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="J12:J26"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="I22:I23"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <hyperlinks>
@@ -4939,8 +4946,9 @@
     <hyperlink ref="G51" r:id="rId22" xr:uid="{181C5DE6-9473-4241-B12C-D25DC1804061}"/>
     <hyperlink ref="G54" r:id="rId23" xr:uid="{19AC5AEB-C68E-4393-AAB8-3C0E0C06A444}"/>
     <hyperlink ref="G46" r:id="rId24" xr:uid="{B027617C-3F89-419E-A842-31851D15B3A1}"/>
+    <hyperlink ref="G9" r:id="rId25" xr:uid="{0C670866-C934-4719-A79D-80B26BA422F7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId25"/>
+  <pageSetup orientation="portrait" r:id="rId26"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
testing different ways to attach linkages
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1230963E-BD47-49E0-B776-60988303A4C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E7E85D-355F-41BE-B9D1-2A47DB24B811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Torque Budget" sheetId="1" r:id="rId1"/>
@@ -1516,30 +1516,6 @@
     <xf numFmtId="166" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1581,6 +1557,30 @@
     </xf>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1916,7 +1916,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="4">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>4</v>
@@ -1927,7 +1927,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>4</v>
@@ -2313,14 +2313,14 @@
       </c>
       <c r="D38" s="14">
         <f>B5/2</f>
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E38" s="15" t="s">
         <v>64</v>
       </c>
       <c r="F38" s="16">
         <f t="shared" ref="F38:F44" si="0">B38*$B$21*D38</f>
-        <v>4.7088000000000005E-2</v>
+        <v>5.8860000000000003E-2</v>
       </c>
       <c r="G38" s="16">
         <v>0</v>
@@ -2336,14 +2336,14 @@
       </c>
       <c r="D39" s="14">
         <f>B5</f>
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="E39" s="15" t="s">
         <v>64</v>
       </c>
       <c r="F39" s="16">
         <f>B39*$B$21*D39</f>
-        <v>1.4126400000000001</v>
+        <v>1.7658000000000003</v>
       </c>
       <c r="G39" s="16">
         <v>0</v>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="D40" s="14">
         <f>B5+B8</f>
-        <v>0.19</v>
+        <v>0.23</v>
       </c>
       <c r="E40" s="14">
         <f>B8</f>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="F40" s="16">
         <f t="shared" si="0"/>
-        <v>0.22366800000000001</v>
+        <v>0.270756</v>
       </c>
       <c r="G40" s="16">
         <f>B40*$B$21*E40</f>
@@ -2384,19 +2384,19 @@
       </c>
       <c r="D41" s="14">
         <f>B5+B6/2</f>
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="E41" s="14">
         <f>B6/2</f>
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="F41" s="16">
         <f t="shared" si="0"/>
-        <v>0.141264</v>
+        <v>0.15303600000000001</v>
       </c>
       <c r="G41" s="16">
         <f>B41*$B$21*E41</f>
-        <v>4.7088000000000005E-2</v>
+        <v>3.5316E-2</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="E42" s="14">
         <f>B6</f>
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="F42" s="16">
         <f t="shared" si="0"/>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="G42" s="16">
         <f>B42*$B$21*E42</f>
-        <v>0.34531200000000006</v>
+        <v>0.25898400000000005</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="E43" s="14">
         <f>B6+B7/2</f>
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="F43" s="16">
         <f t="shared" si="0"/>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="G43" s="16">
         <f>B43*$B$21*E43</f>
-        <v>0.29430000000000001</v>
+        <v>0.23544000000000001</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="E44" s="14">
         <f>B6+B7</f>
-        <v>0.24</v>
+        <v>0.2</v>
       </c>
       <c r="F44" s="16">
         <f t="shared" si="0"/>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="G44" s="16">
         <f>B44*$B$21*E44</f>
-        <v>0.47088000000000002</v>
+        <v>0.39240000000000008</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -2483,11 +2483,11 @@
       <c r="E45" s="18"/>
       <c r="F45" s="19">
         <f>SUM(F38:F44)</f>
-        <v>3.8298240000000003</v>
+        <v>4.253616000000001</v>
       </c>
       <c r="G45" s="19">
         <f>SUM(G38:G44)</f>
-        <v>1.1928960000000002</v>
+        <v>0.95745600000000008</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -2617,11 +2617,11 @@
       </c>
       <c r="B55" s="16">
         <f>F45</f>
-        <v>3.8298240000000003</v>
+        <v>4.253616000000001</v>
       </c>
       <c r="C55" s="16">
         <f t="shared" si="1"/>
-        <v>5.7447360000000005</v>
+        <v>6.3804240000000014</v>
       </c>
       <c r="D55" s="24">
         <f>B30</f>
@@ -2633,11 +2633,11 @@
       </c>
       <c r="F55" s="16">
         <f t="shared" si="2"/>
-        <v>0.9399909760866294</v>
+        <v>0.84633873861674369</v>
       </c>
       <c r="G55" s="25" t="str">
         <f t="shared" si="3"/>
-        <v>MARGINAL</v>
+        <v>UNDERSIZED</v>
       </c>
       <c r="H55" s="26">
         <f>B26*B30*B28</f>
@@ -2654,11 +2654,11 @@
       </c>
       <c r="B56" s="16">
         <f>G45</f>
-        <v>1.1928960000000002</v>
+        <v>0.95745600000000008</v>
       </c>
       <c r="C56" s="16">
         <f t="shared" si="1"/>
-        <v>1.7893440000000003</v>
+        <v>1.4361840000000001</v>
       </c>
       <c r="D56" s="24">
         <f>B31</f>
@@ -2670,7 +2670,7 @@
       </c>
       <c r="F56" s="16">
         <f t="shared" si="2"/>
-        <v>1.5089328826653787</v>
+        <v>1.8799819521732588</v>
       </c>
       <c r="G56" s="25" t="str">
         <f t="shared" si="3"/>
@@ -3496,7 +3496,7 @@
       <c r="G13" s="54"/>
       <c r="H13" s="58"/>
       <c r="I13" s="54"/>
-      <c r="J13" s="68"/>
+      <c r="J13" s="88"/>
       <c r="K13" s="56"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -3527,7 +3527,7 @@
       <c r="I14" s="33">
         <v>3</v>
       </c>
-      <c r="J14" s="69"/>
+      <c r="J14" s="89"/>
       <c r="K14" s="32">
         <f>I14*E14</f>
         <v>38.97</v>
@@ -3561,7 +3561,7 @@
       <c r="I15" s="33">
         <v>1</v>
       </c>
-      <c r="J15" s="69"/>
+      <c r="J15" s="89"/>
       <c r="K15" s="32">
         <f t="shared" ref="K15:K25" si="0">I15*E15</f>
         <v>9.99</v>
@@ -3595,7 +3595,7 @@
       <c r="I16" s="33">
         <v>1</v>
       </c>
-      <c r="J16" s="69"/>
+      <c r="J16" s="89"/>
       <c r="K16" s="32">
         <f t="shared" si="0"/>
         <v>9.7899999999999991</v>
@@ -3611,7 +3611,7 @@
       <c r="G17" s="54"/>
       <c r="H17" s="54"/>
       <c r="I17" s="54"/>
-      <c r="J17" s="68"/>
+      <c r="J17" s="88"/>
       <c r="K17" s="56"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -3642,7 +3642,7 @@
       <c r="I18" s="33">
         <v>1</v>
       </c>
-      <c r="J18" s="69"/>
+      <c r="J18" s="89"/>
       <c r="K18" s="32">
         <f t="shared" si="0"/>
         <v>6.99</v>
@@ -3676,7 +3676,7 @@
       <c r="I19" s="33">
         <v>1</v>
       </c>
-      <c r="J19" s="69"/>
+      <c r="J19" s="89"/>
       <c r="K19" s="32">
         <f t="shared" si="0"/>
         <v>8.99</v>
@@ -3692,7 +3692,7 @@
       <c r="G20" s="54"/>
       <c r="H20" s="54"/>
       <c r="I20" s="54"/>
-      <c r="J20" s="68"/>
+      <c r="J20" s="88"/>
       <c r="K20" s="56"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -3723,7 +3723,7 @@
       <c r="I21" s="33">
         <v>2</v>
       </c>
-      <c r="J21" s="69"/>
+      <c r="J21" s="89"/>
       <c r="K21" s="32">
         <f t="shared" si="0"/>
         <v>15.58</v>
@@ -3748,16 +3748,16 @@
       <c r="F22" s="47" t="s">
         <v>247</v>
       </c>
-      <c r="G22" s="72" t="s">
+      <c r="G22" s="82" t="s">
         <v>176</v>
       </c>
-      <c r="H22" s="70">
+      <c r="H22" s="84">
         <v>46230</v>
       </c>
-      <c r="I22" s="74">
+      <c r="I22" s="86">
         <v>1</v>
       </c>
-      <c r="J22" s="69"/>
+      <c r="J22" s="89"/>
       <c r="K22" s="66">
         <f t="shared" si="0"/>
         <v>22.99</v>
@@ -3780,10 +3780,10 @@
       <c r="F23" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G23" s="73"/>
-      <c r="H23" s="71"/>
-      <c r="I23" s="75"/>
-      <c r="J23" s="69"/>
+      <c r="G23" s="83"/>
+      <c r="H23" s="85"/>
+      <c r="I23" s="87"/>
+      <c r="J23" s="89"/>
       <c r="K23" s="67"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -3808,7 +3808,7 @@
         <v>248</v>
       </c>
       <c r="I24" s="33"/>
-      <c r="J24" s="69"/>
+      <c r="J24" s="89"/>
       <c r="K24" s="32"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -3839,7 +3839,7 @@
       <c r="I25" s="33">
         <v>1</v>
       </c>
-      <c r="J25" s="69"/>
+      <c r="J25" s="89"/>
       <c r="K25" s="32">
         <f t="shared" si="0"/>
         <v>7.29</v>
@@ -3901,14 +3901,14 @@
         <v>1</v>
       </c>
       <c r="E28" s="32"/>
-      <c r="F28" s="76" t="s">
+      <c r="F28" s="68" t="s">
         <v>233</v>
       </c>
-      <c r="G28" s="77"/>
-      <c r="H28" s="77"/>
-      <c r="I28" s="77"/>
-      <c r="J28" s="77"/>
-      <c r="K28" s="78"/>
+      <c r="G28" s="69"/>
+      <c r="H28" s="69"/>
+      <c r="I28" s="69"/>
+      <c r="J28" s="69"/>
+      <c r="K28" s="70"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="33" t="s">
@@ -3924,12 +3924,12 @@
         <v>1</v>
       </c>
       <c r="E29" s="32"/>
-      <c r="F29" s="79"/>
-      <c r="G29" s="80"/>
-      <c r="H29" s="80"/>
-      <c r="I29" s="80"/>
-      <c r="J29" s="80"/>
-      <c r="K29" s="81"/>
+      <c r="F29" s="71"/>
+      <c r="G29" s="72"/>
+      <c r="H29" s="72"/>
+      <c r="I29" s="72"/>
+      <c r="J29" s="72"/>
+      <c r="K29" s="73"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="33" t="s">
@@ -3945,12 +3945,12 @@
         <v>78</v>
       </c>
       <c r="E30" s="32"/>
-      <c r="F30" s="79"/>
-      <c r="G30" s="80"/>
-      <c r="H30" s="80"/>
-      <c r="I30" s="80"/>
-      <c r="J30" s="80"/>
-      <c r="K30" s="81"/>
+      <c r="F30" s="71"/>
+      <c r="G30" s="72"/>
+      <c r="H30" s="72"/>
+      <c r="I30" s="72"/>
+      <c r="J30" s="72"/>
+      <c r="K30" s="73"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="33" t="s">
@@ -3966,12 +3966,12 @@
         <v>39</v>
       </c>
       <c r="E31" s="32"/>
-      <c r="F31" s="79"/>
-      <c r="G31" s="80"/>
-      <c r="H31" s="80"/>
-      <c r="I31" s="80"/>
-      <c r="J31" s="80"/>
-      <c r="K31" s="81"/>
+      <c r="F31" s="71"/>
+      <c r="G31" s="72"/>
+      <c r="H31" s="72"/>
+      <c r="I31" s="72"/>
+      <c r="J31" s="72"/>
+      <c r="K31" s="73"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="33" t="s">
@@ -3987,12 +3987,12 @@
         <v>2</v>
       </c>
       <c r="E32" s="32"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="80"/>
-      <c r="I32" s="80"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="81"/>
+      <c r="F32" s="71"/>
+      <c r="G32" s="72"/>
+      <c r="H32" s="72"/>
+      <c r="I32" s="72"/>
+      <c r="J32" s="72"/>
+      <c r="K32" s="73"/>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="33" t="s">
@@ -4008,12 +4008,12 @@
         <v>2</v>
       </c>
       <c r="E33" s="32"/>
-      <c r="F33" s="79"/>
-      <c r="G33" s="80"/>
-      <c r="H33" s="80"/>
-      <c r="I33" s="80"/>
-      <c r="J33" s="80"/>
-      <c r="K33" s="81"/>
+      <c r="F33" s="71"/>
+      <c r="G33" s="72"/>
+      <c r="H33" s="72"/>
+      <c r="I33" s="72"/>
+      <c r="J33" s="72"/>
+      <c r="K33" s="73"/>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="33" t="s">
@@ -4029,12 +4029,12 @@
         <v>1</v>
       </c>
       <c r="E34" s="32"/>
-      <c r="F34" s="79"/>
-      <c r="G34" s="80"/>
-      <c r="H34" s="80"/>
-      <c r="I34" s="80"/>
-      <c r="J34" s="80"/>
-      <c r="K34" s="81"/>
+      <c r="F34" s="71"/>
+      <c r="G34" s="72"/>
+      <c r="H34" s="72"/>
+      <c r="I34" s="72"/>
+      <c r="J34" s="72"/>
+      <c r="K34" s="73"/>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="33" t="s">
@@ -4050,12 +4050,12 @@
         <v>1</v>
       </c>
       <c r="E35" s="32"/>
-      <c r="F35" s="79"/>
-      <c r="G35" s="80"/>
-      <c r="H35" s="80"/>
-      <c r="I35" s="80"/>
-      <c r="J35" s="80"/>
-      <c r="K35" s="81"/>
+      <c r="F35" s="71"/>
+      <c r="G35" s="72"/>
+      <c r="H35" s="72"/>
+      <c r="I35" s="72"/>
+      <c r="J35" s="72"/>
+      <c r="K35" s="73"/>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="33" t="s">
@@ -4071,12 +4071,12 @@
         <v>1</v>
       </c>
       <c r="E36" s="32"/>
-      <c r="F36" s="79"/>
-      <c r="G36" s="80"/>
-      <c r="H36" s="80"/>
-      <c r="I36" s="80"/>
-      <c r="J36" s="80"/>
-      <c r="K36" s="81"/>
+      <c r="F36" s="71"/>
+      <c r="G36" s="72"/>
+      <c r="H36" s="72"/>
+      <c r="I36" s="72"/>
+      <c r="J36" s="72"/>
+      <c r="K36" s="73"/>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="33" t="s">
@@ -4092,12 +4092,12 @@
         <v>1</v>
       </c>
       <c r="E37" s="32"/>
-      <c r="F37" s="79"/>
-      <c r="G37" s="80"/>
-      <c r="H37" s="80"/>
-      <c r="I37" s="80"/>
-      <c r="J37" s="80"/>
-      <c r="K37" s="81"/>
+      <c r="F37" s="71"/>
+      <c r="G37" s="72"/>
+      <c r="H37" s="72"/>
+      <c r="I37" s="72"/>
+      <c r="J37" s="72"/>
+      <c r="K37" s="73"/>
       <c r="Q37" s="48"/>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
@@ -4114,12 +4114,12 @@
         <v>1</v>
       </c>
       <c r="E38" s="32"/>
-      <c r="F38" s="79"/>
-      <c r="G38" s="80"/>
-      <c r="H38" s="80"/>
-      <c r="I38" s="80"/>
-      <c r="J38" s="80"/>
-      <c r="K38" s="81"/>
+      <c r="F38" s="71"/>
+      <c r="G38" s="72"/>
+      <c r="H38" s="72"/>
+      <c r="I38" s="72"/>
+      <c r="J38" s="72"/>
+      <c r="K38" s="73"/>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="33" t="s">
@@ -4135,12 +4135,12 @@
         <v>1</v>
       </c>
       <c r="E39" s="32"/>
-      <c r="F39" s="79"/>
-      <c r="G39" s="80"/>
-      <c r="H39" s="80"/>
-      <c r="I39" s="80"/>
-      <c r="J39" s="80"/>
-      <c r="K39" s="81"/>
+      <c r="F39" s="71"/>
+      <c r="G39" s="72"/>
+      <c r="H39" s="72"/>
+      <c r="I39" s="72"/>
+      <c r="J39" s="72"/>
+      <c r="K39" s="73"/>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="33" t="s">
@@ -4156,12 +4156,12 @@
         <v>1</v>
       </c>
       <c r="E40" s="32"/>
-      <c r="F40" s="82"/>
-      <c r="G40" s="83"/>
-      <c r="H40" s="83"/>
-      <c r="I40" s="83"/>
-      <c r="J40" s="83"/>
-      <c r="K40" s="84"/>
+      <c r="F40" s="74"/>
+      <c r="G40" s="75"/>
+      <c r="H40" s="75"/>
+      <c r="I40" s="75"/>
+      <c r="J40" s="75"/>
+      <c r="K40" s="76"/>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="36">
@@ -4217,7 +4217,7 @@
       <c r="I42" s="33">
         <v>1</v>
       </c>
-      <c r="J42" s="86">
+      <c r="J42" s="78">
         <v>5.87</v>
       </c>
       <c r="K42" s="32">
@@ -4235,7 +4235,7 @@
       <c r="G43" s="54"/>
       <c r="H43" s="58"/>
       <c r="I43" s="54"/>
-      <c r="J43" s="87"/>
+      <c r="J43" s="79"/>
       <c r="K43" s="56"/>
     </row>
     <row r="44" spans="1:17" ht="30" x14ac:dyDescent="0.25">
@@ -4266,7 +4266,7 @@
       <c r="I44" s="33">
         <v>3</v>
       </c>
-      <c r="J44" s="88"/>
+      <c r="J44" s="80"/>
       <c r="K44" s="32">
         <f>I44*E44</f>
         <v>38.97</v>
@@ -4300,7 +4300,7 @@
       <c r="I45" s="33">
         <v>1</v>
       </c>
-      <c r="J45" s="88"/>
+      <c r="J45" s="80"/>
       <c r="K45" s="32">
         <f t="shared" ref="K45:K46" si="1">I45*E45</f>
         <v>8.09</v>
@@ -4334,7 +4334,7 @@
       <c r="I46" s="33">
         <v>1</v>
       </c>
-      <c r="J46" s="88"/>
+      <c r="J46" s="80"/>
       <c r="K46" s="32">
         <f t="shared" si="1"/>
         <v>9.99</v>
@@ -4350,7 +4350,7 @@
       <c r="G47" s="54"/>
       <c r="H47" s="54"/>
       <c r="I47" s="54"/>
-      <c r="J47" s="87"/>
+      <c r="J47" s="79"/>
       <c r="K47" s="56"/>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.25">
@@ -4379,7 +4379,7 @@
         <v>259</v>
       </c>
       <c r="I48" s="33"/>
-      <c r="J48" s="88"/>
+      <c r="J48" s="80"/>
       <c r="K48" s="32">
         <f t="shared" ref="K48:K55" si="2">I48*E48</f>
         <v>0</v>
@@ -4411,7 +4411,7 @@
         <v>259</v>
       </c>
       <c r="I49" s="33"/>
-      <c r="J49" s="88"/>
+      <c r="J49" s="80"/>
       <c r="K49" s="32">
         <f>I49*E49</f>
         <v>0</v>
@@ -4427,7 +4427,7 @@
       <c r="G50" s="54"/>
       <c r="H50" s="54"/>
       <c r="I50" s="54"/>
-      <c r="J50" s="87"/>
+      <c r="J50" s="79"/>
       <c r="K50" s="56"/>
     </row>
     <row r="51" spans="1:17" ht="30" x14ac:dyDescent="0.25">
@@ -4458,7 +4458,7 @@
       <c r="I51" s="33">
         <v>3</v>
       </c>
-      <c r="J51" s="88"/>
+      <c r="J51" s="80"/>
       <c r="K51" s="32">
         <f t="shared" ref="K51:K52" si="3">I51*E51</f>
         <v>23.37</v>
@@ -4484,14 +4484,14 @@
       <c r="F52" s="47" t="s">
         <v>260</v>
       </c>
-      <c r="G52" s="72" t="s">
+      <c r="G52" s="82" t="s">
         <v>176</v>
       </c>
-      <c r="H52" s="70" t="s">
+      <c r="H52" s="84" t="s">
         <v>259</v>
       </c>
-      <c r="I52" s="74"/>
-      <c r="J52" s="88"/>
+      <c r="I52" s="86"/>
+      <c r="J52" s="80"/>
       <c r="K52" s="66">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -4514,10 +4514,10 @@
       <c r="F53" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G53" s="73"/>
-      <c r="H53" s="71"/>
-      <c r="I53" s="75"/>
-      <c r="J53" s="88"/>
+      <c r="G53" s="83"/>
+      <c r="H53" s="85"/>
+      <c r="I53" s="87"/>
+      <c r="J53" s="80"/>
       <c r="K53" s="67"/>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
@@ -4548,7 +4548,7 @@
       <c r="I54" s="33">
         <v>1</v>
       </c>
-      <c r="J54" s="88"/>
+      <c r="J54" s="80"/>
       <c r="K54" s="32">
         <f>I54*E54</f>
         <v>9.99</v>
@@ -4580,7 +4580,7 @@
         <v>258</v>
       </c>
       <c r="I55" s="47"/>
-      <c r="J55" s="88"/>
+      <c r="J55" s="80"/>
       <c r="K55" s="32">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -4612,7 +4612,7 @@
         <v>248</v>
       </c>
       <c r="I56" s="33"/>
-      <c r="J56" s="89"/>
+      <c r="J56" s="81"/>
       <c r="K56" s="32"/>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.25">
@@ -4642,14 +4642,14 @@
         <v>1</v>
       </c>
       <c r="E58" s="32"/>
-      <c r="F58" s="85" t="s">
+      <c r="F58" s="77" t="s">
         <v>290</v>
       </c>
-      <c r="G58" s="77"/>
-      <c r="H58" s="77"/>
-      <c r="I58" s="77"/>
-      <c r="J58" s="77"/>
-      <c r="K58" s="78"/>
+      <c r="G58" s="69"/>
+      <c r="H58" s="69"/>
+      <c r="I58" s="69"/>
+      <c r="J58" s="69"/>
+      <c r="K58" s="70"/>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="47" t="s">
@@ -4665,12 +4665,12 @@
         <v>1</v>
       </c>
       <c r="E59" s="32"/>
-      <c r="F59" s="79"/>
-      <c r="G59" s="80"/>
-      <c r="H59" s="80"/>
-      <c r="I59" s="80"/>
-      <c r="J59" s="80"/>
-      <c r="K59" s="81"/>
+      <c r="F59" s="71"/>
+      <c r="G59" s="72"/>
+      <c r="H59" s="72"/>
+      <c r="I59" s="72"/>
+      <c r="J59" s="72"/>
+      <c r="K59" s="73"/>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="47" t="s">
@@ -4686,12 +4686,12 @@
         <v>44</v>
       </c>
       <c r="E60" s="32"/>
-      <c r="F60" s="79"/>
-      <c r="G60" s="80"/>
-      <c r="H60" s="80"/>
-      <c r="I60" s="80"/>
-      <c r="J60" s="80"/>
-      <c r="K60" s="81"/>
+      <c r="F60" s="71"/>
+      <c r="G60" s="72"/>
+      <c r="H60" s="72"/>
+      <c r="I60" s="72"/>
+      <c r="J60" s="72"/>
+      <c r="K60" s="73"/>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="47" t="s">
@@ -4707,12 +4707,12 @@
         <v>22</v>
       </c>
       <c r="E61" s="32"/>
-      <c r="F61" s="79"/>
-      <c r="G61" s="80"/>
-      <c r="H61" s="80"/>
-      <c r="I61" s="80"/>
-      <c r="J61" s="80"/>
-      <c r="K61" s="81"/>
+      <c r="F61" s="71"/>
+      <c r="G61" s="72"/>
+      <c r="H61" s="72"/>
+      <c r="I61" s="72"/>
+      <c r="J61" s="72"/>
+      <c r="K61" s="73"/>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="47" t="s">
@@ -4728,12 +4728,12 @@
         <v>2</v>
       </c>
       <c r="E62" s="32"/>
-      <c r="F62" s="79"/>
-      <c r="G62" s="80"/>
-      <c r="H62" s="80"/>
-      <c r="I62" s="80"/>
-      <c r="J62" s="80"/>
-      <c r="K62" s="81"/>
+      <c r="F62" s="71"/>
+      <c r="G62" s="72"/>
+      <c r="H62" s="72"/>
+      <c r="I62" s="72"/>
+      <c r="J62" s="72"/>
+      <c r="K62" s="73"/>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="47" t="s">
@@ -4749,12 +4749,12 @@
         <v>2</v>
       </c>
       <c r="E63" s="32"/>
-      <c r="F63" s="79"/>
-      <c r="G63" s="80"/>
-      <c r="H63" s="80"/>
-      <c r="I63" s="80"/>
-      <c r="J63" s="80"/>
-      <c r="K63" s="81"/>
+      <c r="F63" s="71"/>
+      <c r="G63" s="72"/>
+      <c r="H63" s="72"/>
+      <c r="I63" s="72"/>
+      <c r="J63" s="72"/>
+      <c r="K63" s="73"/>
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="47" t="s">
@@ -4770,12 +4770,12 @@
         <v>1</v>
       </c>
       <c r="E64" s="32"/>
-      <c r="F64" s="79"/>
-      <c r="G64" s="80"/>
-      <c r="H64" s="80"/>
-      <c r="I64" s="80"/>
-      <c r="J64" s="80"/>
-      <c r="K64" s="81"/>
+      <c r="F64" s="71"/>
+      <c r="G64" s="72"/>
+      <c r="H64" s="72"/>
+      <c r="I64" s="72"/>
+      <c r="J64" s="72"/>
+      <c r="K64" s="73"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="47" t="s">
@@ -4791,12 +4791,12 @@
         <v>1</v>
       </c>
       <c r="E65" s="32"/>
-      <c r="F65" s="79"/>
-      <c r="G65" s="80"/>
-      <c r="H65" s="80"/>
-      <c r="I65" s="80"/>
-      <c r="J65" s="80"/>
-      <c r="K65" s="81"/>
+      <c r="F65" s="71"/>
+      <c r="G65" s="72"/>
+      <c r="H65" s="72"/>
+      <c r="I65" s="72"/>
+      <c r="J65" s="72"/>
+      <c r="K65" s="73"/>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="47" t="s">
@@ -4812,12 +4812,12 @@
         <v>1</v>
       </c>
       <c r="E66" s="32"/>
-      <c r="F66" s="79"/>
-      <c r="G66" s="80"/>
-      <c r="H66" s="80"/>
-      <c r="I66" s="80"/>
-      <c r="J66" s="80"/>
-      <c r="K66" s="81"/>
+      <c r="F66" s="71"/>
+      <c r="G66" s="72"/>
+      <c r="H66" s="72"/>
+      <c r="I66" s="72"/>
+      <c r="J66" s="72"/>
+      <c r="K66" s="73"/>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="47" t="s">
@@ -4833,12 +4833,12 @@
         <v>1</v>
       </c>
       <c r="E67" s="32"/>
-      <c r="F67" s="79"/>
-      <c r="G67" s="80"/>
-      <c r="H67" s="80"/>
-      <c r="I67" s="80"/>
-      <c r="J67" s="80"/>
-      <c r="K67" s="81"/>
+      <c r="F67" s="71"/>
+      <c r="G67" s="72"/>
+      <c r="H67" s="72"/>
+      <c r="I67" s="72"/>
+      <c r="J67" s="72"/>
+      <c r="K67" s="73"/>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="47" t="s">
@@ -4854,12 +4854,12 @@
         <v>1</v>
       </c>
       <c r="E68" s="32"/>
-      <c r="F68" s="79"/>
-      <c r="G68" s="80"/>
-      <c r="H68" s="80"/>
-      <c r="I68" s="80"/>
-      <c r="J68" s="80"/>
-      <c r="K68" s="81"/>
+      <c r="F68" s="71"/>
+      <c r="G68" s="72"/>
+      <c r="H68" s="72"/>
+      <c r="I68" s="72"/>
+      <c r="J68" s="72"/>
+      <c r="K68" s="73"/>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="47" t="s">
@@ -4875,12 +4875,12 @@
         <v>1</v>
       </c>
       <c r="E69" s="32"/>
-      <c r="F69" s="79"/>
-      <c r="G69" s="80"/>
-      <c r="H69" s="80"/>
-      <c r="I69" s="80"/>
-      <c r="J69" s="80"/>
-      <c r="K69" s="81"/>
+      <c r="F69" s="71"/>
+      <c r="G69" s="72"/>
+      <c r="H69" s="72"/>
+      <c r="I69" s="72"/>
+      <c r="J69" s="72"/>
+      <c r="K69" s="73"/>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="47" t="s">
@@ -4896,12 +4896,12 @@
         <v>1</v>
       </c>
       <c r="E70" s="32"/>
-      <c r="F70" s="79"/>
-      <c r="G70" s="80"/>
-      <c r="H70" s="80"/>
-      <c r="I70" s="80"/>
-      <c r="J70" s="80"/>
-      <c r="K70" s="81"/>
+      <c r="F70" s="71"/>
+      <c r="G70" s="72"/>
+      <c r="H70" s="72"/>
+      <c r="I70" s="72"/>
+      <c r="J70" s="72"/>
+      <c r="K70" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>

<commit_message>
Testing raw motor torque output
For some reason the motor is not calibrated correctly(?)
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0041F7-5BF2-49D0-A8FA-7A3D94288924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2528FD3-9F86-461D-9786-C3E01D3D0FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Torque Budget" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="320">
   <si>
     <t>6-DoF Arm — Gravity Torque Budget v2 (elbow-mounted forearm roll)</t>
   </si>
@@ -1002,6 +1002,9 @@
   <si>
     <t xml:space="preserve"> ID 10mm x OD 15mm x 4mm (10 pcs)
 Purchase 1 pack for two 15:1 gearboxes</t>
+  </si>
+  <si>
+    <t>ADD THIS TO BOM PLEASE</t>
   </si>
 </sst>
 </file>
@@ -1014,7 +1017,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1131,6 +1134,13 @@
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1351,7 +1361,7 @@
     <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1509,6 +1519,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1581,7 +1592,7 @@
     <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1694,6 +1705,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>10583</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>85280</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>58933</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C6A8FD8F-A74B-4D90-A2F5-3EBC6FACA129}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18478501" y="2106083"/>
+          <a:ext cx="4382112" cy="5191850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1899,17 +1959,17 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="89"/>
-      <c r="C4" s="89"/>
-      <c r="D4" s="89"/>
-      <c r="E4" s="89"/>
-      <c r="F4" s="89"/>
-      <c r="G4" s="89"/>
-      <c r="H4" s="89"/>
-      <c r="I4" s="89"/>
+      <c r="B4" s="65"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -1977,17 +2037,17 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="89" t="s">
+      <c r="A11" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="89"/>
-      <c r="C11" s="89"/>
-      <c r="D11" s="89"/>
-      <c r="E11" s="89"/>
-      <c r="F11" s="89"/>
-      <c r="G11" s="89"/>
-      <c r="H11" s="89"/>
-      <c r="I11" s="89"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="65"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="65"/>
+      <c r="I11" s="65"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -2085,17 +2145,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="89" t="s">
+      <c r="A20" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="89"/>
-      <c r="C20" s="89"/>
-      <c r="D20" s="89"/>
-      <c r="E20" s="89"/>
-      <c r="F20" s="89"/>
-      <c r="G20" s="89"/>
-      <c r="H20" s="89"/>
-      <c r="I20" s="89"/>
+      <c r="B20" s="65"/>
+      <c r="C20" s="65"/>
+      <c r="D20" s="65"/>
+      <c r="E20" s="65"/>
+      <c r="F20" s="65"/>
+      <c r="G20" s="65"/>
+      <c r="H20" s="65"/>
+      <c r="I20" s="65"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
@@ -2120,17 +2180,17 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="89" t="s">
+      <c r="A24" s="65" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="89"/>
-      <c r="C24" s="89"/>
-      <c r="D24" s="89"/>
-      <c r="E24" s="89"/>
-      <c r="F24" s="89"/>
-      <c r="G24" s="89"/>
-      <c r="H24" s="89"/>
-      <c r="I24" s="89"/>
+      <c r="B24" s="65"/>
+      <c r="C24" s="65"/>
+      <c r="D24" s="65"/>
+      <c r="E24" s="65"/>
+      <c r="F24" s="65"/>
+      <c r="G24" s="65"/>
+      <c r="H24" s="65"/>
+      <c r="I24" s="65"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
@@ -2270,17 +2330,17 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="89" t="s">
+      <c r="A36" s="65" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="89"/>
-      <c r="C36" s="89"/>
-      <c r="D36" s="89"/>
-      <c r="E36" s="89"/>
-      <c r="F36" s="89"/>
-      <c r="G36" s="89"/>
-      <c r="H36" s="89"/>
-      <c r="I36" s="89"/>
+      <c r="B36" s="65"/>
+      <c r="C36" s="65"/>
+      <c r="D36" s="65"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="65"/>
+      <c r="G36" s="65"/>
+      <c r="H36" s="65"/>
+      <c r="I36" s="65"/>
     </row>
     <row r="37" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
@@ -2491,17 +2551,17 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="89" t="s">
+      <c r="A47" s="65" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="89"/>
-      <c r="C47" s="89"/>
-      <c r="D47" s="89"/>
-      <c r="E47" s="89"/>
-      <c r="F47" s="89"/>
-      <c r="G47" s="89"/>
-      <c r="H47" s="89"/>
-      <c r="I47" s="89"/>
+      <c r="B47" s="65"/>
+      <c r="C47" s="65"/>
+      <c r="D47" s="65"/>
+      <c r="E47" s="65"/>
+      <c r="F47" s="65"/>
+      <c r="G47" s="65"/>
+      <c r="H47" s="65"/>
+      <c r="I47" s="65"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
@@ -2534,17 +2594,17 @@
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="89" t="s">
+      <c r="A52" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="89"/>
-      <c r="C52" s="89"/>
-      <c r="D52" s="89"/>
-      <c r="E52" s="89"/>
-      <c r="F52" s="89"/>
-      <c r="G52" s="89"/>
-      <c r="H52" s="89"/>
-      <c r="I52" s="89"/>
+      <c r="B52" s="65"/>
+      <c r="C52" s="65"/>
+      <c r="D52" s="65"/>
+      <c r="E52" s="65"/>
+      <c r="F52" s="65"/>
+      <c r="G52" s="65"/>
+      <c r="H52" s="65"/>
+      <c r="I52" s="65"/>
     </row>
     <row r="53" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
@@ -3112,7 +3172,7 @@
     <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="44" t="s">
         <v>102</v>
       </c>
@@ -3147,7 +3207,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
         <v>108</v>
       </c>
@@ -3173,7 +3233,7 @@
         <v>1333.81</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="36" t="s">
         <v>207</v>
       </c>
@@ -3195,7 +3255,7 @@
         <v>1094.8399999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>205</v>
       </c>
@@ -3231,7 +3291,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>203</v>
       </c>
@@ -3267,7 +3327,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
         <v>201</v>
       </c>
@@ -3303,7 +3363,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
         <v>199</v>
       </c>
@@ -3339,7 +3399,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="33"/>
       <c r="B8" s="33"/>
       <c r="C8" s="34"/>
@@ -3352,7 +3412,7 @@
       <c r="J8" s="32"/>
       <c r="K8" s="32"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
         <v>197</v>
       </c>
@@ -3388,7 +3448,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
         <v>256</v>
       </c>
@@ -3423,8 +3483,11 @@
         <f>D10*E10</f>
         <v>207</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P10" s="90" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="36" t="s">
         <v>196</v>
       </c>
@@ -3450,7 +3513,7 @@
         <v>135.47999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
         <v>194</v>
       </c>
@@ -3478,7 +3541,7 @@
       <c r="I12" s="33">
         <v>1</v>
       </c>
-      <c r="J12" s="65">
+      <c r="J12" s="66">
         <v>7.68</v>
       </c>
       <c r="K12" s="32">
@@ -3486,7 +3549,7 @@
         <v>7.21</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="54"/>
       <c r="B13" s="54"/>
       <c r="C13" s="55"/>
@@ -3496,10 +3559,10 @@
       <c r="G13" s="54"/>
       <c r="H13" s="58"/>
       <c r="I13" s="54"/>
-      <c r="J13" s="87"/>
+      <c r="J13" s="88"/>
       <c r="K13" s="56"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="33" t="s">
         <v>193</v>
       </c>
@@ -3527,13 +3590,13 @@
       <c r="I14" s="33">
         <v>3</v>
       </c>
-      <c r="J14" s="88"/>
+      <c r="J14" s="89"/>
       <c r="K14" s="32">
         <f>I14*E14</f>
         <v>38.97</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
         <v>192</v>
       </c>
@@ -3561,13 +3624,13 @@
       <c r="I15" s="33">
         <v>1</v>
       </c>
-      <c r="J15" s="88"/>
+      <c r="J15" s="89"/>
       <c r="K15" s="32">
         <f t="shared" ref="K15:K25" si="0">I15*E15</f>
         <v>9.99</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
         <v>191</v>
       </c>
@@ -3595,7 +3658,7 @@
       <c r="I16" s="33">
         <v>1</v>
       </c>
-      <c r="J16" s="88"/>
+      <c r="J16" s="89"/>
       <c r="K16" s="32">
         <f t="shared" si="0"/>
         <v>9.7899999999999991</v>
@@ -3611,7 +3674,7 @@
       <c r="G17" s="54"/>
       <c r="H17" s="54"/>
       <c r="I17" s="54"/>
-      <c r="J17" s="87"/>
+      <c r="J17" s="88"/>
       <c r="K17" s="56"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -3642,7 +3705,7 @@
       <c r="I18" s="33">
         <v>1</v>
       </c>
-      <c r="J18" s="88"/>
+      <c r="J18" s="89"/>
       <c r="K18" s="32">
         <f t="shared" si="0"/>
         <v>6.99</v>
@@ -3676,7 +3739,7 @@
       <c r="I19" s="33">
         <v>1</v>
       </c>
-      <c r="J19" s="88"/>
+      <c r="J19" s="89"/>
       <c r="K19" s="32">
         <f t="shared" si="0"/>
         <v>8.99</v>
@@ -3692,7 +3755,7 @@
       <c r="G20" s="54"/>
       <c r="H20" s="54"/>
       <c r="I20" s="54"/>
-      <c r="J20" s="87"/>
+      <c r="J20" s="88"/>
       <c r="K20" s="56"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -3723,7 +3786,7 @@
       <c r="I21" s="33">
         <v>2</v>
       </c>
-      <c r="J21" s="88"/>
+      <c r="J21" s="89"/>
       <c r="K21" s="32">
         <f t="shared" si="0"/>
         <v>15.58</v>
@@ -3742,23 +3805,23 @@
       <c r="D22" s="33">
         <v>9</v>
       </c>
-      <c r="E22" s="65">
+      <c r="E22" s="66">
         <v>22.99</v>
       </c>
       <c r="F22" s="47" t="s">
         <v>247</v>
       </c>
-      <c r="G22" s="81" t="s">
+      <c r="G22" s="82" t="s">
         <v>176</v>
       </c>
-      <c r="H22" s="83">
+      <c r="H22" s="84">
         <v>46230</v>
       </c>
-      <c r="I22" s="85">
+      <c r="I22" s="86">
         <v>1</v>
       </c>
-      <c r="J22" s="88"/>
-      <c r="K22" s="65">
+      <c r="J22" s="89"/>
+      <c r="K22" s="66">
         <f t="shared" si="0"/>
         <v>22.99</v>
       </c>
@@ -3776,15 +3839,15 @@
       <c r="D23" s="33">
         <v>7</v>
       </c>
-      <c r="E23" s="66"/>
+      <c r="E23" s="67"/>
       <c r="F23" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G23" s="82"/>
-      <c r="H23" s="84"/>
-      <c r="I23" s="86"/>
-      <c r="J23" s="88"/>
-      <c r="K23" s="66"/>
+      <c r="G23" s="83"/>
+      <c r="H23" s="85"/>
+      <c r="I23" s="87"/>
+      <c r="J23" s="89"/>
+      <c r="K23" s="67"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="47" t="s">
@@ -3808,7 +3871,7 @@
         <v>248</v>
       </c>
       <c r="I24" s="33"/>
-      <c r="J24" s="88"/>
+      <c r="J24" s="89"/>
       <c r="K24" s="32"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -3839,7 +3902,7 @@
       <c r="I25" s="33">
         <v>1</v>
       </c>
-      <c r="J25" s="88"/>
+      <c r="J25" s="89"/>
       <c r="K25" s="32">
         <f t="shared" si="0"/>
         <v>7.29</v>
@@ -3871,7 +3934,7 @@
         <v>248</v>
       </c>
       <c r="I26" s="33"/>
-      <c r="J26" s="66"/>
+      <c r="J26" s="67"/>
       <c r="K26" s="32"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -3901,14 +3964,14 @@
         <v>1</v>
       </c>
       <c r="E28" s="32"/>
-      <c r="F28" s="67" t="s">
+      <c r="F28" s="68" t="s">
         <v>233</v>
       </c>
-      <c r="G28" s="68"/>
-      <c r="H28" s="68"/>
-      <c r="I28" s="68"/>
-      <c r="J28" s="68"/>
-      <c r="K28" s="69"/>
+      <c r="G28" s="69"/>
+      <c r="H28" s="69"/>
+      <c r="I28" s="69"/>
+      <c r="J28" s="69"/>
+      <c r="K28" s="70"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="33" t="s">
@@ -3924,12 +3987,12 @@
         <v>1</v>
       </c>
       <c r="E29" s="32"/>
-      <c r="F29" s="70"/>
-      <c r="G29" s="71"/>
-      <c r="H29" s="71"/>
-      <c r="I29" s="71"/>
-      <c r="J29" s="71"/>
-      <c r="K29" s="72"/>
+      <c r="F29" s="71"/>
+      <c r="G29" s="72"/>
+      <c r="H29" s="72"/>
+      <c r="I29" s="72"/>
+      <c r="J29" s="72"/>
+      <c r="K29" s="73"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="33" t="s">
@@ -3945,12 +4008,12 @@
         <v>78</v>
       </c>
       <c r="E30" s="32"/>
-      <c r="F30" s="70"/>
-      <c r="G30" s="71"/>
-      <c r="H30" s="71"/>
-      <c r="I30" s="71"/>
-      <c r="J30" s="71"/>
-      <c r="K30" s="72"/>
+      <c r="F30" s="71"/>
+      <c r="G30" s="72"/>
+      <c r="H30" s="72"/>
+      <c r="I30" s="72"/>
+      <c r="J30" s="72"/>
+      <c r="K30" s="73"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="33" t="s">
@@ -3966,12 +4029,12 @@
         <v>39</v>
       </c>
       <c r="E31" s="32"/>
-      <c r="F31" s="70"/>
-      <c r="G31" s="71"/>
-      <c r="H31" s="71"/>
-      <c r="I31" s="71"/>
-      <c r="J31" s="71"/>
-      <c r="K31" s="72"/>
+      <c r="F31" s="71"/>
+      <c r="G31" s="72"/>
+      <c r="H31" s="72"/>
+      <c r="I31" s="72"/>
+      <c r="J31" s="72"/>
+      <c r="K31" s="73"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="33" t="s">
@@ -3987,12 +4050,12 @@
         <v>2</v>
       </c>
       <c r="E32" s="32"/>
-      <c r="F32" s="70"/>
-      <c r="G32" s="71"/>
-      <c r="H32" s="71"/>
-      <c r="I32" s="71"/>
-      <c r="J32" s="71"/>
-      <c r="K32" s="72"/>
+      <c r="F32" s="71"/>
+      <c r="G32" s="72"/>
+      <c r="H32" s="72"/>
+      <c r="I32" s="72"/>
+      <c r="J32" s="72"/>
+      <c r="K32" s="73"/>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="33" t="s">
@@ -4008,12 +4071,12 @@
         <v>2</v>
       </c>
       <c r="E33" s="32"/>
-      <c r="F33" s="70"/>
-      <c r="G33" s="71"/>
-      <c r="H33" s="71"/>
-      <c r="I33" s="71"/>
-      <c r="J33" s="71"/>
-      <c r="K33" s="72"/>
+      <c r="F33" s="71"/>
+      <c r="G33" s="72"/>
+      <c r="H33" s="72"/>
+      <c r="I33" s="72"/>
+      <c r="J33" s="72"/>
+      <c r="K33" s="73"/>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="33" t="s">
@@ -4029,12 +4092,12 @@
         <v>1</v>
       </c>
       <c r="E34" s="32"/>
-      <c r="F34" s="70"/>
-      <c r="G34" s="71"/>
-      <c r="H34" s="71"/>
-      <c r="I34" s="71"/>
-      <c r="J34" s="71"/>
-      <c r="K34" s="72"/>
+      <c r="F34" s="71"/>
+      <c r="G34" s="72"/>
+      <c r="H34" s="72"/>
+      <c r="I34" s="72"/>
+      <c r="J34" s="72"/>
+      <c r="K34" s="73"/>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="33" t="s">
@@ -4050,12 +4113,12 @@
         <v>1</v>
       </c>
       <c r="E35" s="32"/>
-      <c r="F35" s="70"/>
-      <c r="G35" s="71"/>
-      <c r="H35" s="71"/>
-      <c r="I35" s="71"/>
-      <c r="J35" s="71"/>
-      <c r="K35" s="72"/>
+      <c r="F35" s="71"/>
+      <c r="G35" s="72"/>
+      <c r="H35" s="72"/>
+      <c r="I35" s="72"/>
+      <c r="J35" s="72"/>
+      <c r="K35" s="73"/>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="33" t="s">
@@ -4071,12 +4134,12 @@
         <v>1</v>
       </c>
       <c r="E36" s="32"/>
-      <c r="F36" s="70"/>
-      <c r="G36" s="71"/>
-      <c r="H36" s="71"/>
-      <c r="I36" s="71"/>
-      <c r="J36" s="71"/>
-      <c r="K36" s="72"/>
+      <c r="F36" s="71"/>
+      <c r="G36" s="72"/>
+      <c r="H36" s="72"/>
+      <c r="I36" s="72"/>
+      <c r="J36" s="72"/>
+      <c r="K36" s="73"/>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="33" t="s">
@@ -4092,12 +4155,12 @@
         <v>1</v>
       </c>
       <c r="E37" s="32"/>
-      <c r="F37" s="70"/>
-      <c r="G37" s="71"/>
-      <c r="H37" s="71"/>
-      <c r="I37" s="71"/>
-      <c r="J37" s="71"/>
-      <c r="K37" s="72"/>
+      <c r="F37" s="71"/>
+      <c r="G37" s="72"/>
+      <c r="H37" s="72"/>
+      <c r="I37" s="72"/>
+      <c r="J37" s="72"/>
+      <c r="K37" s="73"/>
       <c r="Q37" s="48"/>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
@@ -4114,12 +4177,12 @@
         <v>1</v>
       </c>
       <c r="E38" s="32"/>
-      <c r="F38" s="70"/>
-      <c r="G38" s="71"/>
-      <c r="H38" s="71"/>
-      <c r="I38" s="71"/>
-      <c r="J38" s="71"/>
-      <c r="K38" s="72"/>
+      <c r="F38" s="71"/>
+      <c r="G38" s="72"/>
+      <c r="H38" s="72"/>
+      <c r="I38" s="72"/>
+      <c r="J38" s="72"/>
+      <c r="K38" s="73"/>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="33" t="s">
@@ -4135,12 +4198,12 @@
         <v>1</v>
       </c>
       <c r="E39" s="32"/>
-      <c r="F39" s="70"/>
-      <c r="G39" s="71"/>
-      <c r="H39" s="71"/>
-      <c r="I39" s="71"/>
-      <c r="J39" s="71"/>
-      <c r="K39" s="72"/>
+      <c r="F39" s="71"/>
+      <c r="G39" s="72"/>
+      <c r="H39" s="72"/>
+      <c r="I39" s="72"/>
+      <c r="J39" s="72"/>
+      <c r="K39" s="73"/>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="33" t="s">
@@ -4156,12 +4219,12 @@
         <v>1</v>
       </c>
       <c r="E40" s="32"/>
-      <c r="F40" s="73"/>
-      <c r="G40" s="74"/>
-      <c r="H40" s="74"/>
-      <c r="I40" s="74"/>
-      <c r="J40" s="74"/>
-      <c r="K40" s="75"/>
+      <c r="F40" s="74"/>
+      <c r="G40" s="75"/>
+      <c r="H40" s="75"/>
+      <c r="I40" s="75"/>
+      <c r="J40" s="75"/>
+      <c r="K40" s="76"/>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="36">
@@ -4217,7 +4280,7 @@
       <c r="I42" s="33">
         <v>1</v>
       </c>
-      <c r="J42" s="77">
+      <c r="J42" s="78">
         <v>5.87</v>
       </c>
       <c r="K42" s="32">
@@ -4235,7 +4298,7 @@
       <c r="G43" s="54"/>
       <c r="H43" s="58"/>
       <c r="I43" s="54"/>
-      <c r="J43" s="78"/>
+      <c r="J43" s="79"/>
       <c r="K43" s="56"/>
     </row>
     <row r="44" spans="1:17" ht="30" x14ac:dyDescent="0.25">
@@ -4266,7 +4329,7 @@
       <c r="I44" s="33">
         <v>3</v>
       </c>
-      <c r="J44" s="79"/>
+      <c r="J44" s="80"/>
       <c r="K44" s="32">
         <f>I44*E44</f>
         <v>38.97</v>
@@ -4300,7 +4363,7 @@
       <c r="I45" s="33">
         <v>1</v>
       </c>
-      <c r="J45" s="79"/>
+      <c r="J45" s="80"/>
       <c r="K45" s="32">
         <f t="shared" ref="K45:K46" si="1">I45*E45</f>
         <v>8.09</v>
@@ -4334,7 +4397,7 @@
       <c r="I46" s="33">
         <v>1</v>
       </c>
-      <c r="J46" s="79"/>
+      <c r="J46" s="80"/>
       <c r="K46" s="32">
         <f t="shared" si="1"/>
         <v>9.99</v>
@@ -4350,7 +4413,7 @@
       <c r="G47" s="54"/>
       <c r="H47" s="54"/>
       <c r="I47" s="54"/>
-      <c r="J47" s="78"/>
+      <c r="J47" s="79"/>
       <c r="K47" s="56"/>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.25">
@@ -4379,7 +4442,7 @@
         <v>259</v>
       </c>
       <c r="I48" s="33"/>
-      <c r="J48" s="79"/>
+      <c r="J48" s="80"/>
       <c r="K48" s="32">
         <f t="shared" ref="K48:K55" si="2">I48*E48</f>
         <v>0</v>
@@ -4411,7 +4474,7 @@
         <v>259</v>
       </c>
       <c r="I49" s="33"/>
-      <c r="J49" s="79"/>
+      <c r="J49" s="80"/>
       <c r="K49" s="32">
         <f>I49*E49</f>
         <v>0</v>
@@ -4427,7 +4490,7 @@
       <c r="G50" s="54"/>
       <c r="H50" s="54"/>
       <c r="I50" s="54"/>
-      <c r="J50" s="78"/>
+      <c r="J50" s="79"/>
       <c r="K50" s="56"/>
     </row>
     <row r="51" spans="1:17" ht="30" x14ac:dyDescent="0.25">
@@ -4458,7 +4521,7 @@
       <c r="I51" s="33">
         <v>3</v>
       </c>
-      <c r="J51" s="79"/>
+      <c r="J51" s="80"/>
       <c r="K51" s="32">
         <f t="shared" ref="K51:K52" si="3">I51*E51</f>
         <v>23.37</v>
@@ -4478,21 +4541,21 @@
       <c r="D52" s="33">
         <v>9</v>
       </c>
-      <c r="E52" s="65">
+      <c r="E52" s="66">
         <v>22.99</v>
       </c>
       <c r="F52" s="47" t="s">
         <v>260</v>
       </c>
-      <c r="G52" s="81" t="s">
+      <c r="G52" s="82" t="s">
         <v>176</v>
       </c>
-      <c r="H52" s="83" t="s">
+      <c r="H52" s="84" t="s">
         <v>259</v>
       </c>
-      <c r="I52" s="85"/>
-      <c r="J52" s="79"/>
-      <c r="K52" s="65">
+      <c r="I52" s="86"/>
+      <c r="J52" s="80"/>
+      <c r="K52" s="66">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -4510,15 +4573,15 @@
       <c r="D53" s="33">
         <v>7</v>
       </c>
-      <c r="E53" s="66"/>
+      <c r="E53" s="67"/>
       <c r="F53" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G53" s="82"/>
-      <c r="H53" s="84"/>
-      <c r="I53" s="86"/>
-      <c r="J53" s="79"/>
-      <c r="K53" s="66"/>
+      <c r="G53" s="83"/>
+      <c r="H53" s="85"/>
+      <c r="I53" s="87"/>
+      <c r="J53" s="80"/>
+      <c r="K53" s="67"/>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="47" t="s">
@@ -4548,7 +4611,7 @@
       <c r="I54" s="33">
         <v>1</v>
       </c>
-      <c r="J54" s="79"/>
+      <c r="J54" s="80"/>
       <c r="K54" s="32">
         <f>I54*E54</f>
         <v>9.99</v>
@@ -4580,7 +4643,7 @@
         <v>258</v>
       </c>
       <c r="I55" s="47"/>
-      <c r="J55" s="79"/>
+      <c r="J55" s="80"/>
       <c r="K55" s="32">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -4612,7 +4675,7 @@
         <v>248</v>
       </c>
       <c r="I56" s="33"/>
-      <c r="J56" s="80"/>
+      <c r="J56" s="81"/>
       <c r="K56" s="32"/>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.25">
@@ -4642,14 +4705,14 @@
         <v>1</v>
       </c>
       <c r="E58" s="32"/>
-      <c r="F58" s="76" t="s">
+      <c r="F58" s="77" t="s">
         <v>290</v>
       </c>
-      <c r="G58" s="68"/>
-      <c r="H58" s="68"/>
-      <c r="I58" s="68"/>
-      <c r="J58" s="68"/>
-      <c r="K58" s="69"/>
+      <c r="G58" s="69"/>
+      <c r="H58" s="69"/>
+      <c r="I58" s="69"/>
+      <c r="J58" s="69"/>
+      <c r="K58" s="70"/>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="47" t="s">
@@ -4665,12 +4728,12 @@
         <v>1</v>
       </c>
       <c r="E59" s="32"/>
-      <c r="F59" s="70"/>
-      <c r="G59" s="71"/>
-      <c r="H59" s="71"/>
-      <c r="I59" s="71"/>
-      <c r="J59" s="71"/>
-      <c r="K59" s="72"/>
+      <c r="F59" s="71"/>
+      <c r="G59" s="72"/>
+      <c r="H59" s="72"/>
+      <c r="I59" s="72"/>
+      <c r="J59" s="72"/>
+      <c r="K59" s="73"/>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="47" t="s">
@@ -4686,12 +4749,12 @@
         <v>44</v>
       </c>
       <c r="E60" s="32"/>
-      <c r="F60" s="70"/>
-      <c r="G60" s="71"/>
-      <c r="H60" s="71"/>
-      <c r="I60" s="71"/>
-      <c r="J60" s="71"/>
-      <c r="K60" s="72"/>
+      <c r="F60" s="71"/>
+      <c r="G60" s="72"/>
+      <c r="H60" s="72"/>
+      <c r="I60" s="72"/>
+      <c r="J60" s="72"/>
+      <c r="K60" s="73"/>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="47" t="s">
@@ -4707,12 +4770,12 @@
         <v>22</v>
       </c>
       <c r="E61" s="32"/>
-      <c r="F61" s="70"/>
-      <c r="G61" s="71"/>
-      <c r="H61" s="71"/>
-      <c r="I61" s="71"/>
-      <c r="J61" s="71"/>
-      <c r="K61" s="72"/>
+      <c r="F61" s="71"/>
+      <c r="G61" s="72"/>
+      <c r="H61" s="72"/>
+      <c r="I61" s="72"/>
+      <c r="J61" s="72"/>
+      <c r="K61" s="73"/>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="47" t="s">
@@ -4728,12 +4791,12 @@
         <v>2</v>
       </c>
       <c r="E62" s="32"/>
-      <c r="F62" s="70"/>
-      <c r="G62" s="71"/>
-      <c r="H62" s="71"/>
-      <c r="I62" s="71"/>
-      <c r="J62" s="71"/>
-      <c r="K62" s="72"/>
+      <c r="F62" s="71"/>
+      <c r="G62" s="72"/>
+      <c r="H62" s="72"/>
+      <c r="I62" s="72"/>
+      <c r="J62" s="72"/>
+      <c r="K62" s="73"/>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="47" t="s">
@@ -4749,12 +4812,12 @@
         <v>2</v>
       </c>
       <c r="E63" s="32"/>
-      <c r="F63" s="70"/>
-      <c r="G63" s="71"/>
-      <c r="H63" s="71"/>
-      <c r="I63" s="71"/>
-      <c r="J63" s="71"/>
-      <c r="K63" s="72"/>
+      <c r="F63" s="71"/>
+      <c r="G63" s="72"/>
+      <c r="H63" s="72"/>
+      <c r="I63" s="72"/>
+      <c r="J63" s="72"/>
+      <c r="K63" s="73"/>
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="47" t="s">
@@ -4770,12 +4833,12 @@
         <v>1</v>
       </c>
       <c r="E64" s="32"/>
-      <c r="F64" s="70"/>
-      <c r="G64" s="71"/>
-      <c r="H64" s="71"/>
-      <c r="I64" s="71"/>
-      <c r="J64" s="71"/>
-      <c r="K64" s="72"/>
+      <c r="F64" s="71"/>
+      <c r="G64" s="72"/>
+      <c r="H64" s="72"/>
+      <c r="I64" s="72"/>
+      <c r="J64" s="72"/>
+      <c r="K64" s="73"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="47" t="s">
@@ -4791,12 +4854,12 @@
         <v>1</v>
       </c>
       <c r="E65" s="32"/>
-      <c r="F65" s="70"/>
-      <c r="G65" s="71"/>
-      <c r="H65" s="71"/>
-      <c r="I65" s="71"/>
-      <c r="J65" s="71"/>
-      <c r="K65" s="72"/>
+      <c r="F65" s="71"/>
+      <c r="G65" s="72"/>
+      <c r="H65" s="72"/>
+      <c r="I65" s="72"/>
+      <c r="J65" s="72"/>
+      <c r="K65" s="73"/>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="47" t="s">
@@ -4812,12 +4875,12 @@
         <v>1</v>
       </c>
       <c r="E66" s="32"/>
-      <c r="F66" s="70"/>
-      <c r="G66" s="71"/>
-      <c r="H66" s="71"/>
-      <c r="I66" s="71"/>
-      <c r="J66" s="71"/>
-      <c r="K66" s="72"/>
+      <c r="F66" s="71"/>
+      <c r="G66" s="72"/>
+      <c r="H66" s="72"/>
+      <c r="I66" s="72"/>
+      <c r="J66" s="72"/>
+      <c r="K66" s="73"/>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="47" t="s">
@@ -4833,12 +4896,12 @@
         <v>1</v>
       </c>
       <c r="E67" s="32"/>
-      <c r="F67" s="70"/>
-      <c r="G67" s="71"/>
-      <c r="H67" s="71"/>
-      <c r="I67" s="71"/>
-      <c r="J67" s="71"/>
-      <c r="K67" s="72"/>
+      <c r="F67" s="71"/>
+      <c r="G67" s="72"/>
+      <c r="H67" s="72"/>
+      <c r="I67" s="72"/>
+      <c r="J67" s="72"/>
+      <c r="K67" s="73"/>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="47" t="s">
@@ -4854,12 +4917,12 @@
         <v>1</v>
       </c>
       <c r="E68" s="32"/>
-      <c r="F68" s="70"/>
-      <c r="G68" s="71"/>
-      <c r="H68" s="71"/>
-      <c r="I68" s="71"/>
-      <c r="J68" s="71"/>
-      <c r="K68" s="72"/>
+      <c r="F68" s="71"/>
+      <c r="G68" s="72"/>
+      <c r="H68" s="72"/>
+      <c r="I68" s="72"/>
+      <c r="J68" s="72"/>
+      <c r="K68" s="73"/>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="47" t="s">
@@ -4875,12 +4938,12 @@
         <v>1</v>
       </c>
       <c r="E69" s="32"/>
-      <c r="F69" s="70"/>
-      <c r="G69" s="71"/>
-      <c r="H69" s="71"/>
-      <c r="I69" s="71"/>
-      <c r="J69" s="71"/>
-      <c r="K69" s="72"/>
+      <c r="F69" s="71"/>
+      <c r="G69" s="72"/>
+      <c r="H69" s="72"/>
+      <c r="I69" s="72"/>
+      <c r="J69" s="72"/>
+      <c r="K69" s="73"/>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="47" t="s">
@@ -4896,12 +4959,12 @@
         <v>1</v>
       </c>
       <c r="E70" s="32"/>
-      <c r="F70" s="70"/>
-      <c r="G70" s="71"/>
-      <c r="H70" s="71"/>
-      <c r="I70" s="71"/>
-      <c r="J70" s="71"/>
-      <c r="K70" s="72"/>
+      <c r="F70" s="71"/>
+      <c r="G70" s="72"/>
+      <c r="H70" s="72"/>
+      <c r="I70" s="72"/>
+      <c r="J70" s="72"/>
+      <c r="K70" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -4950,5 +5013,6 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId26"/>
+  <drawing r:id="rId27"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Design for 8:1 gear housing
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2528FD3-9F86-461D-9786-C3E01D3D0FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA6D061-99A0-47FB-AD70-F3B3772DA2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="321">
   <si>
     <t>6-DoF Arm — Gravity Torque Budget v2 (elbow-mounted forearm roll)</t>
   </si>
@@ -1005,6 +1005,9 @@
   </si>
   <si>
     <t>ADD THIS TO BOM PLEASE</t>
+  </si>
+  <si>
+    <t>J4, J5, J6 (V1.0 with encoder)</t>
   </si>
 </sst>
 </file>
@@ -1519,7 +1522,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1592,7 +1595,7 @@
     <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1959,17 +1962,17 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="90" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="65"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="65"/>
-      <c r="I4" s="65"/>
+      <c r="B4" s="90"/>
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -2037,17 +2040,17 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="65" t="s">
+      <c r="A11" s="90" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="65"/>
-      <c r="C11" s="65"/>
-      <c r="D11" s="65"/>
-      <c r="E11" s="65"/>
-      <c r="F11" s="65"/>
-      <c r="G11" s="65"/>
-      <c r="H11" s="65"/>
-      <c r="I11" s="65"/>
+      <c r="B11" s="90"/>
+      <c r="C11" s="90"/>
+      <c r="D11" s="90"/>
+      <c r="E11" s="90"/>
+      <c r="F11" s="90"/>
+      <c r="G11" s="90"/>
+      <c r="H11" s="90"/>
+      <c r="I11" s="90"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -2145,17 +2148,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="65" t="s">
+      <c r="A20" s="90" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="65"/>
-      <c r="C20" s="65"/>
-      <c r="D20" s="65"/>
-      <c r="E20" s="65"/>
-      <c r="F20" s="65"/>
-      <c r="G20" s="65"/>
-      <c r="H20" s="65"/>
-      <c r="I20" s="65"/>
+      <c r="B20" s="90"/>
+      <c r="C20" s="90"/>
+      <c r="D20" s="90"/>
+      <c r="E20" s="90"/>
+      <c r="F20" s="90"/>
+      <c r="G20" s="90"/>
+      <c r="H20" s="90"/>
+      <c r="I20" s="90"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
@@ -2180,17 +2183,17 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="65" t="s">
+      <c r="A24" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="65"/>
-      <c r="C24" s="65"/>
-      <c r="D24" s="65"/>
-      <c r="E24" s="65"/>
-      <c r="F24" s="65"/>
-      <c r="G24" s="65"/>
-      <c r="H24" s="65"/>
-      <c r="I24" s="65"/>
+      <c r="B24" s="90"/>
+      <c r="C24" s="90"/>
+      <c r="D24" s="90"/>
+      <c r="E24" s="90"/>
+      <c r="F24" s="90"/>
+      <c r="G24" s="90"/>
+      <c r="H24" s="90"/>
+      <c r="I24" s="90"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
@@ -2330,17 +2333,17 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="65" t="s">
+      <c r="A36" s="90" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="65"/>
-      <c r="C36" s="65"/>
-      <c r="D36" s="65"/>
-      <c r="E36" s="65"/>
-      <c r="F36" s="65"/>
-      <c r="G36" s="65"/>
-      <c r="H36" s="65"/>
-      <c r="I36" s="65"/>
+      <c r="B36" s="90"/>
+      <c r="C36" s="90"/>
+      <c r="D36" s="90"/>
+      <c r="E36" s="90"/>
+      <c r="F36" s="90"/>
+      <c r="G36" s="90"/>
+      <c r="H36" s="90"/>
+      <c r="I36" s="90"/>
     </row>
     <row r="37" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
@@ -2551,17 +2554,17 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="65" t="s">
+      <c r="A47" s="90" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="65"/>
-      <c r="C47" s="65"/>
-      <c r="D47" s="65"/>
-      <c r="E47" s="65"/>
-      <c r="F47" s="65"/>
-      <c r="G47" s="65"/>
-      <c r="H47" s="65"/>
-      <c r="I47" s="65"/>
+      <c r="B47" s="90"/>
+      <c r="C47" s="90"/>
+      <c r="D47" s="90"/>
+      <c r="E47" s="90"/>
+      <c r="F47" s="90"/>
+      <c r="G47" s="90"/>
+      <c r="H47" s="90"/>
+      <c r="I47" s="90"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
@@ -2594,17 +2597,17 @@
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="65" t="s">
+      <c r="A52" s="90" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="65"/>
-      <c r="C52" s="65"/>
-      <c r="D52" s="65"/>
-      <c r="E52" s="65"/>
-      <c r="F52" s="65"/>
-      <c r="G52" s="65"/>
-      <c r="H52" s="65"/>
-      <c r="I52" s="65"/>
+      <c r="B52" s="90"/>
+      <c r="C52" s="90"/>
+      <c r="D52" s="90"/>
+      <c r="E52" s="90"/>
+      <c r="F52" s="90"/>
+      <c r="G52" s="90"/>
+      <c r="H52" s="90"/>
+      <c r="I52" s="90"/>
     </row>
     <row r="53" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
@@ -3429,7 +3432,7 @@
         <v>65</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>180</v>
+        <v>320</v>
       </c>
       <c r="G9" s="46" t="s">
         <v>176</v>
@@ -3483,7 +3486,7 @@
         <f>D10*E10</f>
         <v>207</v>
       </c>
-      <c r="P10" s="90" t="s">
+      <c r="P10" s="65" t="s">
         <v>319</v>
       </c>
     </row>

</xml_diff>

<commit_message>
printing out 15:1 assembly
</commit_message>
<xml_diff>
--- a/6-DOF-Arm.xlsx
+++ b/6-DOF-Arm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erico\Documents\GitHub\6-DOF-Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E67087-4D7F-4308-9817-7100502A31E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A71F57B-C89F-4986-B8E2-5B735575E813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24684" yWindow="2064" windowWidth="24792" windowHeight="14856" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Torque Budget" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="325">
   <si>
     <t>6-DoF Arm — Gravity Torque Budget v2 (elbow-mounted forearm roll)</t>
   </si>
@@ -1004,9 +1004,6 @@
 Purchase 1 pack for two 15:1 gearboxes</t>
   </si>
   <si>
-    <t>ADD THIS TO BOM PLEASE</t>
-  </si>
-  <si>
     <t>J4, J5, J6 (V1.0 with encoder)</t>
   </si>
   <si>
@@ -1020,6 +1017,9 @@
   </si>
   <si>
     <t>https://www.amazon.com/Feggizuli-Connectors-Insulation-Automotive-Electrical/dp/B0B4NSMBTQ/ref=sr_1_4?crid=1QQRUJYCF8IIJ&amp;dib=eyJ2IjoiMSJ9.7JMFXnhOn4EQuI8k8n-MbFSgPqbHDePKJn1EA8NASIBQckj-XOGxBn5wPGUj5ntkQIKP4IVw3ahpaDhUVGwauEk7ikAED8XLtT_EnkKtB3ty_zBfNcrUpQEt7d7Q4nONtcxa5eDnSfLrWRhuW65u4ud42FPDvhrA-J5vyLfzxOuUFQYwFJx-B6eudAMc_6IqVdN4cTmJMB8AQVyQ8Y1X6E2DoyO9-ibVMdCs3kJ9Fos.GInOUC1CjDAXCpQns-V1SNgQFwaVARW5s-_8iPQIXgI&amp;dib_tag=se&amp;keywords=bullet%2Bconnectors%2Bfor%2Bwiring&amp;qid=1786647345&amp;sprefix=bullet%2Bconnectors%2Caps%2C127&amp;sr=8-4&amp;th=1</t>
+  </si>
+  <si>
+    <t>15-camshaft_spacer</t>
   </si>
 </sst>
 </file>
@@ -1535,6 +1535,16 @@
     </xf>
     <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="14" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1606,16 +1616,6 @@
     </xf>
     <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="14" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1729,55 +1729,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>10583</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>85280</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>58933</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C6A8FD8F-A74B-4D90-A2F5-3EBC6FACA129}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="18478501" y="2106083"/>
-          <a:ext cx="4382112" cy="5191850"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1983,17 +1934,17 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="90" t="s">
+      <c r="A4" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="90"/>
-      <c r="I4" s="90"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="69"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -2061,17 +2012,17 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="69" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="90"/>
-      <c r="C11" s="90"/>
-      <c r="D11" s="90"/>
-      <c r="E11" s="90"/>
-      <c r="F11" s="90"/>
-      <c r="G11" s="90"/>
-      <c r="H11" s="90"/>
-      <c r="I11" s="90"/>
+      <c r="B11" s="69"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="69"/>
+      <c r="I11" s="69"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -2169,17 +2120,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="90" t="s">
+      <c r="A20" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="90"/>
-      <c r="C20" s="90"/>
-      <c r="D20" s="90"/>
-      <c r="E20" s="90"/>
-      <c r="F20" s="90"/>
-      <c r="G20" s="90"/>
-      <c r="H20" s="90"/>
-      <c r="I20" s="90"/>
+      <c r="B20" s="69"/>
+      <c r="C20" s="69"/>
+      <c r="D20" s="69"/>
+      <c r="E20" s="69"/>
+      <c r="F20" s="69"/>
+      <c r="G20" s="69"/>
+      <c r="H20" s="69"/>
+      <c r="I20" s="69"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
@@ -2204,17 +2155,17 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="90" t="s">
+      <c r="A24" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="90"/>
-      <c r="C24" s="90"/>
-      <c r="D24" s="90"/>
-      <c r="E24" s="90"/>
-      <c r="F24" s="90"/>
-      <c r="G24" s="90"/>
-      <c r="H24" s="90"/>
-      <c r="I24" s="90"/>
+      <c r="B24" s="69"/>
+      <c r="C24" s="69"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="69"/>
+      <c r="F24" s="69"/>
+      <c r="G24" s="69"/>
+      <c r="H24" s="69"/>
+      <c r="I24" s="69"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
@@ -2354,17 +2305,17 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="90" t="s">
+      <c r="A36" s="69" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="90"/>
-      <c r="C36" s="90"/>
-      <c r="D36" s="90"/>
-      <c r="E36" s="90"/>
-      <c r="F36" s="90"/>
-      <c r="G36" s="90"/>
-      <c r="H36" s="90"/>
-      <c r="I36" s="90"/>
+      <c r="B36" s="69"/>
+      <c r="C36" s="69"/>
+      <c r="D36" s="69"/>
+      <c r="E36" s="69"/>
+      <c r="F36" s="69"/>
+      <c r="G36" s="69"/>
+      <c r="H36" s="69"/>
+      <c r="I36" s="69"/>
     </row>
     <row r="37" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
@@ -2575,17 +2526,17 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="90" t="s">
+      <c r="A47" s="69" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="90"/>
-      <c r="C47" s="90"/>
-      <c r="D47" s="90"/>
-      <c r="E47" s="90"/>
-      <c r="F47" s="90"/>
-      <c r="G47" s="90"/>
-      <c r="H47" s="90"/>
-      <c r="I47" s="90"/>
+      <c r="B47" s="69"/>
+      <c r="C47" s="69"/>
+      <c r="D47" s="69"/>
+      <c r="E47" s="69"/>
+      <c r="F47" s="69"/>
+      <c r="G47" s="69"/>
+      <c r="H47" s="69"/>
+      <c r="I47" s="69"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
@@ -2618,17 +2569,17 @@
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="90" t="s">
+      <c r="A52" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="90"/>
-      <c r="C52" s="90"/>
-      <c r="D52" s="90"/>
-      <c r="E52" s="90"/>
-      <c r="F52" s="90"/>
-      <c r="G52" s="90"/>
-      <c r="H52" s="90"/>
-      <c r="I52" s="90"/>
+      <c r="B52" s="69"/>
+      <c r="C52" s="69"/>
+      <c r="D52" s="69"/>
+      <c r="E52" s="69"/>
+      <c r="F52" s="69"/>
+      <c r="G52" s="69"/>
+      <c r="H52" s="69"/>
+      <c r="I52" s="69"/>
     </row>
     <row r="53" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
@@ -3453,7 +3404,7 @@
         <v>65</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="G9" s="46" t="s">
         <v>176</v>
@@ -3507,9 +3458,7 @@
         <f>D10*E10</f>
         <v>207</v>
       </c>
-      <c r="P10" s="65" t="s">
-        <v>319</v>
-      </c>
+      <c r="P10" s="65"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="36" t="s">
@@ -3565,7 +3514,7 @@
       <c r="I12" s="33">
         <v>1</v>
       </c>
-      <c r="J12" s="66">
+      <c r="J12" s="70">
         <v>7.68</v>
       </c>
       <c r="K12" s="32">
@@ -3583,7 +3532,7 @@
       <c r="G13" s="54"/>
       <c r="H13" s="58"/>
       <c r="I13" s="54"/>
-      <c r="J13" s="88"/>
+      <c r="J13" s="92"/>
       <c r="K13" s="56"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
@@ -3614,7 +3563,7 @@
       <c r="I14" s="33">
         <v>3</v>
       </c>
-      <c r="J14" s="89"/>
+      <c r="J14" s="93"/>
       <c r="K14" s="32">
         <f>I14*E14</f>
         <v>38.97</v>
@@ -3648,7 +3597,7 @@
       <c r="I15" s="33">
         <v>1</v>
       </c>
-      <c r="J15" s="89"/>
+      <c r="J15" s="93"/>
       <c r="K15" s="32">
         <f t="shared" ref="K15:K25" si="0">I15*E15</f>
         <v>9.99</v>
@@ -3682,7 +3631,7 @@
       <c r="I16" s="33">
         <v>1</v>
       </c>
-      <c r="J16" s="89"/>
+      <c r="J16" s="93"/>
       <c r="K16" s="32">
         <f t="shared" si="0"/>
         <v>9.7899999999999991</v>
@@ -3698,7 +3647,7 @@
       <c r="G17" s="54"/>
       <c r="H17" s="54"/>
       <c r="I17" s="54"/>
-      <c r="J17" s="88"/>
+      <c r="J17" s="92"/>
       <c r="K17" s="56"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -3729,7 +3678,7 @@
       <c r="I18" s="33">
         <v>1</v>
       </c>
-      <c r="J18" s="89"/>
+      <c r="J18" s="93"/>
       <c r="K18" s="32">
         <f t="shared" si="0"/>
         <v>6.99</v>
@@ -3763,7 +3712,7 @@
       <c r="I19" s="33">
         <v>1</v>
       </c>
-      <c r="J19" s="89"/>
+      <c r="J19" s="93"/>
       <c r="K19" s="32">
         <f t="shared" si="0"/>
         <v>8.99</v>
@@ -3779,7 +3728,7 @@
       <c r="G20" s="54"/>
       <c r="H20" s="54"/>
       <c r="I20" s="54"/>
-      <c r="J20" s="88"/>
+      <c r="J20" s="92"/>
       <c r="K20" s="56"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -3810,7 +3759,7 @@
       <c r="I21" s="33">
         <v>2</v>
       </c>
-      <c r="J21" s="89"/>
+      <c r="J21" s="93"/>
       <c r="K21" s="32">
         <f t="shared" si="0"/>
         <v>15.58</v>
@@ -3829,23 +3778,23 @@
       <c r="D22" s="33">
         <v>9</v>
       </c>
-      <c r="E22" s="66">
+      <c r="E22" s="70">
         <v>22.99</v>
       </c>
       <c r="F22" s="47" t="s">
         <v>247</v>
       </c>
-      <c r="G22" s="82" t="s">
+      <c r="G22" s="86" t="s">
         <v>176</v>
       </c>
-      <c r="H22" s="84">
+      <c r="H22" s="88">
         <v>46230</v>
       </c>
-      <c r="I22" s="86">
+      <c r="I22" s="90">
         <v>1</v>
       </c>
-      <c r="J22" s="89"/>
-      <c r="K22" s="66">
+      <c r="J22" s="93"/>
+      <c r="K22" s="70">
         <f t="shared" si="0"/>
         <v>22.99</v>
       </c>
@@ -3863,15 +3812,15 @@
       <c r="D23" s="33">
         <v>7</v>
       </c>
-      <c r="E23" s="67"/>
+      <c r="E23" s="71"/>
       <c r="F23" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G23" s="83"/>
-      <c r="H23" s="85"/>
-      <c r="I23" s="87"/>
-      <c r="J23" s="89"/>
-      <c r="K23" s="67"/>
+      <c r="G23" s="87"/>
+      <c r="H23" s="89"/>
+      <c r="I23" s="91"/>
+      <c r="J23" s="93"/>
+      <c r="K23" s="71"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="47" t="s">
@@ -3895,7 +3844,7 @@
         <v>248</v>
       </c>
       <c r="I24" s="33"/>
-      <c r="J24" s="89"/>
+      <c r="J24" s="93"/>
       <c r="K24" s="32"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -3926,7 +3875,7 @@
       <c r="I25" s="33">
         <v>1</v>
       </c>
-      <c r="J25" s="89"/>
+      <c r="J25" s="93"/>
       <c r="K25" s="32">
         <f t="shared" si="0"/>
         <v>7.29</v>
@@ -3958,7 +3907,7 @@
         <v>248</v>
       </c>
       <c r="I26" s="33"/>
-      <c r="J26" s="67"/>
+      <c r="J26" s="71"/>
       <c r="K26" s="32"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -3988,14 +3937,14 @@
         <v>1</v>
       </c>
       <c r="E28" s="32"/>
-      <c r="F28" s="68" t="s">
+      <c r="F28" s="72" t="s">
         <v>233</v>
       </c>
-      <c r="G28" s="69"/>
-      <c r="H28" s="69"/>
-      <c r="I28" s="69"/>
-      <c r="J28" s="69"/>
-      <c r="K28" s="70"/>
+      <c r="G28" s="73"/>
+      <c r="H28" s="73"/>
+      <c r="I28" s="73"/>
+      <c r="J28" s="73"/>
+      <c r="K28" s="74"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="33" t="s">
@@ -4011,12 +3960,12 @@
         <v>1</v>
       </c>
       <c r="E29" s="32"/>
-      <c r="F29" s="71"/>
-      <c r="G29" s="72"/>
-      <c r="H29" s="72"/>
-      <c r="I29" s="72"/>
-      <c r="J29" s="72"/>
-      <c r="K29" s="73"/>
+      <c r="F29" s="75"/>
+      <c r="G29" s="76"/>
+      <c r="H29" s="76"/>
+      <c r="I29" s="76"/>
+      <c r="J29" s="76"/>
+      <c r="K29" s="77"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="33" t="s">
@@ -4032,12 +3981,12 @@
         <v>78</v>
       </c>
       <c r="E30" s="32"/>
-      <c r="F30" s="71"/>
-      <c r="G30" s="72"/>
-      <c r="H30" s="72"/>
-      <c r="I30" s="72"/>
-      <c r="J30" s="72"/>
-      <c r="K30" s="73"/>
+      <c r="F30" s="75"/>
+      <c r="G30" s="76"/>
+      <c r="H30" s="76"/>
+      <c r="I30" s="76"/>
+      <c r="J30" s="76"/>
+      <c r="K30" s="77"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="33" t="s">
@@ -4053,12 +4002,12 @@
         <v>39</v>
       </c>
       <c r="E31" s="32"/>
-      <c r="F31" s="71"/>
-      <c r="G31" s="72"/>
-      <c r="H31" s="72"/>
-      <c r="I31" s="72"/>
-      <c r="J31" s="72"/>
-      <c r="K31" s="73"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="76"/>
+      <c r="H31" s="76"/>
+      <c r="I31" s="76"/>
+      <c r="J31" s="76"/>
+      <c r="K31" s="77"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="33" t="s">
@@ -4074,12 +4023,12 @@
         <v>2</v>
       </c>
       <c r="E32" s="32"/>
-      <c r="F32" s="71"/>
-      <c r="G32" s="72"/>
-      <c r="H32" s="72"/>
-      <c r="I32" s="72"/>
-      <c r="J32" s="72"/>
-      <c r="K32" s="73"/>
+      <c r="F32" s="75"/>
+      <c r="G32" s="76"/>
+      <c r="H32" s="76"/>
+      <c r="I32" s="76"/>
+      <c r="J32" s="76"/>
+      <c r="K32" s="77"/>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="33" t="s">
@@ -4095,12 +4044,12 @@
         <v>2</v>
       </c>
       <c r="E33" s="32"/>
-      <c r="F33" s="71"/>
-      <c r="G33" s="72"/>
-      <c r="H33" s="72"/>
-      <c r="I33" s="72"/>
-      <c r="J33" s="72"/>
-      <c r="K33" s="73"/>
+      <c r="F33" s="75"/>
+      <c r="G33" s="76"/>
+      <c r="H33" s="76"/>
+      <c r="I33" s="76"/>
+      <c r="J33" s="76"/>
+      <c r="K33" s="77"/>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="33" t="s">
@@ -4116,12 +4065,12 @@
         <v>1</v>
       </c>
       <c r="E34" s="32"/>
-      <c r="F34" s="71"/>
-      <c r="G34" s="72"/>
-      <c r="H34" s="72"/>
-      <c r="I34" s="72"/>
-      <c r="J34" s="72"/>
-      <c r="K34" s="73"/>
+      <c r="F34" s="75"/>
+      <c r="G34" s="76"/>
+      <c r="H34" s="76"/>
+      <c r="I34" s="76"/>
+      <c r="J34" s="76"/>
+      <c r="K34" s="77"/>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="33" t="s">
@@ -4137,12 +4086,12 @@
         <v>1</v>
       </c>
       <c r="E35" s="32"/>
-      <c r="F35" s="71"/>
-      <c r="G35" s="72"/>
-      <c r="H35" s="72"/>
-      <c r="I35" s="72"/>
-      <c r="J35" s="72"/>
-      <c r="K35" s="73"/>
+      <c r="F35" s="75"/>
+      <c r="G35" s="76"/>
+      <c r="H35" s="76"/>
+      <c r="I35" s="76"/>
+      <c r="J35" s="76"/>
+      <c r="K35" s="77"/>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="33" t="s">
@@ -4158,12 +4107,12 @@
         <v>1</v>
       </c>
       <c r="E36" s="32"/>
-      <c r="F36" s="71"/>
-      <c r="G36" s="72"/>
-      <c r="H36" s="72"/>
-      <c r="I36" s="72"/>
-      <c r="J36" s="72"/>
-      <c r="K36" s="73"/>
+      <c r="F36" s="75"/>
+      <c r="G36" s="76"/>
+      <c r="H36" s="76"/>
+      <c r="I36" s="76"/>
+      <c r="J36" s="76"/>
+      <c r="K36" s="77"/>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="33" t="s">
@@ -4179,12 +4128,12 @@
         <v>1</v>
       </c>
       <c r="E37" s="32"/>
-      <c r="F37" s="71"/>
-      <c r="G37" s="72"/>
-      <c r="H37" s="72"/>
-      <c r="I37" s="72"/>
-      <c r="J37" s="72"/>
-      <c r="K37" s="73"/>
+      <c r="F37" s="75"/>
+      <c r="G37" s="76"/>
+      <c r="H37" s="76"/>
+      <c r="I37" s="76"/>
+      <c r="J37" s="76"/>
+      <c r="K37" s="77"/>
       <c r="Q37" s="48"/>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
@@ -4201,12 +4150,12 @@
         <v>1</v>
       </c>
       <c r="E38" s="32"/>
-      <c r="F38" s="71"/>
-      <c r="G38" s="72"/>
-      <c r="H38" s="72"/>
-      <c r="I38" s="72"/>
-      <c r="J38" s="72"/>
-      <c r="K38" s="73"/>
+      <c r="F38" s="75"/>
+      <c r="G38" s="76"/>
+      <c r="H38" s="76"/>
+      <c r="I38" s="76"/>
+      <c r="J38" s="76"/>
+      <c r="K38" s="77"/>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="33" t="s">
@@ -4222,12 +4171,12 @@
         <v>1</v>
       </c>
       <c r="E39" s="32"/>
-      <c r="F39" s="71"/>
-      <c r="G39" s="72"/>
-      <c r="H39" s="72"/>
-      <c r="I39" s="72"/>
-      <c r="J39" s="72"/>
-      <c r="K39" s="73"/>
+      <c r="F39" s="75"/>
+      <c r="G39" s="76"/>
+      <c r="H39" s="76"/>
+      <c r="I39" s="76"/>
+      <c r="J39" s="76"/>
+      <c r="K39" s="77"/>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="33" t="s">
@@ -4243,12 +4192,12 @@
         <v>1</v>
       </c>
       <c r="E40" s="32"/>
-      <c r="F40" s="74"/>
-      <c r="G40" s="75"/>
-      <c r="H40" s="75"/>
-      <c r="I40" s="75"/>
-      <c r="J40" s="75"/>
-      <c r="K40" s="76"/>
+      <c r="F40" s="78"/>
+      <c r="G40" s="79"/>
+      <c r="H40" s="79"/>
+      <c r="I40" s="79"/>
+      <c r="J40" s="79"/>
+      <c r="K40" s="80"/>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="36">
@@ -4304,7 +4253,7 @@
       <c r="I42" s="33">
         <v>1</v>
       </c>
-      <c r="J42" s="78">
+      <c r="J42" s="82">
         <v>5.87</v>
       </c>
       <c r="K42" s="32">
@@ -4322,7 +4271,7 @@
       <c r="G43" s="54"/>
       <c r="H43" s="58"/>
       <c r="I43" s="54"/>
-      <c r="J43" s="79"/>
+      <c r="J43" s="83"/>
       <c r="K43" s="56"/>
     </row>
     <row r="44" spans="1:17" ht="30" x14ac:dyDescent="0.25">
@@ -4353,7 +4302,7 @@
       <c r="I44" s="33">
         <v>3</v>
       </c>
-      <c r="J44" s="80"/>
+      <c r="J44" s="84"/>
       <c r="K44" s="32">
         <f>I44*E44</f>
         <v>38.97</v>
@@ -4387,7 +4336,7 @@
       <c r="I45" s="33">
         <v>1</v>
       </c>
-      <c r="J45" s="80"/>
+      <c r="J45" s="84"/>
       <c r="K45" s="32">
         <f t="shared" ref="K45:K46" si="1">I45*E45</f>
         <v>8.09</v>
@@ -4421,7 +4370,7 @@
       <c r="I46" s="33">
         <v>1</v>
       </c>
-      <c r="J46" s="80"/>
+      <c r="J46" s="84"/>
       <c r="K46" s="32">
         <f t="shared" si="1"/>
         <v>9.99</v>
@@ -4437,7 +4386,7 @@
       <c r="G47" s="54"/>
       <c r="H47" s="54"/>
       <c r="I47" s="54"/>
-      <c r="J47" s="79"/>
+      <c r="J47" s="83"/>
       <c r="K47" s="56"/>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.25">
@@ -4466,7 +4415,7 @@
         <v>259</v>
       </c>
       <c r="I48" s="33"/>
-      <c r="J48" s="80"/>
+      <c r="J48" s="84"/>
       <c r="K48" s="32">
         <f t="shared" ref="K48:K55" si="2">I48*E48</f>
         <v>0</v>
@@ -4498,7 +4447,7 @@
         <v>259</v>
       </c>
       <c r="I49" s="33"/>
-      <c r="J49" s="80"/>
+      <c r="J49" s="84"/>
       <c r="K49" s="32">
         <f>I49*E49</f>
         <v>0</v>
@@ -4514,7 +4463,7 @@
       <c r="G50" s="54"/>
       <c r="H50" s="54"/>
       <c r="I50" s="54"/>
-      <c r="J50" s="79"/>
+      <c r="J50" s="83"/>
       <c r="K50" s="56"/>
     </row>
     <row r="51" spans="1:17" ht="30" x14ac:dyDescent="0.25">
@@ -4545,7 +4494,7 @@
       <c r="I51" s="33">
         <v>3</v>
       </c>
-      <c r="J51" s="80"/>
+      <c r="J51" s="84"/>
       <c r="K51" s="32">
         <f t="shared" ref="K51:K52" si="3">I51*E51</f>
         <v>23.37</v>
@@ -4565,21 +4514,21 @@
       <c r="D52" s="33">
         <v>9</v>
       </c>
-      <c r="E52" s="66">
+      <c r="E52" s="70">
         <v>22.99</v>
       </c>
       <c r="F52" s="47" t="s">
         <v>260</v>
       </c>
-      <c r="G52" s="82" t="s">
+      <c r="G52" s="86" t="s">
         <v>176</v>
       </c>
-      <c r="H52" s="84" t="s">
+      <c r="H52" s="88" t="s">
         <v>259</v>
       </c>
-      <c r="I52" s="86"/>
-      <c r="J52" s="80"/>
-      <c r="K52" s="66">
+      <c r="I52" s="90"/>
+      <c r="J52" s="84"/>
+      <c r="K52" s="70">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -4597,15 +4546,15 @@
       <c r="D53" s="33">
         <v>7</v>
       </c>
-      <c r="E53" s="67"/>
+      <c r="E53" s="71"/>
       <c r="F53" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G53" s="83"/>
-      <c r="H53" s="85"/>
-      <c r="I53" s="87"/>
-      <c r="J53" s="80"/>
-      <c r="K53" s="67"/>
+      <c r="G53" s="87"/>
+      <c r="H53" s="89"/>
+      <c r="I53" s="91"/>
+      <c r="J53" s="84"/>
+      <c r="K53" s="71"/>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="47" t="s">
@@ -4635,7 +4584,7 @@
       <c r="I54" s="33">
         <v>1</v>
       </c>
-      <c r="J54" s="80"/>
+      <c r="J54" s="84"/>
       <c r="K54" s="32">
         <f>I54*E54</f>
         <v>9.99</v>
@@ -4667,7 +4616,7 @@
         <v>258</v>
       </c>
       <c r="I55" s="47"/>
-      <c r="J55" s="80"/>
+      <c r="J55" s="84"/>
       <c r="K55" s="32">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -4699,7 +4648,7 @@
         <v>248</v>
       </c>
       <c r="I56" s="33"/>
-      <c r="J56" s="81"/>
+      <c r="J56" s="85"/>
       <c r="K56" s="32"/>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.25">
@@ -4729,14 +4678,14 @@
         <v>1</v>
       </c>
       <c r="E58" s="32"/>
-      <c r="F58" s="77" t="s">
+      <c r="F58" s="81" t="s">
         <v>290</v>
       </c>
-      <c r="G58" s="69"/>
-      <c r="H58" s="69"/>
-      <c r="I58" s="69"/>
-      <c r="J58" s="69"/>
-      <c r="K58" s="70"/>
+      <c r="G58" s="73"/>
+      <c r="H58" s="73"/>
+      <c r="I58" s="73"/>
+      <c r="J58" s="73"/>
+      <c r="K58" s="74"/>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="47" t="s">
@@ -4752,12 +4701,12 @@
         <v>1</v>
       </c>
       <c r="E59" s="32"/>
-      <c r="F59" s="71"/>
-      <c r="G59" s="72"/>
-      <c r="H59" s="72"/>
-      <c r="I59" s="72"/>
-      <c r="J59" s="72"/>
-      <c r="K59" s="73"/>
+      <c r="F59" s="75"/>
+      <c r="G59" s="76"/>
+      <c r="H59" s="76"/>
+      <c r="I59" s="76"/>
+      <c r="J59" s="76"/>
+      <c r="K59" s="77"/>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="47" t="s">
@@ -4773,12 +4722,12 @@
         <v>44</v>
       </c>
       <c r="E60" s="32"/>
-      <c r="F60" s="71"/>
-      <c r="G60" s="72"/>
-      <c r="H60" s="72"/>
-      <c r="I60" s="72"/>
-      <c r="J60" s="72"/>
-      <c r="K60" s="73"/>
+      <c r="F60" s="75"/>
+      <c r="G60" s="76"/>
+      <c r="H60" s="76"/>
+      <c r="I60" s="76"/>
+      <c r="J60" s="76"/>
+      <c r="K60" s="77"/>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="47" t="s">
@@ -4794,12 +4743,12 @@
         <v>22</v>
       </c>
       <c r="E61" s="32"/>
-      <c r="F61" s="71"/>
-      <c r="G61" s="72"/>
-      <c r="H61" s="72"/>
-      <c r="I61" s="72"/>
-      <c r="J61" s="72"/>
-      <c r="K61" s="73"/>
+      <c r="F61" s="75"/>
+      <c r="G61" s="76"/>
+      <c r="H61" s="76"/>
+      <c r="I61" s="76"/>
+      <c r="J61" s="76"/>
+      <c r="K61" s="77"/>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="47" t="s">
@@ -4815,12 +4764,12 @@
         <v>2</v>
       </c>
       <c r="E62" s="32"/>
-      <c r="F62" s="71"/>
-      <c r="G62" s="72"/>
-      <c r="H62" s="72"/>
-      <c r="I62" s="72"/>
-      <c r="J62" s="72"/>
-      <c r="K62" s="73"/>
+      <c r="F62" s="75"/>
+      <c r="G62" s="76"/>
+      <c r="H62" s="76"/>
+      <c r="I62" s="76"/>
+      <c r="J62" s="76"/>
+      <c r="K62" s="77"/>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="47" t="s">
@@ -4836,12 +4785,12 @@
         <v>2</v>
       </c>
       <c r="E63" s="32"/>
-      <c r="F63" s="71"/>
-      <c r="G63" s="72"/>
-      <c r="H63" s="72"/>
-      <c r="I63" s="72"/>
-      <c r="J63" s="72"/>
-      <c r="K63" s="73"/>
+      <c r="F63" s="75"/>
+      <c r="G63" s="76"/>
+      <c r="H63" s="76"/>
+      <c r="I63" s="76"/>
+      <c r="J63" s="76"/>
+      <c r="K63" s="77"/>
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="47" t="s">
@@ -4857,12 +4806,12 @@
         <v>1</v>
       </c>
       <c r="E64" s="32"/>
-      <c r="F64" s="71"/>
-      <c r="G64" s="72"/>
-      <c r="H64" s="72"/>
-      <c r="I64" s="72"/>
-      <c r="J64" s="72"/>
-      <c r="K64" s="73"/>
+      <c r="F64" s="75"/>
+      <c r="G64" s="76"/>
+      <c r="H64" s="76"/>
+      <c r="I64" s="76"/>
+      <c r="J64" s="76"/>
+      <c r="K64" s="77"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="47" t="s">
@@ -4878,12 +4827,12 @@
         <v>1</v>
       </c>
       <c r="E65" s="32"/>
-      <c r="F65" s="71"/>
-      <c r="G65" s="72"/>
-      <c r="H65" s="72"/>
-      <c r="I65" s="72"/>
-      <c r="J65" s="72"/>
-      <c r="K65" s="73"/>
+      <c r="F65" s="75"/>
+      <c r="G65" s="76"/>
+      <c r="H65" s="76"/>
+      <c r="I65" s="76"/>
+      <c r="J65" s="76"/>
+      <c r="K65" s="77"/>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="47" t="s">
@@ -4899,12 +4848,12 @@
         <v>1</v>
       </c>
       <c r="E66" s="32"/>
-      <c r="F66" s="71"/>
-      <c r="G66" s="72"/>
-      <c r="H66" s="72"/>
-      <c r="I66" s="72"/>
-      <c r="J66" s="72"/>
-      <c r="K66" s="73"/>
+      <c r="F66" s="75"/>
+      <c r="G66" s="76"/>
+      <c r="H66" s="76"/>
+      <c r="I66" s="76"/>
+      <c r="J66" s="76"/>
+      <c r="K66" s="77"/>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="47" t="s">
@@ -4920,12 +4869,12 @@
         <v>1</v>
       </c>
       <c r="E67" s="32"/>
-      <c r="F67" s="71"/>
-      <c r="G67" s="72"/>
-      <c r="H67" s="72"/>
-      <c r="I67" s="72"/>
-      <c r="J67" s="72"/>
-      <c r="K67" s="73"/>
+      <c r="F67" s="75"/>
+      <c r="G67" s="76"/>
+      <c r="H67" s="76"/>
+      <c r="I67" s="76"/>
+      <c r="J67" s="76"/>
+      <c r="K67" s="77"/>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="47" t="s">
@@ -4941,12 +4890,12 @@
         <v>1</v>
       </c>
       <c r="E68" s="32"/>
-      <c r="F68" s="71"/>
-      <c r="G68" s="72"/>
-      <c r="H68" s="72"/>
-      <c r="I68" s="72"/>
-      <c r="J68" s="72"/>
-      <c r="K68" s="73"/>
+      <c r="F68" s="75"/>
+      <c r="G68" s="76"/>
+      <c r="H68" s="76"/>
+      <c r="I68" s="76"/>
+      <c r="J68" s="76"/>
+      <c r="K68" s="77"/>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="47" t="s">
@@ -4962,12 +4911,12 @@
         <v>1</v>
       </c>
       <c r="E69" s="32"/>
-      <c r="F69" s="71"/>
-      <c r="G69" s="72"/>
-      <c r="H69" s="72"/>
-      <c r="I69" s="72"/>
-      <c r="J69" s="72"/>
-      <c r="K69" s="73"/>
+      <c r="F69" s="75"/>
+      <c r="G69" s="76"/>
+      <c r="H69" s="76"/>
+      <c r="I69" s="76"/>
+      <c r="J69" s="76"/>
+      <c r="K69" s="77"/>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="47" t="s">
@@ -4983,12 +4932,27 @@
         <v>1</v>
       </c>
       <c r="E70" s="32"/>
-      <c r="F70" s="71"/>
-      <c r="G70" s="72"/>
-      <c r="H70" s="72"/>
-      <c r="I70" s="72"/>
-      <c r="J70" s="72"/>
-      <c r="K70" s="73"/>
+      <c r="F70" s="75"/>
+      <c r="G70" s="76"/>
+      <c r="H70" s="76"/>
+      <c r="I70" s="76"/>
+      <c r="J70" s="76"/>
+      <c r="K70" s="77"/>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A71" s="47" t="s">
+        <v>312</v>
+      </c>
+      <c r="B71" s="33">
+        <v>3</v>
+      </c>
+      <c r="C71" s="50" t="s">
+        <v>324</v>
+      </c>
+      <c r="D71" s="33">
+        <v>3</v>
+      </c>
+      <c r="E71" s="32"/>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="36">
@@ -4998,7 +4962,7 @@
         <v>3</v>
       </c>
       <c r="C73" s="37" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D73" s="36"/>
       <c r="E73" s="35" t="s">
@@ -5032,7 +4996,7 @@
         <v>240</v>
       </c>
       <c r="G74" s="45" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H74" s="63">
         <v>46237</v>
@@ -5040,7 +5004,7 @@
       <c r="I74" s="33">
         <v>1</v>
       </c>
-      <c r="J74" s="91">
+      <c r="J74" s="66">
         <v>5.87</v>
       </c>
       <c r="K74" s="32">
@@ -5058,7 +5022,7 @@
       <c r="G75" s="54"/>
       <c r="H75" s="58"/>
       <c r="I75" s="54"/>
-      <c r="J75" s="92"/>
+      <c r="J75" s="67"/>
       <c r="K75" s="56"/>
     </row>
     <row r="76" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -5079,7 +5043,7 @@
         <v>289</v>
       </c>
       <c r="G76" s="46" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H76" s="63">
         <v>46237</v>
@@ -5087,7 +5051,7 @@
       <c r="I76" s="33">
         <v>3</v>
       </c>
-      <c r="J76" s="93"/>
+      <c r="J76" s="68"/>
       <c r="K76" s="32">
         <f>I76*E76</f>
         <v>38.97</v>
@@ -5111,7 +5075,7 @@
         <v>318</v>
       </c>
       <c r="G77" s="46" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H77" s="63">
         <v>46237</v>
@@ -5119,7 +5083,7 @@
       <c r="I77" s="33">
         <v>1</v>
       </c>
-      <c r="J77" s="93"/>
+      <c r="J77" s="68"/>
       <c r="K77" s="32">
         <f t="shared" ref="K77:K78" si="4">I77*E77</f>
         <v>8.09</v>
@@ -5135,7 +5099,7 @@
       <c r="G78" s="46"/>
       <c r="H78" s="63"/>
       <c r="I78" s="33"/>
-      <c r="J78" s="93"/>
+      <c r="J78" s="68"/>
       <c r="K78" s="32">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -5190,6 +5154,5 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId27"/>
-  <drawing r:id="rId28"/>
 </worksheet>
 </file>
</xml_diff>